<commit_message>
Adopt Brick Atom gap escalation workflow
</commit_message>
<xml_diff>
--- a/playground/component-coverage.xlsx
+++ b/playground/component-coverage.xlsx
@@ -18,15 +18,15 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Index'!$A$1:$N$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Instructions'!$A$4:$B$18</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Instructions'!$A$1:$B$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Button'!$A$8:$M$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Button'!$A$8:$M$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Button'!$1:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Button'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Card'!$A$8:$M$33</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Button'!$A$1:$M$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Card'!$A$8:$M$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Card'!$1:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Card'!$A$1:$M$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Dialog'!$A$8:$M$33</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Card'!$A$1:$M$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Dialog'!$A$8:$M$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Dialog'!$1:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'Dialog'!$A$1:$M$33</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Dialog'!$A$1:$M$34</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -367,8 +367,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ButtonEvidence" displayName="ButtonEvidence" ref="A8:M33" headerRowCount="1">
-  <autoFilter ref="A8:M33"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ButtonEvidence" displayName="ButtonEvidence" ref="A8:M34" headerRowCount="1">
+  <autoFilter ref="A8:M34"/>
   <tableColumns count="13">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Area"/>
@@ -389,8 +389,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CardEvidence" displayName="CardEvidence" ref="A8:M33" headerRowCount="1">
-  <autoFilter ref="A8:M33"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CardEvidence" displayName="CardEvidence" ref="A8:M34" headerRowCount="1">
+  <autoFilter ref="A8:M34"/>
   <tableColumns count="13">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Area"/>
@@ -411,8 +411,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="DialogEvidence" displayName="DialogEvidence" ref="A8:M33" headerRowCount="1">
-  <autoFilter ref="A8:M33"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="DialogEvidence" displayName="DialogEvidence" ref="A8:M34" headerRowCount="1">
+  <autoFilter ref="A8:M34"/>
   <tableColumns count="13">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Area"/>
@@ -871,51 +871,51 @@
         </is>
       </c>
       <c r="B8" s="8">
-        <f>COUNTA('Button'!A9:A33)</f>
+        <f>COUNTA('Button'!A9:A34)</f>
         <v/>
       </c>
       <c r="C8" s="8">
-        <f>COUNTIF('Button'!H9:H33,"not started")</f>
+        <f>COUNTIF('Button'!H9:H34,"not started")</f>
         <v/>
       </c>
       <c r="D8" s="8">
-        <f>COUNTIF('Button'!H9:H33,"partial")</f>
+        <f>COUNTIF('Button'!H9:H34,"partial")</f>
         <v/>
       </c>
       <c r="E8" s="8">
-        <f>COUNTIF('Button'!H9:H33,"implemented")</f>
+        <f>COUNTIF('Button'!H9:H34,"implemented")</f>
         <v/>
       </c>
       <c r="F8" s="8">
-        <f>COUNTIF('Button'!H9:H33,"tested")</f>
+        <f>COUNTIF('Button'!H9:H34,"tested")</f>
         <v/>
       </c>
       <c r="G8" s="8">
-        <f>COUNTIF('Button'!H9:H33,"verified")</f>
+        <f>COUNTIF('Button'!H9:H34,"verified")</f>
         <v/>
       </c>
       <c r="H8" s="8">
-        <f>COUNTIF('Button'!H9:H33,"blocked")</f>
+        <f>COUNTIF('Button'!H9:H34,"blocked")</f>
         <v/>
       </c>
       <c r="I8" s="8">
-        <f>COUNTIF('Button'!H9:H33,"not applicable")</f>
+        <f>COUNTIF('Button'!H9:H34,"not applicable")</f>
         <v/>
       </c>
       <c r="J8" s="9">
-        <f>IFERROR(SUM('Button'!M9:M33)/SUM('Button'!L9:L33),0)</f>
+        <f>IFERROR(SUM('Button'!M9:M34)/SUM('Button'!L9:L34),0)</f>
         <v/>
       </c>
       <c r="K8" s="8">
-        <f>IF(COUNTIFS('Button'!E9:E33,"package",'Button'!M9:M33,"&lt;1")=0,"complete","open")</f>
+        <f>IF(COUNTIFS('Button'!E9:E34,"package",'Button'!M9:M34,"&lt;1")=0,"complete","open")</f>
         <v/>
       </c>
       <c r="L8" s="8">
-        <f>IF(COUNTIFS('Button'!E9:E33,"consumer",'Button'!M9:M33,"&lt;1")=0,"complete","open")</f>
+        <f>IF(COUNTIFS('Button'!E9:E34,"consumer",'Button'!M9:M34,"&lt;1")=0,"complete","open")</f>
         <v/>
       </c>
       <c r="M8" s="8">
-        <f>IF(COUNTIFS('Button'!E9:E33,"retirement",'Button'!M9:M33,"&lt;1")=0,"complete","open")</f>
+        <f>IF(COUNTIFS('Button'!E9:E34,"retirement",'Button'!M9:M34,"&lt;1")=0,"complete","open")</f>
         <v/>
       </c>
       <c r="N8" s="8">
@@ -930,51 +930,51 @@
         </is>
       </c>
       <c r="B9" s="8">
-        <f>COUNTA('Card'!A9:A33)</f>
+        <f>COUNTA('Card'!A9:A34)</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>COUNTIF('Card'!H9:H33,"not started")</f>
+        <f>COUNTIF('Card'!H9:H34,"not started")</f>
         <v/>
       </c>
       <c r="D9" s="8">
-        <f>COUNTIF('Card'!H9:H33,"partial")</f>
+        <f>COUNTIF('Card'!H9:H34,"partial")</f>
         <v/>
       </c>
       <c r="E9" s="8">
-        <f>COUNTIF('Card'!H9:H33,"implemented")</f>
+        <f>COUNTIF('Card'!H9:H34,"implemented")</f>
         <v/>
       </c>
       <c r="F9" s="8">
-        <f>COUNTIF('Card'!H9:H33,"tested")</f>
+        <f>COUNTIF('Card'!H9:H34,"tested")</f>
         <v/>
       </c>
       <c r="G9" s="8">
-        <f>COUNTIF('Card'!H9:H33,"verified")</f>
+        <f>COUNTIF('Card'!H9:H34,"verified")</f>
         <v/>
       </c>
       <c r="H9" s="8">
-        <f>COUNTIF('Card'!H9:H33,"blocked")</f>
+        <f>COUNTIF('Card'!H9:H34,"blocked")</f>
         <v/>
       </c>
       <c r="I9" s="8">
-        <f>COUNTIF('Card'!H9:H33,"not applicable")</f>
+        <f>COUNTIF('Card'!H9:H34,"not applicable")</f>
         <v/>
       </c>
       <c r="J9" s="9">
-        <f>IFERROR(SUM('Card'!M9:M33)/SUM('Card'!L9:L33),0)</f>
+        <f>IFERROR(SUM('Card'!M9:M34)/SUM('Card'!L9:L34),0)</f>
         <v/>
       </c>
       <c r="K9" s="8">
-        <f>IF(COUNTIFS('Card'!E9:E33,"package",'Card'!M9:M33,"&lt;1")=0,"complete","open")</f>
+        <f>IF(COUNTIFS('Card'!E9:E34,"package",'Card'!M9:M34,"&lt;1")=0,"complete","open")</f>
         <v/>
       </c>
       <c r="L9" s="8">
-        <f>IF(COUNTIFS('Card'!E9:E33,"consumer",'Card'!M9:M33,"&lt;1")=0,"complete","open")</f>
+        <f>IF(COUNTIFS('Card'!E9:E34,"consumer",'Card'!M9:M34,"&lt;1")=0,"complete","open")</f>
         <v/>
       </c>
       <c r="M9" s="8">
-        <f>IF(COUNTIFS('Card'!E9:E33,"retirement",'Card'!M9:M33,"&lt;1")=0,"complete","open")</f>
+        <f>IF(COUNTIFS('Card'!E9:E34,"retirement",'Card'!M9:M34,"&lt;1")=0,"complete","open")</f>
         <v/>
       </c>
       <c r="N9" s="8">
@@ -989,51 +989,51 @@
         </is>
       </c>
       <c r="B10" s="8">
-        <f>COUNTA('Dialog'!A9:A33)</f>
+        <f>COUNTA('Dialog'!A9:A34)</f>
         <v/>
       </c>
       <c r="C10" s="8">
-        <f>COUNTIF('Dialog'!H9:H33,"not started")</f>
+        <f>COUNTIF('Dialog'!H9:H34,"not started")</f>
         <v/>
       </c>
       <c r="D10" s="8">
-        <f>COUNTIF('Dialog'!H9:H33,"partial")</f>
+        <f>COUNTIF('Dialog'!H9:H34,"partial")</f>
         <v/>
       </c>
       <c r="E10" s="8">
-        <f>COUNTIF('Dialog'!H9:H33,"implemented")</f>
+        <f>COUNTIF('Dialog'!H9:H34,"implemented")</f>
         <v/>
       </c>
       <c r="F10" s="8">
-        <f>COUNTIF('Dialog'!H9:H33,"tested")</f>
+        <f>COUNTIF('Dialog'!H9:H34,"tested")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>COUNTIF('Dialog'!H9:H33,"verified")</f>
+        <f>COUNTIF('Dialog'!H9:H34,"verified")</f>
         <v/>
       </c>
       <c r="H10" s="8">
-        <f>COUNTIF('Dialog'!H9:H33,"blocked")</f>
+        <f>COUNTIF('Dialog'!H9:H34,"blocked")</f>
         <v/>
       </c>
       <c r="I10" s="8">
-        <f>COUNTIF('Dialog'!H9:H33,"not applicable")</f>
+        <f>COUNTIF('Dialog'!H9:H34,"not applicable")</f>
         <v/>
       </c>
       <c r="J10" s="9">
-        <f>IFERROR(SUM('Dialog'!M9:M33)/SUM('Dialog'!L9:L33),0)</f>
+        <f>IFERROR(SUM('Dialog'!M9:M34)/SUM('Dialog'!L9:L34),0)</f>
         <v/>
       </c>
       <c r="K10" s="8">
-        <f>IF(COUNTIFS('Dialog'!E9:E33,"package",'Dialog'!M9:M33,"&lt;1")=0,"complete","open")</f>
+        <f>IF(COUNTIFS('Dialog'!E9:E34,"package",'Dialog'!M9:M34,"&lt;1")=0,"complete","open")</f>
         <v/>
       </c>
       <c r="L10" s="8">
-        <f>IF(COUNTIFS('Dialog'!E9:E33,"consumer",'Dialog'!M9:M33,"&lt;1")=0,"complete","open")</f>
+        <f>IF(COUNTIFS('Dialog'!E9:E34,"consumer",'Dialog'!M9:M34,"&lt;1")=0,"complete","open")</f>
         <v/>
       </c>
       <c r="M10" s="8">
-        <f>IF(COUNTIFS('Dialog'!E9:E33,"retirement",'Dialog'!M9:M33,"&lt;1")=0,"complete","open")</f>
+        <f>IF(COUNTIFS('Dialog'!E9:E34,"retirement",'Dialog'!M9:M34,"&lt;1")=0,"complete","open")</f>
         <v/>
       </c>
       <c r="N10" s="8">
@@ -1309,7 +1309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M33"/>
+  <dimension ref="A1:M34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1348,7 +1348,7 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>COUNTA(A9:A33)</f>
+        <f>COUNTA(A9:A34)</f>
         <v/>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -1357,7 +1357,7 @@
         </is>
       </c>
       <c r="D4" s="4">
-        <f>SUM(M9:M33)</f>
+        <f>SUM(M9:M34)</f>
         <v/>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -1366,7 +1366,7 @@
         </is>
       </c>
       <c r="F4" s="5">
-        <f>IFERROR(D4/SUM(L9:L33),0)</f>
+        <f>IFERROR(D4/SUM(L9:L34),0)</f>
         <v/>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -1375,7 +1375,7 @@
         </is>
       </c>
       <c r="H4" s="4">
-        <f>COUNTIF(H9:H33,"blocked")</f>
+        <f>COUNTIF(H9:H34,"blocked")</f>
         <v/>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="J4" s="4">
-        <f>IF(COUNTIFS(E9:E33,"package",M9:M33,"&lt;1")=0,"complete","open")</f>
+        <f>IF(COUNTIFS(E9:E34,"package",M9:M34,"&lt;1")=0,"complete","open")</f>
         <v/>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -1393,7 +1393,7 @@
         </is>
       </c>
       <c r="L4" s="4">
-        <f>IF(COUNTIFS(E9:E33,"retirement",M9:M33,"&lt;1")=0,"complete","open")</f>
+        <f>IF(COUNTIFS(E9:E34,"retirement",M9:M34,"&lt;1")=0,"complete","open")</f>
         <v/>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>Public API</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>Public export and declaration surface match the approved brief</t>
+          <t>Atom capability audit covers mobile behavior and every Atom-owned gap is resolved through a released dependency</t>
         </is>
       </c>
       <c r="E10" s="15" t="inlineStr">
@@ -1551,7 +1551,7 @@
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>types</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="G10" s="15" t="inlineStr"/>
@@ -1562,7 +1562,7 @@
       </c>
       <c r="I10" s="15" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="J10" s="15" t="inlineStr"/>
@@ -1593,7 +1593,7 @@
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>Native props, refs, composition, and public slots follow the adopted API contract</t>
+          <t>Public export and declaration surface match the approved brief</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Visual system</t>
+          <t>Public API</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>Compiled CSS uses public brick classes, variables, layers, and semantic tokens</t>
+          <t>Native props, refs, composition, and public slots follow the adopted API contract</t>
         </is>
       </c>
       <c r="E12" s="15" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="F12" s="15" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>types</t>
         </is>
       </c>
       <c r="G12" s="15" t="inlineStr"/>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
-          <t>Default recipe and every approved visual option are implemented</t>
+          <t>Compiled CSS uses public brick classes, variables, layers, and semantic tokens</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J13" s="15" t="inlineStr"/>
@@ -1739,7 +1739,7 @@
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>Playground</t>
+          <t>Visual system</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="D14" s="15" t="inlineStr">
         <is>
-          <t>Canonical overview and shortest finished state</t>
+          <t>Default recipe and every approved visual option are implemented</t>
         </is>
       </c>
       <c r="E14" s="15" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="F14" s="15" t="inlineStr">
         <is>
-          <t>playground</t>
+          <t>source</t>
         </is>
       </c>
       <c r="G14" s="15" t="inlineStr"/>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="D15" s="15" t="inlineStr">
         <is>
-          <t>Every public recipe, size, and important state</t>
+          <t>Canonical overview and shortest finished state</t>
         </is>
       </c>
       <c r="E15" s="15" t="inlineStr">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="D16" s="15" t="inlineStr">
         <is>
-          <t>Mobile-first constrained viewport and intentional wide layout</t>
+          <t>Every public recipe, size, and important state</t>
         </is>
       </c>
       <c r="E16" s="15" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="D17" s="15" t="inlineStr">
         <is>
-          <t>Light, dark, and relevant preference modes</t>
+          <t>Mobile-first constrained viewport and intentional wide layout</t>
         </is>
       </c>
       <c r="E17" s="15" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="D18" s="15" t="inlineStr">
         <is>
-          <t>Long content, localization, zoom, and RTL stress</t>
+          <t>Light, dark, and relevant preference modes</t>
         </is>
       </c>
       <c r="E18" s="15" t="inlineStr">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="D19" s="15" t="inlineStr">
         <is>
-          <t>Token, className, style, slot, and documented part customization</t>
+          <t>Long content, localization, zoom, and RTL stress</t>
         </is>
       </c>
       <c r="E19" s="15" t="inlineStr">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>Stable route and deterministic state inputs for browser tests</t>
+          <t>Token, className, style, slot, and documented part customization</t>
         </is>
       </c>
       <c r="E20" s="15" t="inlineStr">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="I20" s="15" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="J20" s="15" t="inlineStr"/>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>Automated tests</t>
+          <t>Playground</t>
         </is>
       </c>
       <c r="C21" s="15" t="inlineStr">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>Vitest and Testing Library component contract tests</t>
+          <t>Stable route and deterministic state inputs for browser tests</t>
         </is>
       </c>
       <c r="E21" s="15" t="inlineStr">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="F21" s="15" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>playground</t>
         </is>
       </c>
       <c r="G21" s="15" t="inlineStr"/>
@@ -2165,7 +2165,7 @@
       </c>
       <c r="D22" s="15" t="inlineStr">
         <is>
-          <t>Public type and declaration fixtures</t>
+          <t>Vitest and Testing Library component contract tests</t>
         </is>
       </c>
       <c r="E22" s="15" t="inlineStr">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="D23" s="15" t="inlineStr">
         <is>
-          <t>Playwright keyboard, pointer, focus, and state interactions</t>
+          <t>Public type and declaration fixtures</t>
         </is>
       </c>
       <c r="E23" s="15" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="D24" s="15" t="inlineStr">
         <is>
-          <t>Axe checks for canonical browser states</t>
+          <t>Playwright keyboard, pointer, focus, and state interactions</t>
         </is>
       </c>
       <c r="E24" s="15" t="inlineStr">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="D25" s="15" t="inlineStr">
         <is>
-          <t>Risk-based Chromium visual baselines reviewed</t>
+          <t>Axe checks for canonical browser states</t>
         </is>
       </c>
       <c r="E25" s="15" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="I25" s="15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J25" s="15" t="inlineStr"/>
@@ -2373,7 +2373,7 @@
       </c>
       <c r="D26" s="15" t="inlineStr">
         <is>
-          <t>Relevant Chromium, Firefox, WebKit, and mobile-profile checks</t>
+          <t>Risk-based Chromium visual baselines reviewed</t>
         </is>
       </c>
       <c r="E26" s="15" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="I26" s="15" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="J26" s="15" t="inlineStr"/>
@@ -2425,7 +2425,7 @@
       </c>
       <c r="D27" s="15" t="inlineStr">
         <is>
-          <t>SSR or server-safe consumer behavior where applicable</t>
+          <t>Relevant Chromium, Firefox, WebKit, and mobile-profile checks</t>
         </is>
       </c>
       <c r="E27" s="15" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>Manual evidence</t>
+          <t>Automated tests</t>
         </is>
       </c>
       <c r="C28" s="15" t="inlineStr">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="D28" s="15" t="inlineStr">
         <is>
-          <t>Numbered component manual-test protocol is complete</t>
+          <t>SSR or server-safe consumer behavior where applicable</t>
         </is>
       </c>
       <c r="E28" s="15" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="F28" s="15" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>test</t>
         </is>
       </c>
       <c r="G28" s="15" t="inlineStr"/>
@@ -2529,7 +2529,7 @@
       </c>
       <c r="D29" s="15" t="inlineStr">
         <is>
-          <t>Latest required manual run is recorded and passes</t>
+          <t>Numbered component manual-test protocol is complete</t>
         </is>
       </c>
       <c r="E29" s="15" t="inlineStr">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="I29" s="15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J29" s="15" t="inlineStr"/>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="B30" s="15" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Manual evidence</t>
         </is>
       </c>
       <c r="C30" s="15" t="inlineStr">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="D30" s="15" t="inlineStr">
         <is>
-          <t>Public component documentation follows the standard template</t>
+          <t>Latest required manual run is recorded and passes</t>
         </is>
       </c>
       <c r="E30" s="15" t="inlineStr">
@@ -2591,7 +2591,7 @@
       </c>
       <c r="F30" s="15" t="inlineStr">
         <is>
-          <t>docs</t>
+          <t>manual</t>
         </is>
       </c>
       <c r="G30" s="15" t="inlineStr"/>
@@ -2633,7 +2633,7 @@
       </c>
       <c r="D31" s="15" t="inlineStr">
         <is>
-          <t>Component changelog and applicable package release notes are updated</t>
+          <t>Public component documentation follows the standard template</t>
         </is>
       </c>
       <c r="E31" s="15" t="inlineStr">
@@ -2654,7 +2654,7 @@
       </c>
       <c r="I31" s="15" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="J31" s="15" t="inlineStr"/>
@@ -2675,7 +2675,7 @@
       </c>
       <c r="B32" s="15" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C32" s="15" t="inlineStr">
@@ -2685,17 +2685,17 @@
       </c>
       <c r="D32" s="15" t="inlineStr">
         <is>
-          <t>Live consumer cutover is verified without adding new legacy Core coupling</t>
+          <t>Component changelog and applicable package release notes are updated</t>
         </is>
       </c>
       <c r="E32" s="15" t="inlineStr">
         <is>
-          <t>consumer</t>
+          <t>package</t>
         </is>
       </c>
       <c r="F32" s="15" t="inlineStr">
         <is>
-          <t>consumer</t>
+          <t>docs</t>
         </is>
       </c>
       <c r="G32" s="15" t="inlineStr"/>
@@ -2706,7 +2706,7 @@
       </c>
       <c r="I32" s="15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J32" s="15" t="inlineStr"/>
@@ -2727,7 +2727,7 @@
       </c>
       <c r="B33" s="15" t="inlineStr">
         <is>
-          <t>Retirement</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="C33" s="15" t="inlineStr">
@@ -2737,17 +2737,17 @@
       </c>
       <c r="D33" s="15" t="inlineStr">
         <is>
-          <t>Legacy Core slice and authorized stale consumer evidence are removed</t>
+          <t>Live consumer cutover is verified without adding new legacy Core coupling</t>
         </is>
       </c>
       <c r="E33" s="15" t="inlineStr">
         <is>
-          <t>retirement</t>
+          <t>consumer</t>
         </is>
       </c>
       <c r="F33" s="15" t="inlineStr">
         <is>
-          <t>removal</t>
+          <t>consumer</t>
         </is>
       </c>
       <c r="G33" s="15" t="inlineStr"/>
@@ -2771,14 +2771,66 @@
         <v/>
       </c>
     </row>
+    <row r="34" ht="43" customHeight="1">
+      <c r="A34" s="15" t="inlineStr">
+        <is>
+          <t>BUT-26</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="inlineStr">
+        <is>
+          <t>Retirement</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
+          <t>Legacy Core slice and authorized stale consumer evidence are removed</t>
+        </is>
+      </c>
+      <c r="E34" s="15" t="inlineStr">
+        <is>
+          <t>retirement</t>
+        </is>
+      </c>
+      <c r="F34" s="15" t="inlineStr">
+        <is>
+          <t>removal</t>
+        </is>
+      </c>
+      <c r="G34" s="15" t="inlineStr"/>
+      <c r="H34" s="15" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
+      <c r="I34" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J34" s="15" t="inlineStr"/>
+      <c r="K34" s="15" t="inlineStr"/>
+      <c r="L34" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="M34" s="16">
+        <f>IF(H34="not applicable",IF(K34&lt;&gt;"",1,0),IF(I34="yes",IF(H34="verified",1,0),IF(OR(H34="tested",H34="verified"),1,0)))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:M33"/>
+  <autoFilter ref="A8:M34"/>
   <mergeCells count="3">
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A6:M6"/>
     <mergeCell ref="A1:M1"/>
   </mergeCells>
-  <conditionalFormatting sqref="H9:H33">
+  <conditionalFormatting sqref="H9:H34">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H9="not started"</formula>
     </cfRule>
@@ -2802,10 +2854,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="H9:H33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H9:H34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>=_Lists!$A$1:$A$7</formula1>
     </dataValidation>
-    <dataValidation sqref="I9:I33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="I9:I34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>=_Lists!$B$1:$B$2</formula1>
     </dataValidation>
   </dataValidations>
@@ -2823,7 +2875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M33"/>
+  <dimension ref="A1:M34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2862,7 +2914,7 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>COUNTA(A9:A33)</f>
+        <f>COUNTA(A9:A34)</f>
         <v/>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -2871,7 +2923,7 @@
         </is>
       </c>
       <c r="D4" s="4">
-        <f>SUM(M9:M33)</f>
+        <f>SUM(M9:M34)</f>
         <v/>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -2880,7 +2932,7 @@
         </is>
       </c>
       <c r="F4" s="5">
-        <f>IFERROR(D4/SUM(L9:L33),0)</f>
+        <f>IFERROR(D4/SUM(L9:L34),0)</f>
         <v/>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -2889,7 +2941,7 @@
         </is>
       </c>
       <c r="H4" s="4">
-        <f>COUNTIF(H9:H33,"blocked")</f>
+        <f>COUNTIF(H9:H34,"blocked")</f>
         <v/>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -2898,7 +2950,7 @@
         </is>
       </c>
       <c r="J4" s="4">
-        <f>IF(COUNTIFS(E9:E33,"package",M9:M33,"&lt;1")=0,"complete","open")</f>
+        <f>IF(COUNTIFS(E9:E34,"package",M9:M34,"&lt;1")=0,"complete","open")</f>
         <v/>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -2907,7 +2959,7 @@
         </is>
       </c>
       <c r="L4" s="4">
-        <f>IF(COUNTIFS(E9:E33,"retirement",M9:M33,"&lt;1")=0,"complete","open")</f>
+        <f>IF(COUNTIFS(E9:E34,"retirement",M9:M34,"&lt;1")=0,"complete","open")</f>
         <v/>
       </c>
     </row>
@@ -3045,7 +3097,7 @@
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>Public API</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
@@ -3055,7 +3107,7 @@
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>Public export and declaration surface match the approved brief</t>
+          <t>Atom capability audit covers mobile behavior and every Atom-owned gap is resolved through a released dependency</t>
         </is>
       </c>
       <c r="E10" s="15" t="inlineStr">
@@ -3065,7 +3117,7 @@
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>types</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="G10" s="15" t="inlineStr"/>
@@ -3076,7 +3128,7 @@
       </c>
       <c r="I10" s="15" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="J10" s="15" t="inlineStr"/>
@@ -3107,7 +3159,7 @@
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>Native props, refs, composition, and public slots follow the adopted API contract</t>
+          <t>Public export and declaration surface match the approved brief</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
@@ -3149,7 +3201,7 @@
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Visual system</t>
+          <t>Public API</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
@@ -3159,7 +3211,7 @@
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>Compiled CSS uses public brick classes, variables, layers, and semantic tokens</t>
+          <t>Native props, refs, composition, and public slots follow the adopted API contract</t>
         </is>
       </c>
       <c r="E12" s="15" t="inlineStr">
@@ -3169,7 +3221,7 @@
       </c>
       <c r="F12" s="15" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>types</t>
         </is>
       </c>
       <c r="G12" s="15" t="inlineStr"/>
@@ -3211,7 +3263,7 @@
       </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
-          <t>Default recipe and every approved visual option are implemented</t>
+          <t>Compiled CSS uses public brick classes, variables, layers, and semantic tokens</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
@@ -3232,7 +3284,7 @@
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J13" s="15" t="inlineStr"/>
@@ -3253,7 +3305,7 @@
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>Playground</t>
+          <t>Visual system</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
@@ -3263,7 +3315,7 @@
       </c>
       <c r="D14" s="15" t="inlineStr">
         <is>
-          <t>Canonical overview and shortest finished state</t>
+          <t>Default recipe and every approved visual option are implemented</t>
         </is>
       </c>
       <c r="E14" s="15" t="inlineStr">
@@ -3273,7 +3325,7 @@
       </c>
       <c r="F14" s="15" t="inlineStr">
         <is>
-          <t>playground</t>
+          <t>source</t>
         </is>
       </c>
       <c r="G14" s="15" t="inlineStr"/>
@@ -3315,7 +3367,7 @@
       </c>
       <c r="D15" s="15" t="inlineStr">
         <is>
-          <t>Every public recipe, size, and important state</t>
+          <t>Canonical overview and shortest finished state</t>
         </is>
       </c>
       <c r="E15" s="15" t="inlineStr">
@@ -3367,7 +3419,7 @@
       </c>
       <c r="D16" s="15" t="inlineStr">
         <is>
-          <t>Mobile-first constrained viewport and intentional wide layout</t>
+          <t>Every public recipe, size, and important state</t>
         </is>
       </c>
       <c r="E16" s="15" t="inlineStr">
@@ -3419,7 +3471,7 @@
       </c>
       <c r="D17" s="15" t="inlineStr">
         <is>
-          <t>Light, dark, and relevant preference modes</t>
+          <t>Mobile-first constrained viewport and intentional wide layout</t>
         </is>
       </c>
       <c r="E17" s="15" t="inlineStr">
@@ -3471,7 +3523,7 @@
       </c>
       <c r="D18" s="15" t="inlineStr">
         <is>
-          <t>Long content, localization, zoom, and RTL stress</t>
+          <t>Light, dark, and relevant preference modes</t>
         </is>
       </c>
       <c r="E18" s="15" t="inlineStr">
@@ -3523,7 +3575,7 @@
       </c>
       <c r="D19" s="15" t="inlineStr">
         <is>
-          <t>Token, className, style, slot, and documented part customization</t>
+          <t>Long content, localization, zoom, and RTL stress</t>
         </is>
       </c>
       <c r="E19" s="15" t="inlineStr">
@@ -3575,7 +3627,7 @@
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>Stable route and deterministic state inputs for browser tests</t>
+          <t>Token, className, style, slot, and documented part customization</t>
         </is>
       </c>
       <c r="E20" s="15" t="inlineStr">
@@ -3596,7 +3648,7 @@
       </c>
       <c r="I20" s="15" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="J20" s="15" t="inlineStr"/>
@@ -3617,7 +3669,7 @@
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>Automated tests</t>
+          <t>Playground</t>
         </is>
       </c>
       <c r="C21" s="15" t="inlineStr">
@@ -3627,7 +3679,7 @@
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>Vitest and Testing Library component contract tests</t>
+          <t>Stable route and deterministic state inputs for browser tests</t>
         </is>
       </c>
       <c r="E21" s="15" t="inlineStr">
@@ -3637,7 +3689,7 @@
       </c>
       <c r="F21" s="15" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>playground</t>
         </is>
       </c>
       <c r="G21" s="15" t="inlineStr"/>
@@ -3679,7 +3731,7 @@
       </c>
       <c r="D22" s="15" t="inlineStr">
         <is>
-          <t>Public type and declaration fixtures</t>
+          <t>Vitest and Testing Library component contract tests</t>
         </is>
       </c>
       <c r="E22" s="15" t="inlineStr">
@@ -3731,7 +3783,7 @@
       </c>
       <c r="D23" s="15" t="inlineStr">
         <is>
-          <t>Playwright keyboard, pointer, focus, and state interactions</t>
+          <t>Public type and declaration fixtures</t>
         </is>
       </c>
       <c r="E23" s="15" t="inlineStr">
@@ -3783,7 +3835,7 @@
       </c>
       <c r="D24" s="15" t="inlineStr">
         <is>
-          <t>Axe checks for canonical browser states</t>
+          <t>Playwright keyboard, pointer, focus, and state interactions</t>
         </is>
       </c>
       <c r="E24" s="15" t="inlineStr">
@@ -3835,7 +3887,7 @@
       </c>
       <c r="D25" s="15" t="inlineStr">
         <is>
-          <t>Risk-based Chromium visual baselines reviewed</t>
+          <t>Axe checks for canonical browser states</t>
         </is>
       </c>
       <c r="E25" s="15" t="inlineStr">
@@ -3856,7 +3908,7 @@
       </c>
       <c r="I25" s="15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J25" s="15" t="inlineStr"/>
@@ -3887,7 +3939,7 @@
       </c>
       <c r="D26" s="15" t="inlineStr">
         <is>
-          <t>Relevant Chromium, Firefox, WebKit, and mobile-profile checks</t>
+          <t>Risk-based Chromium visual baselines reviewed</t>
         </is>
       </c>
       <c r="E26" s="15" t="inlineStr">
@@ -3908,7 +3960,7 @@
       </c>
       <c r="I26" s="15" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="J26" s="15" t="inlineStr"/>
@@ -3939,7 +3991,7 @@
       </c>
       <c r="D27" s="15" t="inlineStr">
         <is>
-          <t>SSR or server-safe consumer behavior where applicable</t>
+          <t>Relevant Chromium, Firefox, WebKit, and mobile-profile checks</t>
         </is>
       </c>
       <c r="E27" s="15" t="inlineStr">
@@ -3981,7 +4033,7 @@
       </c>
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>Manual evidence</t>
+          <t>Automated tests</t>
         </is>
       </c>
       <c r="C28" s="15" t="inlineStr">
@@ -3991,7 +4043,7 @@
       </c>
       <c r="D28" s="15" t="inlineStr">
         <is>
-          <t>Numbered component manual-test protocol is complete</t>
+          <t>SSR or server-safe consumer behavior where applicable</t>
         </is>
       </c>
       <c r="E28" s="15" t="inlineStr">
@@ -4001,7 +4053,7 @@
       </c>
       <c r="F28" s="15" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>test</t>
         </is>
       </c>
       <c r="G28" s="15" t="inlineStr"/>
@@ -4043,7 +4095,7 @@
       </c>
       <c r="D29" s="15" t="inlineStr">
         <is>
-          <t>Latest required manual run is recorded and passes</t>
+          <t>Numbered component manual-test protocol is complete</t>
         </is>
       </c>
       <c r="E29" s="15" t="inlineStr">
@@ -4064,7 +4116,7 @@
       </c>
       <c r="I29" s="15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J29" s="15" t="inlineStr"/>
@@ -4085,7 +4137,7 @@
       </c>
       <c r="B30" s="15" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Manual evidence</t>
         </is>
       </c>
       <c r="C30" s="15" t="inlineStr">
@@ -4095,7 +4147,7 @@
       </c>
       <c r="D30" s="15" t="inlineStr">
         <is>
-          <t>Public component documentation follows the standard template</t>
+          <t>Latest required manual run is recorded and passes</t>
         </is>
       </c>
       <c r="E30" s="15" t="inlineStr">
@@ -4105,7 +4157,7 @@
       </c>
       <c r="F30" s="15" t="inlineStr">
         <is>
-          <t>docs</t>
+          <t>manual</t>
         </is>
       </c>
       <c r="G30" s="15" t="inlineStr"/>
@@ -4147,7 +4199,7 @@
       </c>
       <c r="D31" s="15" t="inlineStr">
         <is>
-          <t>Component changelog and applicable package release notes are updated</t>
+          <t>Public component documentation follows the standard template</t>
         </is>
       </c>
       <c r="E31" s="15" t="inlineStr">
@@ -4168,7 +4220,7 @@
       </c>
       <c r="I31" s="15" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="J31" s="15" t="inlineStr"/>
@@ -4189,7 +4241,7 @@
       </c>
       <c r="B32" s="15" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C32" s="15" t="inlineStr">
@@ -4199,17 +4251,17 @@
       </c>
       <c r="D32" s="15" t="inlineStr">
         <is>
-          <t>Live consumer cutover is verified without adding new legacy Core coupling</t>
+          <t>Component changelog and applicable package release notes are updated</t>
         </is>
       </c>
       <c r="E32" s="15" t="inlineStr">
         <is>
-          <t>consumer</t>
+          <t>package</t>
         </is>
       </c>
       <c r="F32" s="15" t="inlineStr">
         <is>
-          <t>consumer</t>
+          <t>docs</t>
         </is>
       </c>
       <c r="G32" s="15" t="inlineStr"/>
@@ -4220,7 +4272,7 @@
       </c>
       <c r="I32" s="15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J32" s="15" t="inlineStr"/>
@@ -4241,7 +4293,7 @@
       </c>
       <c r="B33" s="15" t="inlineStr">
         <is>
-          <t>Retirement</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="C33" s="15" t="inlineStr">
@@ -4251,17 +4303,17 @@
       </c>
       <c r="D33" s="15" t="inlineStr">
         <is>
-          <t>Legacy Core slice and authorized stale consumer evidence are removed</t>
+          <t>Live consumer cutover is verified without adding new legacy Core coupling</t>
         </is>
       </c>
       <c r="E33" s="15" t="inlineStr">
         <is>
-          <t>retirement</t>
+          <t>consumer</t>
         </is>
       </c>
       <c r="F33" s="15" t="inlineStr">
         <is>
-          <t>removal</t>
+          <t>consumer</t>
         </is>
       </c>
       <c r="G33" s="15" t="inlineStr"/>
@@ -4285,14 +4337,66 @@
         <v/>
       </c>
     </row>
+    <row r="34" ht="43" customHeight="1">
+      <c r="A34" s="15" t="inlineStr">
+        <is>
+          <t>CAR-26</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="inlineStr">
+        <is>
+          <t>Retirement</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
+          <t>Legacy Core slice and authorized stale consumer evidence are removed</t>
+        </is>
+      </c>
+      <c r="E34" s="15" t="inlineStr">
+        <is>
+          <t>retirement</t>
+        </is>
+      </c>
+      <c r="F34" s="15" t="inlineStr">
+        <is>
+          <t>removal</t>
+        </is>
+      </c>
+      <c r="G34" s="15" t="inlineStr"/>
+      <c r="H34" s="15" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
+      <c r="I34" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J34" s="15" t="inlineStr"/>
+      <c r="K34" s="15" t="inlineStr"/>
+      <c r="L34" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="M34" s="16">
+        <f>IF(H34="not applicable",IF(K34&lt;&gt;"",1,0),IF(I34="yes",IF(H34="verified",1,0),IF(OR(H34="tested",H34="verified"),1,0)))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:M33"/>
+  <autoFilter ref="A8:M34"/>
   <mergeCells count="3">
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A6:M6"/>
     <mergeCell ref="A1:M1"/>
   </mergeCells>
-  <conditionalFormatting sqref="H9:H33">
+  <conditionalFormatting sqref="H9:H34">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H9="not started"</formula>
     </cfRule>
@@ -4316,10 +4420,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="H9:H33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H9:H34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>=_Lists!$A$1:$A$7</formula1>
     </dataValidation>
-    <dataValidation sqref="I9:I33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="I9:I34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>=_Lists!$B$1:$B$2</formula1>
     </dataValidation>
   </dataValidations>
@@ -4337,7 +4441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M33"/>
+  <dimension ref="A1:M34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4376,7 +4480,7 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>COUNTA(A9:A33)</f>
+        <f>COUNTA(A9:A34)</f>
         <v/>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -4385,7 +4489,7 @@
         </is>
       </c>
       <c r="D4" s="4">
-        <f>SUM(M9:M33)</f>
+        <f>SUM(M9:M34)</f>
         <v/>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -4394,7 +4498,7 @@
         </is>
       </c>
       <c r="F4" s="5">
-        <f>IFERROR(D4/SUM(L9:L33),0)</f>
+        <f>IFERROR(D4/SUM(L9:L34),0)</f>
         <v/>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -4403,7 +4507,7 @@
         </is>
       </c>
       <c r="H4" s="4">
-        <f>COUNTIF(H9:H33,"blocked")</f>
+        <f>COUNTIF(H9:H34,"blocked")</f>
         <v/>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -4412,7 +4516,7 @@
         </is>
       </c>
       <c r="J4" s="4">
-        <f>IF(COUNTIFS(E9:E33,"package",M9:M33,"&lt;1")=0,"complete","open")</f>
+        <f>IF(COUNTIFS(E9:E34,"package",M9:M34,"&lt;1")=0,"complete","open")</f>
         <v/>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -4421,7 +4525,7 @@
         </is>
       </c>
       <c r="L4" s="4">
-        <f>IF(COUNTIFS(E9:E33,"retirement",M9:M33,"&lt;1")=0,"complete","open")</f>
+        <f>IF(COUNTIFS(E9:E34,"retirement",M9:M34,"&lt;1")=0,"complete","open")</f>
         <v/>
       </c>
     </row>
@@ -4559,7 +4663,7 @@
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>Public API</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
@@ -4569,7 +4673,7 @@
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>Public export and declaration surface match the approved brief</t>
+          <t>Atom capability audit covers mobile behavior and every Atom-owned gap is resolved through a released dependency</t>
         </is>
       </c>
       <c r="E10" s="15" t="inlineStr">
@@ -4579,7 +4683,7 @@
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>types</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="G10" s="15" t="inlineStr"/>
@@ -4590,7 +4694,7 @@
       </c>
       <c r="I10" s="15" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="J10" s="15" t="inlineStr"/>
@@ -4621,7 +4725,7 @@
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>Native props, refs, composition, and public slots follow the adopted API contract</t>
+          <t>Public export and declaration surface match the approved brief</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
@@ -4663,7 +4767,7 @@
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Visual system</t>
+          <t>Public API</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
@@ -4673,7 +4777,7 @@
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>Compiled CSS uses public brick classes, variables, layers, and semantic tokens</t>
+          <t>Native props, refs, composition, and public slots follow the adopted API contract</t>
         </is>
       </c>
       <c r="E12" s="15" t="inlineStr">
@@ -4683,7 +4787,7 @@
       </c>
       <c r="F12" s="15" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>types</t>
         </is>
       </c>
       <c r="G12" s="15" t="inlineStr"/>
@@ -4725,7 +4829,7 @@
       </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
-          <t>Default recipe and every approved visual option are implemented</t>
+          <t>Compiled CSS uses public brick classes, variables, layers, and semantic tokens</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
@@ -4746,7 +4850,7 @@
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J13" s="15" t="inlineStr"/>
@@ -4767,7 +4871,7 @@
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>Playground</t>
+          <t>Visual system</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
@@ -4777,7 +4881,7 @@
       </c>
       <c r="D14" s="15" t="inlineStr">
         <is>
-          <t>Canonical overview and shortest finished state</t>
+          <t>Default recipe and every approved visual option are implemented</t>
         </is>
       </c>
       <c r="E14" s="15" t="inlineStr">
@@ -4787,7 +4891,7 @@
       </c>
       <c r="F14" s="15" t="inlineStr">
         <is>
-          <t>playground</t>
+          <t>source</t>
         </is>
       </c>
       <c r="G14" s="15" t="inlineStr"/>
@@ -4829,7 +4933,7 @@
       </c>
       <c r="D15" s="15" t="inlineStr">
         <is>
-          <t>Every public recipe, size, and important state</t>
+          <t>Canonical overview and shortest finished state</t>
         </is>
       </c>
       <c r="E15" s="15" t="inlineStr">
@@ -4881,7 +4985,7 @@
       </c>
       <c r="D16" s="15" t="inlineStr">
         <is>
-          <t>Mobile-first constrained viewport and intentional wide layout</t>
+          <t>Every public recipe, size, and important state</t>
         </is>
       </c>
       <c r="E16" s="15" t="inlineStr">
@@ -4933,7 +5037,7 @@
       </c>
       <c r="D17" s="15" t="inlineStr">
         <is>
-          <t>Light, dark, and relevant preference modes</t>
+          <t>Mobile-first constrained viewport and intentional wide layout</t>
         </is>
       </c>
       <c r="E17" s="15" t="inlineStr">
@@ -4985,7 +5089,7 @@
       </c>
       <c r="D18" s="15" t="inlineStr">
         <is>
-          <t>Long content, localization, zoom, and RTL stress</t>
+          <t>Light, dark, and relevant preference modes</t>
         </is>
       </c>
       <c r="E18" s="15" t="inlineStr">
@@ -5037,7 +5141,7 @@
       </c>
       <c r="D19" s="15" t="inlineStr">
         <is>
-          <t>Token, className, style, slot, and documented part customization</t>
+          <t>Long content, localization, zoom, and RTL stress</t>
         </is>
       </c>
       <c r="E19" s="15" t="inlineStr">
@@ -5089,7 +5193,7 @@
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>Stable route and deterministic state inputs for browser tests</t>
+          <t>Token, className, style, slot, and documented part customization</t>
         </is>
       </c>
       <c r="E20" s="15" t="inlineStr">
@@ -5110,7 +5214,7 @@
       </c>
       <c r="I20" s="15" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="J20" s="15" t="inlineStr"/>
@@ -5131,7 +5235,7 @@
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>Automated tests</t>
+          <t>Playground</t>
         </is>
       </c>
       <c r="C21" s="15" t="inlineStr">
@@ -5141,7 +5245,7 @@
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>Vitest and Testing Library component contract tests</t>
+          <t>Stable route and deterministic state inputs for browser tests</t>
         </is>
       </c>
       <c r="E21" s="15" t="inlineStr">
@@ -5151,7 +5255,7 @@
       </c>
       <c r="F21" s="15" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>playground</t>
         </is>
       </c>
       <c r="G21" s="15" t="inlineStr"/>
@@ -5193,7 +5297,7 @@
       </c>
       <c r="D22" s="15" t="inlineStr">
         <is>
-          <t>Public type and declaration fixtures</t>
+          <t>Vitest and Testing Library component contract tests</t>
         </is>
       </c>
       <c r="E22" s="15" t="inlineStr">
@@ -5245,7 +5349,7 @@
       </c>
       <c r="D23" s="15" t="inlineStr">
         <is>
-          <t>Playwright keyboard, pointer, focus, and state interactions</t>
+          <t>Public type and declaration fixtures</t>
         </is>
       </c>
       <c r="E23" s="15" t="inlineStr">
@@ -5297,7 +5401,7 @@
       </c>
       <c r="D24" s="15" t="inlineStr">
         <is>
-          <t>Axe checks for canonical browser states</t>
+          <t>Playwright keyboard, pointer, focus, and state interactions</t>
         </is>
       </c>
       <c r="E24" s="15" t="inlineStr">
@@ -5349,7 +5453,7 @@
       </c>
       <c r="D25" s="15" t="inlineStr">
         <is>
-          <t>Risk-based Chromium visual baselines reviewed</t>
+          <t>Axe checks for canonical browser states</t>
         </is>
       </c>
       <c r="E25" s="15" t="inlineStr">
@@ -5370,7 +5474,7 @@
       </c>
       <c r="I25" s="15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J25" s="15" t="inlineStr"/>
@@ -5401,7 +5505,7 @@
       </c>
       <c r="D26" s="15" t="inlineStr">
         <is>
-          <t>Relevant Chromium, Firefox, WebKit, and mobile-profile checks</t>
+          <t>Risk-based Chromium visual baselines reviewed</t>
         </is>
       </c>
       <c r="E26" s="15" t="inlineStr">
@@ -5422,7 +5526,7 @@
       </c>
       <c r="I26" s="15" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="J26" s="15" t="inlineStr"/>
@@ -5453,7 +5557,7 @@
       </c>
       <c r="D27" s="15" t="inlineStr">
         <is>
-          <t>SSR or server-safe consumer behavior where applicable</t>
+          <t>Relevant Chromium, Firefox, WebKit, and mobile-profile checks</t>
         </is>
       </c>
       <c r="E27" s="15" t="inlineStr">
@@ -5495,7 +5599,7 @@
       </c>
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>Manual evidence</t>
+          <t>Automated tests</t>
         </is>
       </c>
       <c r="C28" s="15" t="inlineStr">
@@ -5505,7 +5609,7 @@
       </c>
       <c r="D28" s="15" t="inlineStr">
         <is>
-          <t>Numbered component manual-test protocol is complete</t>
+          <t>SSR or server-safe consumer behavior where applicable</t>
         </is>
       </c>
       <c r="E28" s="15" t="inlineStr">
@@ -5515,7 +5619,7 @@
       </c>
       <c r="F28" s="15" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>test</t>
         </is>
       </c>
       <c r="G28" s="15" t="inlineStr"/>
@@ -5557,7 +5661,7 @@
       </c>
       <c r="D29" s="15" t="inlineStr">
         <is>
-          <t>Latest required manual run is recorded and passes</t>
+          <t>Numbered component manual-test protocol is complete</t>
         </is>
       </c>
       <c r="E29" s="15" t="inlineStr">
@@ -5578,7 +5682,7 @@
       </c>
       <c r="I29" s="15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J29" s="15" t="inlineStr"/>
@@ -5599,7 +5703,7 @@
       </c>
       <c r="B30" s="15" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Manual evidence</t>
         </is>
       </c>
       <c r="C30" s="15" t="inlineStr">
@@ -5609,7 +5713,7 @@
       </c>
       <c r="D30" s="15" t="inlineStr">
         <is>
-          <t>Public component documentation follows the standard template</t>
+          <t>Latest required manual run is recorded and passes</t>
         </is>
       </c>
       <c r="E30" s="15" t="inlineStr">
@@ -5619,7 +5723,7 @@
       </c>
       <c r="F30" s="15" t="inlineStr">
         <is>
-          <t>docs</t>
+          <t>manual</t>
         </is>
       </c>
       <c r="G30" s="15" t="inlineStr"/>
@@ -5661,7 +5765,7 @@
       </c>
       <c r="D31" s="15" t="inlineStr">
         <is>
-          <t>Component changelog and applicable package release notes are updated</t>
+          <t>Public component documentation follows the standard template</t>
         </is>
       </c>
       <c r="E31" s="15" t="inlineStr">
@@ -5682,7 +5786,7 @@
       </c>
       <c r="I31" s="15" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="J31" s="15" t="inlineStr"/>
@@ -5703,7 +5807,7 @@
       </c>
       <c r="B32" s="15" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C32" s="15" t="inlineStr">
@@ -5713,17 +5817,17 @@
       </c>
       <c r="D32" s="15" t="inlineStr">
         <is>
-          <t>Live consumer cutover is verified without adding new legacy Core coupling</t>
+          <t>Component changelog and applicable package release notes are updated</t>
         </is>
       </c>
       <c r="E32" s="15" t="inlineStr">
         <is>
-          <t>consumer</t>
+          <t>package</t>
         </is>
       </c>
       <c r="F32" s="15" t="inlineStr">
         <is>
-          <t>consumer</t>
+          <t>docs</t>
         </is>
       </c>
       <c r="G32" s="15" t="inlineStr"/>
@@ -5734,7 +5838,7 @@
       </c>
       <c r="I32" s="15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J32" s="15" t="inlineStr"/>
@@ -5755,7 +5859,7 @@
       </c>
       <c r="B33" s="15" t="inlineStr">
         <is>
-          <t>Retirement</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="C33" s="15" t="inlineStr">
@@ -5765,17 +5869,17 @@
       </c>
       <c r="D33" s="15" t="inlineStr">
         <is>
-          <t>Legacy Core slice and authorized stale consumer evidence are removed</t>
+          <t>Live consumer cutover is verified without adding new legacy Core coupling</t>
         </is>
       </c>
       <c r="E33" s="15" t="inlineStr">
         <is>
-          <t>retirement</t>
+          <t>consumer</t>
         </is>
       </c>
       <c r="F33" s="15" t="inlineStr">
         <is>
-          <t>removal</t>
+          <t>consumer</t>
         </is>
       </c>
       <c r="G33" s="15" t="inlineStr"/>
@@ -5799,14 +5903,66 @@
         <v/>
       </c>
     </row>
+    <row r="34" ht="43" customHeight="1">
+      <c r="A34" s="15" t="inlineStr">
+        <is>
+          <t>DIA-26</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="inlineStr">
+        <is>
+          <t>Retirement</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
+          <t>Legacy Core slice and authorized stale consumer evidence are removed</t>
+        </is>
+      </c>
+      <c r="E34" s="15" t="inlineStr">
+        <is>
+          <t>retirement</t>
+        </is>
+      </c>
+      <c r="F34" s="15" t="inlineStr">
+        <is>
+          <t>removal</t>
+        </is>
+      </c>
+      <c r="G34" s="15" t="inlineStr"/>
+      <c r="H34" s="15" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
+      <c r="I34" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J34" s="15" t="inlineStr"/>
+      <c r="K34" s="15" t="inlineStr"/>
+      <c r="L34" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="M34" s="16">
+        <f>IF(H34="not applicable",IF(K34&lt;&gt;"",1,0),IF(I34="yes",IF(H34="verified",1,0),IF(OR(H34="tested",H34="verified"),1,0)))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:M33"/>
+  <autoFilter ref="A8:M34"/>
   <mergeCells count="3">
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A6:M6"/>
     <mergeCell ref="A1:M1"/>
   </mergeCells>
-  <conditionalFormatting sqref="H9:H33">
+  <conditionalFormatting sqref="H9:H34">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H9="not started"</formula>
     </cfRule>
@@ -5830,10 +5986,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="H9:H33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H9:H34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>=_Lists!$A$1:$A$7</formula1>
     </dataValidation>
-    <dataValidation sqref="I9:I33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="I9:I34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>=_Lists!$B$1:$B$2</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: replace template starter with brick consumer
</commit_message>
<xml_diff>
--- a/playground/component-coverage.xlsx
+++ b/playground/component-coverage.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="779" uniqueCount="221">
   <si>
     <t xml:space="preserve">Brick Component Coverage Index</t>
   </si>
@@ -476,22 +476,25 @@
     <t xml:space="preserve">consumer</t>
   </si>
   <si>
+    <t xml:space="preserve">../../../../apps/brick-consumer/tests/consumer.spec.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUT-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retirement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legacy Core slice and authorized stale consumer evidence are removed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">retirement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">removal</t>
+  </si>
+  <si>
     <t xml:space="preserve">not started</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BUT-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retirement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Legacy Core slice and authorized stale consumer evidence are removed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">retirement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">removal</t>
   </si>
   <si>
     <t xml:space="preserve">Card Evidence Matrix</t>
@@ -1570,7 +1573,7 @@
       </c>
       <c r="H4" s="6" t="n">
         <f aca="false">IFERROR(SUMPRODUCT(B8:B10,J8:J10)/SUM(B8:B10),0)</f>
-        <v>0.307692307692308</v>
+        <v>0.320512820512821</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1627,7 +1630,7 @@
       </c>
       <c r="C8" s="8" t="n">
         <f aca="false">COUNTIF(Button!H9:H34,"not started")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D8" s="8" t="n">
         <f aca="false">COUNTIF(Button!H9:H34,"partial")</f>
@@ -1643,7 +1646,7 @@
       </c>
       <c r="G8" s="8" t="n">
         <f aca="false">COUNTIF(Button!H9:H34,"verified")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H8" s="8" t="n">
         <f aca="false">COUNTIF(Button!H9:H34,"blocked")</f>
@@ -1655,7 +1658,7 @@
       </c>
       <c r="J8" s="9" t="n">
         <f aca="false">IFERROR(SUM(Button!M9:M34)/SUM(Button!L9:L34),0)</f>
-        <v>0.923076923076923</v>
+        <v>0.961538461538462</v>
       </c>
       <c r="K8" s="8" t="str">
         <f aca="false">IF(COUNTIFS(Button!E9:E34,"package",Button!M9:M34,"&lt;1")=0,"complete","open")</f>
@@ -1663,7 +1666,7 @@
       </c>
       <c r="L8" s="8" t="str">
         <f aca="false">IF(COUNTIFS(Button!E9:E34,"consumer",Button!M9:M34,"&lt;1")=0,"complete","open")</f>
-        <v>open</v>
+        <v>complete</v>
       </c>
       <c r="M8" s="8" t="str">
         <f aca="false">IF(COUNTIFS(Button!E9:E34,"retirement",Button!M9:M34,"&lt;1")=0,"complete","open")</f>
@@ -2072,14 +2075,14 @@
       </c>
       <c r="D4" s="5" t="n">
         <f aca="false">SUM(M9:M34)</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F4" s="6" t="n">
         <f aca="false">IFERROR(D4/SUM(L9:L34),0)</f>
-        <v>0.923076923076923</v>
+        <v>0.961538461538462</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>4</v>
@@ -3140,21 +3143,25 @@
       <c r="F33" s="15" t="s">
         <v>144</v>
       </c>
-      <c r="G33" s="15"/>
+      <c r="G33" s="15" t="s">
+        <v>145</v>
+      </c>
       <c r="H33" s="15" t="s">
-        <v>145</v>
+        <v>71</v>
       </c>
       <c r="I33" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="J33" s="15"/>
+      <c r="J33" s="19" t="n">
+        <v>46219</v>
+      </c>
       <c r="K33" s="15"/>
       <c r="L33" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M33" s="18" t="n">
         <f aca="false">IF(H33="not applicable",IF(K33&lt;&gt;"",1,0),IF(I33="yes",IF(H33="verified",1,0),IF(OR(H33="tested",H33="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3178,7 +3185,7 @@
       </c>
       <c r="G34" s="15"/>
       <c r="H34" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I34" s="15" t="s">
         <v>72</v>
@@ -3296,7 +3303,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3313,7 +3320,7 @@
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -3432,7 +3439,7 @@
     </row>
     <row r="9" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B9" s="15" t="s">
         <v>59</v>
@@ -3441,7 +3448,7 @@
         <v>6</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E9" s="15" t="s">
         <v>61</v>
@@ -3451,7 +3458,7 @@
       </c>
       <c r="G9" s="15"/>
       <c r="H9" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I9" s="15" t="s">
         <v>65</v>
@@ -3468,7 +3475,7 @@
     </row>
     <row r="10" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B10" s="15" t="s">
         <v>67</v>
@@ -3477,7 +3484,7 @@
         <v>6</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E10" s="15" t="s">
         <v>61</v>
@@ -3487,7 +3494,7 @@
       </c>
       <c r="G10" s="15"/>
       <c r="H10" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I10" s="15" t="s">
         <v>72</v>
@@ -3504,7 +3511,7 @@
     </row>
     <row r="11" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B11" s="15" t="s">
         <v>59</v>
@@ -3513,7 +3520,7 @@
         <v>6</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E11" s="15" t="s">
         <v>61</v>
@@ -3523,7 +3530,7 @@
       </c>
       <c r="G11" s="15"/>
       <c r="H11" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I11" s="15" t="s">
         <v>65</v>
@@ -3540,7 +3547,7 @@
     </row>
     <row r="12" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B12" s="15" t="s">
         <v>59</v>
@@ -3549,7 +3556,7 @@
         <v>6</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E12" s="15" t="s">
         <v>61</v>
@@ -3559,7 +3566,7 @@
       </c>
       <c r="G12" s="15"/>
       <c r="H12" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I12" s="15" t="s">
         <v>65</v>
@@ -3576,7 +3583,7 @@
     </row>
     <row r="13" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B13" s="15" t="s">
         <v>81</v>
@@ -3595,7 +3602,7 @@
       </c>
       <c r="G13" s="15"/>
       <c r="H13" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I13" s="15" t="s">
         <v>65</v>
@@ -3612,7 +3619,7 @@
     </row>
     <row r="14" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B14" s="15" t="s">
         <v>81</v>
@@ -3621,7 +3628,7 @@
         <v>6</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E14" s="15" t="s">
         <v>61</v>
@@ -3631,7 +3638,7 @@
       </c>
       <c r="G14" s="15"/>
       <c r="H14" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I14" s="15" t="s">
         <v>72</v>
@@ -3648,7 +3655,7 @@
     </row>
     <row r="15" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>88</v>
@@ -3667,7 +3674,7 @@
       </c>
       <c r="G15" s="15"/>
       <c r="H15" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I15" s="15" t="s">
         <v>72</v>
@@ -3684,7 +3691,7 @@
     </row>
     <row r="16" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B16" s="15" t="s">
         <v>88</v>
@@ -3693,7 +3700,7 @@
         <v>6</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E16" s="15" t="s">
         <v>61</v>
@@ -3703,7 +3710,7 @@
       </c>
       <c r="G16" s="15"/>
       <c r="H16" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I16" s="15" t="s">
         <v>72</v>
@@ -3720,7 +3727,7 @@
     </row>
     <row r="17" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B17" s="15" t="s">
         <v>88</v>
@@ -3739,7 +3746,7 @@
       </c>
       <c r="G17" s="15"/>
       <c r="H17" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I17" s="15" t="s">
         <v>72</v>
@@ -3756,7 +3763,7 @@
     </row>
     <row r="18" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B18" s="15" t="s">
         <v>88</v>
@@ -3765,7 +3772,7 @@
         <v>6</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E18" s="15" t="s">
         <v>61</v>
@@ -3775,7 +3782,7 @@
       </c>
       <c r="G18" s="15"/>
       <c r="H18" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I18" s="15" t="s">
         <v>72</v>
@@ -3792,7 +3799,7 @@
     </row>
     <row r="19" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B19" s="15" t="s">
         <v>88</v>
@@ -3811,7 +3818,7 @@
       </c>
       <c r="G19" s="15"/>
       <c r="H19" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I19" s="15" t="s">
         <v>72</v>
@@ -3828,7 +3835,7 @@
     </row>
     <row r="20" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B20" s="15" t="s">
         <v>88</v>
@@ -3837,7 +3844,7 @@
         <v>6</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E20" s="15" t="s">
         <v>61</v>
@@ -3847,7 +3854,7 @@
       </c>
       <c r="G20" s="15"/>
       <c r="H20" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I20" s="15" t="s">
         <v>72</v>
@@ -3864,7 +3871,7 @@
     </row>
     <row r="21" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B21" s="15" t="s">
         <v>88</v>
@@ -3883,7 +3890,7 @@
       </c>
       <c r="G21" s="15"/>
       <c r="H21" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I21" s="15" t="s">
         <v>65</v>
@@ -3900,7 +3907,7 @@
     </row>
     <row r="22" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>107</v>
@@ -3919,7 +3926,7 @@
       </c>
       <c r="G22" s="15"/>
       <c r="H22" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I22" s="15" t="s">
         <v>65</v>
@@ -3936,7 +3943,7 @@
     </row>
     <row r="23" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B23" s="15" t="s">
         <v>107</v>
@@ -3945,7 +3952,7 @@
         <v>6</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E23" s="15" t="s">
         <v>61</v>
@@ -3955,7 +3962,7 @@
       </c>
       <c r="G23" s="15"/>
       <c r="H23" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I23" s="15" t="s">
         <v>65</v>
@@ -3972,7 +3979,7 @@
     </row>
     <row r="24" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B24" s="15" t="s">
         <v>107</v>
@@ -3991,7 +3998,7 @@
       </c>
       <c r="G24" s="15"/>
       <c r="H24" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I24" s="15" t="s">
         <v>65</v>
@@ -4008,7 +4015,7 @@
     </row>
     <row r="25" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B25" s="15" t="s">
         <v>107</v>
@@ -4027,7 +4034,7 @@
       </c>
       <c r="G25" s="15"/>
       <c r="H25" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I25" s="15" t="s">
         <v>65</v>
@@ -4044,7 +4051,7 @@
     </row>
     <row r="26" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B26" s="15" t="s">
         <v>107</v>
@@ -4063,7 +4070,7 @@
       </c>
       <c r="G26" s="15"/>
       <c r="H26" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I26" s="15" t="s">
         <v>72</v>
@@ -4080,7 +4087,7 @@
     </row>
     <row r="27" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B27" s="15" t="s">
         <v>107</v>
@@ -4099,7 +4106,7 @@
       </c>
       <c r="G27" s="15"/>
       <c r="H27" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I27" s="15" t="s">
         <v>65</v>
@@ -4116,7 +4123,7 @@
     </row>
     <row r="28" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B28" s="15" t="s">
         <v>107</v>
@@ -4125,7 +4132,7 @@
         <v>6</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E28" s="15" t="s">
         <v>61</v>
@@ -4135,7 +4142,7 @@
       </c>
       <c r="G28" s="15"/>
       <c r="H28" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I28" s="15" t="s">
         <v>65</v>
@@ -4152,7 +4159,7 @@
     </row>
     <row r="29" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B29" s="15" t="s">
         <v>128</v>
@@ -4171,7 +4178,7 @@
       </c>
       <c r="G29" s="15"/>
       <c r="H29" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I29" s="15" t="s">
         <v>65</v>
@@ -4188,7 +4195,7 @@
     </row>
     <row r="30" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="15" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B30" s="15" t="s">
         <v>128</v>
@@ -4207,7 +4214,7 @@
       </c>
       <c r="G30" s="15"/>
       <c r="H30" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I30" s="15" t="s">
         <v>72</v>
@@ -4224,7 +4231,7 @@
     </row>
     <row r="31" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="15" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B31" s="15" t="s">
         <v>134</v>
@@ -4243,7 +4250,7 @@
       </c>
       <c r="G31" s="15"/>
       <c r="H31" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I31" s="15" t="s">
         <v>72</v>
@@ -4260,7 +4267,7 @@
     </row>
     <row r="32" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="15" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B32" s="15" t="s">
         <v>134</v>
@@ -4279,7 +4286,7 @@
       </c>
       <c r="G32" s="15"/>
       <c r="H32" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I32" s="15" t="s">
         <v>65</v>
@@ -4296,7 +4303,7 @@
     </row>
     <row r="33" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="15" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B33" s="15" t="s">
         <v>142</v>
@@ -4315,7 +4322,7 @@
       </c>
       <c r="G33" s="15"/>
       <c r="H33" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I33" s="15" t="s">
         <v>72</v>
@@ -4332,7 +4339,7 @@
     </row>
     <row r="34" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="15" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B34" s="15" t="s">
         <v>147</v>
@@ -4351,7 +4358,7 @@
       </c>
       <c r="G34" s="15"/>
       <c r="H34" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I34" s="15" t="s">
         <v>72</v>
@@ -4445,7 +4452,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4462,7 +4469,7 @@
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -4581,7 +4588,7 @@
     </row>
     <row r="9" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B9" s="15" t="s">
         <v>59</v>
@@ -4590,7 +4597,7 @@
         <v>6</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E9" s="15" t="s">
         <v>61</v>
@@ -4600,7 +4607,7 @@
       </c>
       <c r="G9" s="15"/>
       <c r="H9" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I9" s="15" t="s">
         <v>65</v>
@@ -4617,7 +4624,7 @@
     </row>
     <row r="10" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B10" s="15" t="s">
         <v>67</v>
@@ -4626,7 +4633,7 @@
         <v>6</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E10" s="15" t="s">
         <v>61</v>
@@ -4636,7 +4643,7 @@
       </c>
       <c r="G10" s="15"/>
       <c r="H10" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I10" s="15" t="s">
         <v>72</v>
@@ -4653,7 +4660,7 @@
     </row>
     <row r="11" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B11" s="15" t="s">
         <v>59</v>
@@ -4662,7 +4669,7 @@
         <v>6</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E11" s="15" t="s">
         <v>61</v>
@@ -4672,7 +4679,7 @@
       </c>
       <c r="G11" s="15"/>
       <c r="H11" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I11" s="15" t="s">
         <v>65</v>
@@ -4689,7 +4696,7 @@
     </row>
     <row r="12" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B12" s="15" t="s">
         <v>59</v>
@@ -4698,7 +4705,7 @@
         <v>6</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E12" s="15" t="s">
         <v>61</v>
@@ -4708,7 +4715,7 @@
       </c>
       <c r="G12" s="15"/>
       <c r="H12" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I12" s="15" t="s">
         <v>65</v>
@@ -4725,7 +4732,7 @@
     </row>
     <row r="13" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B13" s="15" t="s">
         <v>81</v>
@@ -4744,7 +4751,7 @@
       </c>
       <c r="G13" s="15"/>
       <c r="H13" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I13" s="15" t="s">
         <v>65</v>
@@ -4761,7 +4768,7 @@
     </row>
     <row r="14" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B14" s="15" t="s">
         <v>81</v>
@@ -4770,7 +4777,7 @@
         <v>6</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E14" s="15" t="s">
         <v>61</v>
@@ -4780,7 +4787,7 @@
       </c>
       <c r="G14" s="15"/>
       <c r="H14" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I14" s="15" t="s">
         <v>72</v>
@@ -4797,7 +4804,7 @@
     </row>
     <row r="15" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>88</v>
@@ -4816,7 +4823,7 @@
       </c>
       <c r="G15" s="15"/>
       <c r="H15" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I15" s="15" t="s">
         <v>72</v>
@@ -4833,7 +4840,7 @@
     </row>
     <row r="16" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B16" s="15" t="s">
         <v>88</v>
@@ -4842,7 +4849,7 @@
         <v>6</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E16" s="15" t="s">
         <v>61</v>
@@ -4852,7 +4859,7 @@
       </c>
       <c r="G16" s="15"/>
       <c r="H16" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I16" s="15" t="s">
         <v>72</v>
@@ -4869,7 +4876,7 @@
     </row>
     <row r="17" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B17" s="15" t="s">
         <v>88</v>
@@ -4888,7 +4895,7 @@
       </c>
       <c r="G17" s="15"/>
       <c r="H17" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I17" s="15" t="s">
         <v>72</v>
@@ -4905,7 +4912,7 @@
     </row>
     <row r="18" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="15" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B18" s="15" t="s">
         <v>88</v>
@@ -4914,7 +4921,7 @@
         <v>6</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E18" s="15" t="s">
         <v>61</v>
@@ -4924,7 +4931,7 @@
       </c>
       <c r="G18" s="15"/>
       <c r="H18" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I18" s="15" t="s">
         <v>72</v>
@@ -4941,7 +4948,7 @@
     </row>
     <row r="19" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B19" s="15" t="s">
         <v>88</v>
@@ -4960,7 +4967,7 @@
       </c>
       <c r="G19" s="15"/>
       <c r="H19" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I19" s="15" t="s">
         <v>72</v>
@@ -4977,7 +4984,7 @@
     </row>
     <row r="20" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B20" s="15" t="s">
         <v>88</v>
@@ -4986,7 +4993,7 @@
         <v>6</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E20" s="15" t="s">
         <v>61</v>
@@ -4996,7 +5003,7 @@
       </c>
       <c r="G20" s="15"/>
       <c r="H20" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I20" s="15" t="s">
         <v>72</v>
@@ -5013,7 +5020,7 @@
     </row>
     <row r="21" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B21" s="15" t="s">
         <v>88</v>
@@ -5032,7 +5039,7 @@
       </c>
       <c r="G21" s="15"/>
       <c r="H21" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I21" s="15" t="s">
         <v>65</v>
@@ -5049,7 +5056,7 @@
     </row>
     <row r="22" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>107</v>
@@ -5068,7 +5075,7 @@
       </c>
       <c r="G22" s="15"/>
       <c r="H22" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I22" s="15" t="s">
         <v>65</v>
@@ -5085,7 +5092,7 @@
     </row>
     <row r="23" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B23" s="15" t="s">
         <v>107</v>
@@ -5094,7 +5101,7 @@
         <v>6</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E23" s="15" t="s">
         <v>61</v>
@@ -5104,7 +5111,7 @@
       </c>
       <c r="G23" s="15"/>
       <c r="H23" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I23" s="15" t="s">
         <v>65</v>
@@ -5121,7 +5128,7 @@
     </row>
     <row r="24" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B24" s="15" t="s">
         <v>107</v>
@@ -5140,7 +5147,7 @@
       </c>
       <c r="G24" s="15"/>
       <c r="H24" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I24" s="15" t="s">
         <v>65</v>
@@ -5157,7 +5164,7 @@
     </row>
     <row r="25" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B25" s="15" t="s">
         <v>107</v>
@@ -5176,7 +5183,7 @@
       </c>
       <c r="G25" s="15"/>
       <c r="H25" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I25" s="15" t="s">
         <v>65</v>
@@ -5193,7 +5200,7 @@
     </row>
     <row r="26" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B26" s="15" t="s">
         <v>107</v>
@@ -5212,7 +5219,7 @@
       </c>
       <c r="G26" s="15"/>
       <c r="H26" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I26" s="15" t="s">
         <v>72</v>
@@ -5229,7 +5236,7 @@
     </row>
     <row r="27" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B27" s="15" t="s">
         <v>107</v>
@@ -5248,7 +5255,7 @@
       </c>
       <c r="G27" s="15"/>
       <c r="H27" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I27" s="15" t="s">
         <v>65</v>
@@ -5265,7 +5272,7 @@
     </row>
     <row r="28" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="15" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B28" s="15" t="s">
         <v>107</v>
@@ -5274,7 +5281,7 @@
         <v>6</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E28" s="15" t="s">
         <v>61</v>
@@ -5284,7 +5291,7 @@
       </c>
       <c r="G28" s="15"/>
       <c r="H28" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I28" s="15" t="s">
         <v>65</v>
@@ -5301,7 +5308,7 @@
     </row>
     <row r="29" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B29" s="15" t="s">
         <v>128</v>
@@ -5320,7 +5327,7 @@
       </c>
       <c r="G29" s="15"/>
       <c r="H29" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I29" s="15" t="s">
         <v>65</v>
@@ -5337,7 +5344,7 @@
     </row>
     <row r="30" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="15" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B30" s="15" t="s">
         <v>128</v>
@@ -5356,7 +5363,7 @@
       </c>
       <c r="G30" s="15"/>
       <c r="H30" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I30" s="15" t="s">
         <v>72</v>
@@ -5373,7 +5380,7 @@
     </row>
     <row r="31" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="15" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B31" s="15" t="s">
         <v>134</v>
@@ -5392,7 +5399,7 @@
       </c>
       <c r="G31" s="15"/>
       <c r="H31" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I31" s="15" t="s">
         <v>72</v>
@@ -5409,7 +5416,7 @@
     </row>
     <row r="32" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="15" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B32" s="15" t="s">
         <v>134</v>
@@ -5428,7 +5435,7 @@
       </c>
       <c r="G32" s="15"/>
       <c r="H32" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I32" s="15" t="s">
         <v>65</v>
@@ -5445,7 +5452,7 @@
     </row>
     <row r="33" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="15" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B33" s="15" t="s">
         <v>142</v>
@@ -5464,7 +5471,7 @@
       </c>
       <c r="G33" s="15"/>
       <c r="H33" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I33" s="15" t="s">
         <v>72</v>
@@ -5481,7 +5488,7 @@
     </row>
     <row r="34" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="15" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B34" s="15" t="s">
         <v>147</v>
@@ -5500,7 +5507,7 @@
       </c>
       <c r="G34" s="15"/>
       <c r="H34" s="15" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="I34" s="15" t="s">
         <v>72</v>
@@ -5579,7 +5586,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>72</v>
@@ -5587,7 +5594,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>65</v>
@@ -5595,7 +5602,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5610,12 +5617,12 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(brick): record card coverage
</commit_message>
<xml_diff>
--- a/playground/component-coverage.xlsx
+++ b/playground/component-coverage.xlsx
@@ -5,21 +5,21 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="2" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Index" sheetId="1" state="hidden" r:id="rId3"/>
-    <sheet name="Instructions" sheetId="2" state="hidden" r:id="rId4"/>
+    <sheet name="Index" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Instructions" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Button" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Card" sheetId="4" state="hidden" r:id="rId6"/>
-    <sheet name="Dialog" sheetId="5" state="hidden" r:id="rId7"/>
+    <sheet name="Card" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Dialog" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="_Lists" sheetId="6" state="hidden" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">Button!$A$1:$M$34</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Titles" vbProcedure="false">Button!$1:$8</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Button!$A$8:$M$34</definedName>
-    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Card!$A$1:$M$34</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Card!$A$1:$M$41</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Titles" vbProcedure="false">Card!$1:$8</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Card!$A$8:$M$34</definedName>
     <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Area" vbProcedure="false">Dialog!$A$1:$M$34</definedName>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="779" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="869" uniqueCount="285">
   <si>
     <t xml:space="preserve">Brick Component Coverage Index</t>
   </si>
@@ -500,180 +500,375 @@
     <t xml:space="preserve">Card Evidence Matrix</t>
   </si>
   <si>
+    <t xml:space="preserve">Evidence gates for the adopted static Card compound, its seven public parts, package proof, consumer cutover, and dependency-blocked legacy retirement.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Namespace</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Static Card namespace implementation has no Core, application, or local behavior wrapper</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../src/components/card/Card.tsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atom capability audit confirms Card owns no behavior and requires no Atom patch or local workaround</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../../docs/card-component-brief.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Root and card subpath exports, declarations, defaults, and closed unions match the adopted brief</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../src/card.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All parts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Native props, refs, className, style, events, children, and overridable slots forward on every public part</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../test/components/card.test.tsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Root</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neutral div default, restricted semantic elements, variant and size defaults, and no invented role or focus state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Header</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Title, description, and compact trailing action preserve source order and resilient narrow-screen layout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">manual-tests/card.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heading defaults to h3 and supports only h1 through h6 with native heading semantics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supporting text renders as a native paragraph and forwards its complete public DOM contract</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Action</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compact trailing layout creates no role, focus, click, keyboard, or generated control behavior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/card.spec.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Content</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional body region renders one native element and omitted anatomy creates no empty regions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Footer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional footer preserves explicit controls, logical order, wrapping, and visible focus at narrow widths</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compiled CSS uses public brick classes, component tokens, layers, logical properties, and semantic roles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../src/components/card/card.css</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outline, elevated, and subtle variants plus small, medium, and large density recipes remain distinct in light and dark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Canonical article and every partial anatomy are built from public Card parts and Brick Button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every variant and size plus media and single-action-link composition are represented</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mobile-first constrained layouts and intentional wide layouts preserve natural Card height and containment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Light, dark, scoped appearance, forced colors, and reduced motion retain hierarchy and boundaries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Long content, unbroken text, localization, 400 percent zoom, and RTL remain contained and readable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Public Card tokens, stable classes, style, data attributes, and overridable part slots are inspectable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stable Card route and deterministic scenario selectors support repeatable browser tests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vitest and Testing Library cover the complete component and native DOM contract</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Public type, declaration, invalid-prop, root export, and card-subpath fixtures pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Playwright verifies static semantics, explicit-control focus, accessible link naming, reflow, and zoom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Axe reports no automatically detectable violations for canonical Card states</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Six deterministic Chromium visual baselines are reviewed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chromium, Firefox, WebKit, Pixel, and iPhone release matrix records 73 passes and 42 intentional skips</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../playwright.config.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SSR, package boundary, tarball, and clean React 18 and React 19 consumer verification pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../test/package/ssr.test.mjs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numbered ten-step Card manual-test protocol is complete</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latest owner run is recorded and passes after every discovered finding was corrected and retested</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Public Card documentation follows the standard template and documents whole-card accessibility</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../docs/components/card/README.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Card changelog and package release notes record the initial contract and dark-elevation correction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../docs/components/card/CHANGELOG.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Independent consumer uses public Card for project, checklist, and invitation surfaces and passes ten browser checks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAR-33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legacy Card family</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legacy Card source, exports, compatibility, and stale evidence are removed only after dependents are resolved</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../../docs/core-dependency-ledger.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">blocked</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dialog, Drawer, and AlertDialog still consume legacy Card parts or types.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dialog Evidence Matrix</t>
+  </si>
+  <si>
     <t xml:space="preserve">Common requirements from Brick's adopted quality contract. Add approved anatomy and component-specific rows after the component brief lands.</t>
   </si>
   <si>
-    <t xml:space="preserve">CAR-01</t>
+    <t xml:space="preserve">DIA-01</t>
   </si>
   <si>
     <t xml:space="preserve">Implementation uses public Atom behavior without Core or local headless wrappers</t>
   </si>
   <si>
-    <t xml:space="preserve">CAR-02</t>
+    <t xml:space="preserve">DIA-02</t>
   </si>
   <si>
     <t xml:space="preserve">Atom capability audit covers mobile behavior and every Atom-owned gap is resolved through a released dependency</t>
   </si>
   <si>
-    <t xml:space="preserve">CAR-03</t>
+    <t xml:space="preserve">DIA-03</t>
   </si>
   <si>
     <t xml:space="preserve">Public export and declaration surface match the approved brief</t>
   </si>
   <si>
-    <t xml:space="preserve">CAR-04</t>
+    <t xml:space="preserve">DIA-04</t>
   </si>
   <si>
     <t xml:space="preserve">Native props, refs, composition, and public slots follow the adopted API contract</t>
   </si>
   <si>
-    <t xml:space="preserve">CAR-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR-06</t>
+    <t xml:space="preserve">DIA-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-06</t>
   </si>
   <si>
     <t xml:space="preserve">Default recipe and every approved visual option are implemented</t>
   </si>
   <si>
-    <t xml:space="preserve">CAR-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR-08</t>
+    <t xml:space="preserve">DIA-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-08</t>
   </si>
   <si>
     <t xml:space="preserve">Every public recipe, size, and important state</t>
   </si>
   <si>
-    <t xml:space="preserve">CAR-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR-10</t>
+    <t xml:space="preserve">DIA-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-10</t>
   </si>
   <si>
     <t xml:space="preserve">Light, dark, and relevant preference modes</t>
   </si>
   <si>
-    <t xml:space="preserve">CAR-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR-12</t>
+    <t xml:space="preserve">DIA-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-12</t>
   </si>
   <si>
     <t xml:space="preserve">Token, className, style, slot, and documented part customization</t>
   </si>
   <si>
-    <t xml:space="preserve">CAR-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR-15</t>
+    <t xml:space="preserve">DIA-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-15</t>
   </si>
   <si>
     <t xml:space="preserve">Public type and declaration fixtures</t>
   </si>
   <si>
-    <t xml:space="preserve">CAR-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR-20</t>
+    <t xml:space="preserve">DIA-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-20</t>
   </si>
   <si>
     <t xml:space="preserve">SSR or server-safe consumer behavior where applicable</t>
   </si>
   <si>
-    <t xml:space="preserve">CAR-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dialog Evidence Matrix</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIA-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIA-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIA-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIA-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIA-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIA-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIA-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIA-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIA-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIA-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIA-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIA-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIA-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIA-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIA-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIA-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIA-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIA-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIA-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIA-20</t>
-  </si>
-  <si>
     <t xml:space="preserve">DIA-21</t>
   </si>
   <si>
@@ -696,9 +891,6 @@
   </si>
   <si>
     <t xml:space="preserve">implemented</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blocked</t>
   </si>
   <si>
     <t xml:space="preserve">not applicable</t>
@@ -974,7 +1166,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="19">
+  <dxfs count="21">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1017,7 +1209,23 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFFEE2E2"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FF475569"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF991B1B"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1242,8 +1450,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="CardEvidence" displayName="CardEvidence" ref="A8:M34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A8:M34"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="CardEvidence" displayName="CardEvidence" ref="A8:M41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A8:M41"/>
   <tableColumns count="13">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Area"/>
@@ -1566,14 +1774,14 @@
       </c>
       <c r="F4" s="5" t="n">
         <f aca="false">SUM(H8:H10)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>5</v>
       </c>
       <c r="H4" s="6" t="n">
         <f aca="false">IFERROR(SUMPRODUCT(B8:B10,J8:J10)/SUM(B8:B10),0)</f>
-        <v>0.320512820512821</v>
+        <v>0.670588235294118</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1682,56 +1890,56 @@
         <v>20</v>
       </c>
       <c r="B9" s="8" t="n">
-        <f aca="false">COUNTA(Card!A9:A34)</f>
-        <v>26</v>
+        <f aca="false">COUNTA(Card!A9:A41)</f>
+        <v>33</v>
       </c>
       <c r="C9" s="8" t="n">
-        <f aca="false">COUNTIF(Card!H9:H34,"not started")</f>
-        <v>26</v>
+        <f aca="false">COUNTIF(Card!H9:H41,"not started")</f>
+        <v>0</v>
       </c>
       <c r="D9" s="8" t="n">
-        <f aca="false">COUNTIF(Card!H9:H34,"partial")</f>
+        <f aca="false">COUNTIF(Card!H9:H41,"partial")</f>
         <v>0</v>
       </c>
       <c r="E9" s="8" t="n">
-        <f aca="false">COUNTIF(Card!H9:H34,"implemented")</f>
+        <f aca="false">COUNTIF(Card!H9:H41,"implemented")</f>
         <v>0</v>
       </c>
       <c r="F9" s="8" t="n">
-        <f aca="false">COUNTIF(Card!H9:H34,"tested")</f>
+        <f aca="false">COUNTIF(Card!H9:H41,"tested")</f>
+        <v>18</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <f aca="false">COUNTIF(Card!H9:H41,"verified")</f>
+        <v>14</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <f aca="false">COUNTIF(Card!H9:H41,"blocked")</f>
+        <v>1</v>
+      </c>
+      <c r="I9" s="8" t="n">
+        <f aca="false">COUNTIF(Card!H9:H41,"not applicable")</f>
         <v>0</v>
       </c>
-      <c r="G9" s="8" t="n">
-        <f aca="false">COUNTIF(Card!H9:H34,"verified")</f>
-        <v>0</v>
-      </c>
-      <c r="H9" s="8" t="n">
-        <f aca="false">COUNTIF(Card!H9:H34,"blocked")</f>
-        <v>0</v>
-      </c>
-      <c r="I9" s="8" t="n">
-        <f aca="false">COUNTIF(Card!H9:H34,"not applicable")</f>
-        <v>0</v>
-      </c>
       <c r="J9" s="9" t="n">
-        <f aca="false">IFERROR(SUM(Card!M9:M34)/SUM(Card!L9:L34),0)</f>
-        <v>0</v>
+        <f aca="false">IFERROR(SUM(Card!M9:M41)/SUM(Card!L9:L41),0)</f>
+        <v>0.96969696969697</v>
       </c>
       <c r="K9" s="8" t="str">
-        <f aca="false">IF(COUNTIFS(Card!E9:E34,"package",Card!M9:M34,"&lt;1")=0,"complete","open")</f>
-        <v>open</v>
+        <f aca="false">IF(COUNTIFS(Card!E9:E41,"package",Card!M9:M41,"&lt;1")=0,"complete","open")</f>
+        <v>complete</v>
       </c>
       <c r="L9" s="8" t="str">
-        <f aca="false">IF(COUNTIFS(Card!E9:E34,"consumer",Card!M9:M34,"&lt;1")=0,"complete","open")</f>
-        <v>open</v>
+        <f aca="false">IF(COUNTIFS(Card!E9:E41,"consumer",Card!M9:M41,"&lt;1")=0,"complete","open")</f>
+        <v>complete</v>
       </c>
       <c r="M9" s="8" t="str">
-        <f aca="false">IF(COUNTIFS(Card!E9:E34,"retirement",Card!M9:M34,"&lt;1")=0,"complete","open")</f>
+        <f aca="false">IF(COUNTIFS(Card!E9:E41,"retirement",Card!M9:M41,"&lt;1")=0,"complete","open")</f>
         <v>open</v>
       </c>
       <c r="N9" s="8" t="str">
         <f aca="false">IF(H9&gt;0,"blocked",IF(AND(J9=1,K9="complete",L9="complete",M9="complete"),"complete",IF(J9=0,"not started","in progress")))</f>
-        <v>not started</v>
+        <v>blocked</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1797,25 +2005,25 @@
     <mergeCell ref="A2:N2"/>
   </mergeCells>
   <conditionalFormatting sqref="N8:N10">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>$N8="not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>$N8="partial"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>$N8="implemented"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>$N8="tested"</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>$N8="verified"</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>$N8="blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$N8="not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3208,25 +3416,25 @@
     <mergeCell ref="A6:M6"/>
   </mergeCells>
   <conditionalFormatting sqref="H9:H34">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>$H9="not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>$H9="partial"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>$H9="implemented"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>$H9="tested"</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>$H9="verified"</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>$H9="blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$H9="not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3258,11 +3466,14 @@
     <hyperlink ref="G23" r:id="rId15" display="../test/types/public-api.test.ts"/>
     <hyperlink ref="G24" r:id="rId16" display="tests/button.spec.ts"/>
     <hyperlink ref="G25" r:id="rId17" display="tests/foundation.spec.ts"/>
-    <hyperlink ref="G27" r:id="rId18" display="../../playwright.config.ts"/>
-    <hyperlink ref="G28" r:id="rId19" display="../scripts/verify-consumers.mjs"/>
-    <hyperlink ref="G29" r:id="rId20" display="manual-tests/button.md"/>
-    <hyperlink ref="G31" r:id="rId21" display="../docs/components/button/README.md"/>
-    <hyperlink ref="G32" r:id="rId22" display="../docs/components/button/CHANGELOG.md"/>
+    <hyperlink ref="G26" r:id="rId18" display="tests/visual.spec.ts"/>
+    <hyperlink ref="G27" r:id="rId19" display="../../playwright.config.ts"/>
+    <hyperlink ref="G28" r:id="rId20" display="../scripts/verify-consumers.mjs"/>
+    <hyperlink ref="G29" r:id="rId21" display="manual-tests/button.md"/>
+    <hyperlink ref="G30" r:id="rId22" display="manual-tests/button.md"/>
+    <hyperlink ref="G31" r:id="rId23" display="../docs/components/button/README.md"/>
+    <hyperlink ref="G32" r:id="rId24" display="../docs/components/button/CHANGELOG.md"/>
+    <hyperlink ref="G33" r:id="rId25" display="../../../../apps/brick-consumer/tests/consumer.spec.ts"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3271,9 +3482,9 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId23"/>
+  <drawing r:id="rId26"/>
   <tableParts>
-    <tablePart r:id="rId24"/>
+    <tablePart r:id="rId27"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3283,7 +3494,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:M34"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr defaultColWidth="8.8046875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
@@ -3340,42 +3551,42 @@
         <v>7</v>
       </c>
       <c r="B4" s="5" t="n">
-        <f aca="false">COUNTA(A9:A34)</f>
-        <v>26</v>
+        <f aca="false">COUNTA(A9:A41)</f>
+        <v>33</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>45</v>
       </c>
       <c r="D4" s="5" t="n">
-        <f aca="false">SUM(M9:M34)</f>
-        <v>0</v>
+        <f aca="false">SUM(M9:M41)</f>
+        <v>32</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F4" s="6" t="n">
-        <f aca="false">IFERROR(D4/SUM(L9:L34),0)</f>
-        <v>0</v>
+        <f aca="false">IFERROR(D4/SUM(L9:L41),0)</f>
+        <v>0.96969696969697</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>4</v>
       </c>
       <c r="H4" s="5" t="n">
-        <f aca="false">COUNTIF(H9:H34,"blocked")</f>
-        <v>0</v>
+        <f aca="false">COUNTIF(H9:H41,"blocked")</f>
+        <v>1</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>15</v>
       </c>
       <c r="J4" s="5" t="str">
-        <f aca="false">IF(COUNTIFS(E9:E34,"package",M9:M34,"&lt;1")=0,"complete","open")</f>
-        <v>open</v>
+        <f aca="false">IF(COUNTIFS(E9:E41,"package",M9:M41,"&lt;1")=0,"complete","open")</f>
+        <v>complete</v>
       </c>
       <c r="K4" s="4" t="s">
         <v>17</v>
       </c>
       <c r="L4" s="5" t="str">
-        <f aca="false">IF(COUNTIFS(E9:E34,"retirement",M9:M34,"&lt;1")=0,"complete","open")</f>
+        <f aca="false">IF(COUNTIFS(E9:E41,"retirement",M9:M41,"&lt;1")=0,"complete","open")</f>
         <v>open</v>
       </c>
     </row>
@@ -3445,10 +3656,10 @@
         <v>59</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>6</v>
+        <v>155</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E9" s="15" t="s">
         <v>61</v>
@@ -3456,26 +3667,30 @@
       <c r="F9" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="G9" s="15"/>
+      <c r="G9" s="15" t="s">
+        <v>157</v>
+      </c>
       <c r="H9" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I9" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="J9" s="15"/>
+      <c r="J9" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K9" s="15"/>
       <c r="L9" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M9" s="18" t="n">
         <f aca="false">IF(H9="not applicable",IF(K9&lt;&gt;"",1,0),IF(I9="yes",IF(H9="verified",1,0),IF(OR(H9="tested",H9="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B10" s="15" t="s">
         <v>67</v>
@@ -3484,7 +3699,7 @@
         <v>6</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E10" s="15" t="s">
         <v>61</v>
@@ -3492,35 +3707,39 @@
       <c r="F10" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="G10" s="15"/>
+      <c r="G10" s="15" t="s">
+        <v>160</v>
+      </c>
       <c r="H10" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I10" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="J10" s="15"/>
+      <c r="J10" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K10" s="15"/>
       <c r="L10" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M10" s="18" t="n">
         <f aca="false">IF(H10="not applicable",IF(K10&lt;&gt;"",1,0),IF(I10="yes",IF(H10="verified",1,0),IF(OR(H10="tested",H10="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B11" s="15" t="s">
         <v>59</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>6</v>
+        <v>155</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="E11" s="15" t="s">
         <v>61</v>
@@ -3528,503 +3747,559 @@
       <c r="F11" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="G11" s="15"/>
+      <c r="G11" s="15" t="s">
+        <v>163</v>
+      </c>
       <c r="H11" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I11" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="J11" s="15"/>
+      <c r="J11" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K11" s="15"/>
       <c r="L11" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M11" s="18" t="n">
         <f aca="false">IF(H11="not applicable",IF(K11&lt;&gt;"",1,0),IF(I11="yes",IF(H11="verified",1,0),IF(OR(H11="tested",H11="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B12" s="15" t="s">
         <v>59</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>6</v>
+        <v>165</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="E12" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="G12" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G12" s="15" t="s">
+        <v>167</v>
+      </c>
       <c r="H12" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I12" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="J12" s="15"/>
+      <c r="J12" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K12" s="15"/>
       <c r="L12" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M12" s="18" t="n">
         <f aca="false">IF(H12="not applicable",IF(K12&lt;&gt;"",1,0),IF(I12="yes",IF(H12="verified",1,0),IF(OR(H12="tested",H12="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>6</v>
+        <v>169</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>82</v>
+        <v>170</v>
       </c>
       <c r="E13" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="G13" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G13" s="15" t="s">
+        <v>167</v>
+      </c>
       <c r="H13" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I13" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="J13" s="15"/>
+      <c r="J13" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K13" s="15"/>
       <c r="L13" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M13" s="18" t="n">
         <f aca="false">IF(H13="not applicable",IF(K13&lt;&gt;"",1,0),IF(I13="yes",IF(H13="verified",1,0),IF(OR(H13="tested",H13="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>6</v>
+        <v>172</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="E14" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F14" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="G14" s="15"/>
+        <v>130</v>
+      </c>
+      <c r="G14" s="15" t="s">
+        <v>174</v>
+      </c>
       <c r="H14" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I14" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="J14" s="15"/>
+      <c r="J14" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K14" s="15"/>
       <c r="L14" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M14" s="18" t="n">
         <f aca="false">IF(H14="not applicable",IF(K14&lt;&gt;"",1,0),IF(I14="yes",IF(H14="verified",1,0),IF(OR(H14="tested",H14="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>6</v>
+        <v>176</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>89</v>
+        <v>177</v>
       </c>
       <c r="E15" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="G15" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G15" s="15" t="s">
+        <v>167</v>
+      </c>
       <c r="H15" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I15" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="J15" s="15"/>
+        <v>65</v>
+      </c>
+      <c r="J15" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K15" s="15"/>
       <c r="L15" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M15" s="18" t="n">
         <f aca="false">IF(H15="not applicable",IF(K15&lt;&gt;"",1,0),IF(I15="yes",IF(H15="verified",1,0),IF(OR(H15="tested",H15="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>6</v>
+        <v>179</v>
       </c>
       <c r="D16" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F16" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="G16" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="E16" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="F16" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="G16" s="15"/>
       <c r="H16" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I16" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="J16" s="15"/>
+        <v>65</v>
+      </c>
+      <c r="J16" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K16" s="15"/>
       <c r="L16" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M16" s="18" t="n">
         <f aca="false">IF(H16="not applicable",IF(K16&lt;&gt;"",1,0),IF(I16="yes",IF(H16="verified",1,0),IF(OR(H16="tested",H16="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>6</v>
+        <v>182</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>95</v>
+        <v>183</v>
       </c>
       <c r="E17" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="G17" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G17" s="15" t="s">
+        <v>184</v>
+      </c>
       <c r="H17" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I17" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="J17" s="15"/>
+        <v>65</v>
+      </c>
+      <c r="J17" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K17" s="15"/>
       <c r="L17" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M17" s="18" t="n">
         <f aca="false">IF(H17="not applicable",IF(K17&lt;&gt;"",1,0),IF(I17="yes",IF(H17="verified",1,0),IF(OR(H17="tested",H17="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="15" t="s">
-        <v>169</v>
+        <v>185</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>6</v>
+        <v>186</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>170</v>
+        <v>187</v>
       </c>
       <c r="E18" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F18" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="G18" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G18" s="15" t="s">
+        <v>167</v>
+      </c>
       <c r="H18" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I18" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="J18" s="15"/>
+        <v>65</v>
+      </c>
+      <c r="J18" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K18" s="15"/>
       <c r="L18" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M18" s="18" t="n">
         <f aca="false">IF(H18="not applicable",IF(K18&lt;&gt;"",1,0),IF(I18="yes",IF(H18="verified",1,0),IF(OR(H18="tested",H18="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>171</v>
+        <v>188</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>6</v>
+        <v>189</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>100</v>
+        <v>190</v>
       </c>
       <c r="E19" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="G19" s="15"/>
+        <v>130</v>
+      </c>
+      <c r="G19" s="15" t="s">
+        <v>174</v>
+      </c>
       <c r="H19" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I19" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="J19" s="15"/>
+      <c r="J19" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K19" s="15"/>
       <c r="L19" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M19" s="18" t="n">
         <f aca="false">IF(H19="not applicable",IF(K19&lt;&gt;"",1,0),IF(I19="yes",IF(H19="verified",1,0),IF(OR(H19="tested",H19="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
-        <v>172</v>
+        <v>191</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>6</v>
+        <v>165</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>173</v>
+        <v>192</v>
       </c>
       <c r="E20" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="G20" s="15"/>
+        <v>62</v>
+      </c>
+      <c r="G20" s="15" t="s">
+        <v>193</v>
+      </c>
       <c r="H20" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I20" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="J20" s="15"/>
+        <v>65</v>
+      </c>
+      <c r="J20" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K20" s="15"/>
       <c r="L20" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M20" s="18" t="n">
         <f aca="false">IF(H20="not applicable",IF(K20&lt;&gt;"",1,0),IF(I20="yes",IF(H20="verified",1,0),IF(OR(H20="tested",H20="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>195</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F21" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="G21" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="B21" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="C21" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="D21" s="15" t="s">
-        <v>104</v>
-      </c>
-      <c r="E21" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="F21" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="G21" s="15"/>
       <c r="H21" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I21" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="J21" s="15"/>
+        <v>72</v>
+      </c>
+      <c r="J21" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K21" s="15"/>
       <c r="L21" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M21" s="18" t="n">
         <f aca="false">IF(H21="not applicable",IF(K21&lt;&gt;"",1,0),IF(I21="yes",IF(H21="verified",1,0),IF(OR(H21="tested",H21="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>175</v>
+        <v>196</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>6</v>
+        <v>165</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>108</v>
+        <v>197</v>
       </c>
       <c r="E22" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F22" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="G22" s="15"/>
+        <v>90</v>
+      </c>
+      <c r="G22" s="15" t="s">
+        <v>174</v>
+      </c>
       <c r="H22" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I22" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="J22" s="15"/>
+        <v>72</v>
+      </c>
+      <c r="J22" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K22" s="15"/>
       <c r="L22" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M22" s="18" t="n">
         <f aca="false">IF(H22="not applicable",IF(K22&lt;&gt;"",1,0),IF(I22="yes",IF(H22="verified",1,0),IF(OR(H22="tested",H22="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="s">
-        <v>176</v>
+        <v>198</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>6</v>
+        <v>169</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>177</v>
+        <v>199</v>
       </c>
       <c r="E23" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="G23" s="15"/>
+        <v>90</v>
+      </c>
+      <c r="G23" s="15" t="s">
+        <v>184</v>
+      </c>
       <c r="H23" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I23" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="J23" s="15"/>
+        <v>72</v>
+      </c>
+      <c r="J23" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K23" s="15"/>
       <c r="L23" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M23" s="18" t="n">
         <f aca="false">IF(H23="not applicable",IF(K23&lt;&gt;"",1,0),IF(I23="yes",IF(H23="verified",1,0),IF(OR(H23="tested",H23="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>178</v>
+        <v>200</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>6</v>
+        <v>165</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>114</v>
+        <v>201</v>
       </c>
       <c r="E24" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F24" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="G24" s="15"/>
+        <v>130</v>
+      </c>
+      <c r="G24" s="15" t="s">
+        <v>174</v>
+      </c>
       <c r="H24" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I24" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="J24" s="15"/>
+        <v>72</v>
+      </c>
+      <c r="J24" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K24" s="15"/>
       <c r="L24" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M24" s="18" t="n">
         <f aca="false">IF(H24="not applicable",IF(K24&lt;&gt;"",1,0),IF(I24="yes",IF(H24="verified",1,0),IF(OR(H24="tested",H24="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>179</v>
+        <v>202</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>6</v>
+        <v>169</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>116</v>
+        <v>203</v>
       </c>
       <c r="E25" s="15" t="s">
         <v>61</v>
@@ -4032,344 +4307,666 @@
       <c r="F25" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="G25" s="15"/>
+      <c r="G25" s="15" t="s">
+        <v>98</v>
+      </c>
       <c r="H25" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I25" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="J25" s="15"/>
+        <v>72</v>
+      </c>
+      <c r="J25" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K25" s="15"/>
       <c r="L25" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M25" s="18" t="n">
         <f aca="false">IF(H25="not applicable",IF(K25&lt;&gt;"",1,0),IF(I25="yes",IF(H25="verified",1,0),IF(OR(H25="tested",H25="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>180</v>
+        <v>204</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>6</v>
+        <v>165</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>119</v>
+        <v>205</v>
       </c>
       <c r="E26" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F26" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="G26" s="15"/>
+        <v>130</v>
+      </c>
+      <c r="G26" s="15" t="s">
+        <v>174</v>
+      </c>
       <c r="H26" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I26" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="J26" s="15"/>
+      <c r="J26" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K26" s="15"/>
       <c r="L26" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M26" s="18" t="n">
         <f aca="false">IF(H26="not applicable",IF(K26&lt;&gt;"",1,0),IF(I26="yes",IF(H26="verified",1,0),IF(OR(H26="tested",H26="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="s">
-        <v>181</v>
+        <v>206</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>6</v>
+        <v>165</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>122</v>
+        <v>207</v>
       </c>
       <c r="E27" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F27" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="G27" s="15"/>
+        <v>130</v>
+      </c>
+      <c r="G27" s="15" t="s">
+        <v>174</v>
+      </c>
       <c r="H27" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I27" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="J27" s="15"/>
+        <v>72</v>
+      </c>
+      <c r="J27" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K27" s="15"/>
       <c r="L27" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M27" s="18" t="n">
         <f aca="false">IF(H27="not applicable",IF(K27&lt;&gt;"",1,0),IF(I27="yes",IF(H27="verified",1,0),IF(OR(H27="tested",H27="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="15" t="s">
-        <v>182</v>
+        <v>208</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="C28" s="15" t="s">
         <v>6</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>183</v>
+        <v>209</v>
       </c>
       <c r="E28" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F28" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="G28" s="15"/>
+        <v>90</v>
+      </c>
+      <c r="G28" s="15" t="s">
+        <v>184</v>
+      </c>
       <c r="H28" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I28" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="J28" s="15"/>
+      <c r="J28" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K28" s="15"/>
       <c r="L28" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M28" s="18" t="n">
         <f aca="false">IF(H28="not applicable",IF(K28&lt;&gt;"",1,0),IF(I28="yes",IF(H28="verified",1,0),IF(OR(H28="tested",H28="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
-        <v>184</v>
+        <v>210</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>128</v>
+        <v>107</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>6</v>
+        <v>165</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>129</v>
+        <v>211</v>
       </c>
       <c r="E29" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F29" s="15" t="s">
-        <v>130</v>
-      </c>
-      <c r="G29" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G29" s="15" t="s">
+        <v>167</v>
+      </c>
       <c r="H29" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I29" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="J29" s="15"/>
+      <c r="J29" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K29" s="15"/>
       <c r="L29" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M29" s="18" t="n">
         <f aca="false">IF(H29="not applicable",IF(K29&lt;&gt;"",1,0),IF(I29="yes",IF(H29="verified",1,0),IF(OR(H29="tested",H29="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="15" t="s">
-        <v>185</v>
+        <v>212</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>128</v>
+        <v>107</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>6</v>
+        <v>155</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>132</v>
+        <v>213</v>
       </c>
       <c r="E30" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F30" s="15" t="s">
-        <v>130</v>
-      </c>
-      <c r="G30" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G30" s="15" t="s">
+        <v>112</v>
+      </c>
       <c r="H30" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I30" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="J30" s="15"/>
+        <v>65</v>
+      </c>
+      <c r="J30" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K30" s="15"/>
       <c r="L30" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M30" s="18" t="n">
         <f aca="false">IF(H30="not applicable",IF(K30&lt;&gt;"",1,0),IF(I30="yes",IF(H30="verified",1,0),IF(OR(H30="tested",H30="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="15" t="s">
-        <v>186</v>
+        <v>214</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>134</v>
+        <v>107</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>6</v>
+        <v>169</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>135</v>
+        <v>215</v>
       </c>
       <c r="E31" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F31" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="G31" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G31" s="15" t="s">
+        <v>184</v>
+      </c>
       <c r="H31" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I31" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="J31" s="15"/>
+        <v>65</v>
+      </c>
+      <c r="J31" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K31" s="15"/>
       <c r="L31" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M31" s="18" t="n">
         <f aca="false">IF(H31="not applicable",IF(K31&lt;&gt;"",1,0),IF(I31="yes",IF(H31="verified",1,0),IF(OR(H31="tested",H31="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="15" t="s">
-        <v>187</v>
+        <v>216</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>134</v>
+        <v>107</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>6</v>
+        <v>169</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>139</v>
+        <v>217</v>
       </c>
       <c r="E32" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F32" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="G32" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G32" s="15" t="s">
+        <v>117</v>
+      </c>
       <c r="H32" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I32" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="J32" s="15"/>
+      <c r="J32" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K32" s="15"/>
       <c r="L32" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M32" s="18" t="n">
         <f aca="false">IF(H32="not applicable",IF(K32&lt;&gt;"",1,0),IF(I32="yes",IF(H32="verified",1,0),IF(OR(H32="tested",H32="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="15" t="s">
-        <v>188</v>
+        <v>218</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>142</v>
+        <v>107</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>6</v>
+        <v>169</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>143</v>
+        <v>219</v>
       </c>
       <c r="E33" s="15" t="s">
-        <v>144</v>
+        <v>61</v>
       </c>
       <c r="F33" s="15" t="s">
-        <v>144</v>
-      </c>
-      <c r="G33" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G33" s="15" t="s">
+        <v>120</v>
+      </c>
       <c r="H33" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I33" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="J33" s="15"/>
+      <c r="J33" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K33" s="15"/>
       <c r="L33" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M33" s="18" t="n">
         <f aca="false">IF(H33="not applicable",IF(K33&lt;&gt;"",1,0),IF(I33="yes",IF(H33="verified",1,0),IF(OR(H33="tested",H33="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="15" t="s">
-        <v>189</v>
+        <v>220</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>147</v>
+        <v>107</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>6</v>
+        <v>165</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>148</v>
+        <v>221</v>
       </c>
       <c r="E34" s="15" t="s">
-        <v>149</v>
+        <v>61</v>
       </c>
       <c r="F34" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="G34" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G34" s="15" t="s">
+        <v>222</v>
+      </c>
       <c r="H34" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I34" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="J34" s="15"/>
+        <v>65</v>
+      </c>
+      <c r="J34" s="17" t="n">
+        <v>46220</v>
+      </c>
       <c r="K34" s="15"/>
       <c r="L34" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M34" s="18" t="n">
         <f aca="false">IF(H34="not applicable",IF(K34&lt;&gt;"",1,0),IF(I34="yes",IF(H34="verified",1,0),IF(OR(H34="tested",H34="verified"),1,0)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="26.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="15" t="s">
+        <v>223</v>
+      </c>
+      <c r="B35" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>224</v>
+      </c>
+      <c r="E35" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F35" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="G35" s="15" t="s">
+        <v>225</v>
+      </c>
+      <c r="H35" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="I35" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="J35" s="17" t="n">
+        <v>46220</v>
+      </c>
+      <c r="K35" s="15"/>
+      <c r="L35" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M35" s="18" t="n">
+        <f aca="false">IF(H35="not applicable",IF(K35&lt;&gt;"",1,0),IF(I35="yes",IF(H35="verified",1,0),IF(OR(H35="tested",H35="verified"),1,0)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="15" t="s">
+        <v>226</v>
+      </c>
+      <c r="B36" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="C36" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="D36" s="15" t="s">
+        <v>227</v>
+      </c>
+      <c r="E36" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F36" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="G36" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="H36" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="I36" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="J36" s="17" t="n">
+        <v>46220</v>
+      </c>
+      <c r="K36" s="15"/>
+      <c r="L36" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M36" s="18" t="n">
+        <f aca="false">IF(H36="not applicable",IF(K36&lt;&gt;"",1,0),IF(I36="yes",IF(H36="verified",1,0),IF(OR(H36="tested",H36="verified"),1,0)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="26.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="C37" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="D37" s="15" t="s">
+        <v>229</v>
+      </c>
+      <c r="E37" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F37" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="G37" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="H37" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="I37" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="J37" s="17" t="n">
+        <v>46220</v>
+      </c>
+      <c r="K37" s="15"/>
+      <c r="L37" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M37" s="18" t="n">
+        <f aca="false">IF(H37="not applicable",IF(K37&lt;&gt;"",1,0),IF(I37="yes",IF(H37="verified",1,0),IF(OR(H37="tested",H37="verified"),1,0)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="26.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="15" t="s">
+        <v>230</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="D38" s="15" t="s">
+        <v>231</v>
+      </c>
+      <c r="E38" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F38" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G38" s="15" t="s">
+        <v>232</v>
+      </c>
+      <c r="H38" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="I38" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="J38" s="17" t="n">
+        <v>46220</v>
+      </c>
+      <c r="K38" s="15"/>
+      <c r="L38" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M38" s="18" t="n">
+        <f aca="false">IF(H38="not applicable",IF(K38&lt;&gt;"",1,0),IF(I38="yes",IF(H38="verified",1,0),IF(OR(H38="tested",H38="verified"),1,0)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="26.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="15" t="s">
+        <v>233</v>
+      </c>
+      <c r="B39" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="C39" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="D39" s="15" t="s">
+        <v>234</v>
+      </c>
+      <c r="E39" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F39" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G39" s="15" t="s">
+        <v>235</v>
+      </c>
+      <c r="H39" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="I39" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="J39" s="17" t="n">
+        <v>46220</v>
+      </c>
+      <c r="K39" s="15"/>
+      <c r="L39" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M39" s="18" t="n">
+        <f aca="false">IF(H39="not applicable",IF(K39&lt;&gt;"",1,0),IF(I39="yes",IF(H39="verified",1,0),IF(OR(H39="tested",H39="verified"),1,0)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="26.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="15" t="s">
+        <v>236</v>
+      </c>
+      <c r="B40" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="C40" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="D40" s="15" t="s">
+        <v>237</v>
+      </c>
+      <c r="E40" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="F40" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="G40" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="H40" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="I40" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="J40" s="17" t="n">
+        <v>46220</v>
+      </c>
+      <c r="K40" s="15"/>
+      <c r="L40" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M40" s="18" t="n">
+        <f aca="false">IF(H40="not applicable",IF(K40&lt;&gt;"",1,0),IF(I40="yes",IF(H40="verified",1,0),IF(OR(H40="tested",H40="verified"),1,0)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="26.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="15" t="s">
+        <v>238</v>
+      </c>
+      <c r="B41" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="C41" s="15" t="s">
+        <v>239</v>
+      </c>
+      <c r="D41" s="15" t="s">
+        <v>240</v>
+      </c>
+      <c r="E41" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="F41" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="G41" s="15" t="s">
+        <v>241</v>
+      </c>
+      <c r="H41" s="15" t="s">
+        <v>242</v>
+      </c>
+      <c r="I41" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="J41" s="17" t="n">
+        <v>46220</v>
+      </c>
+      <c r="K41" s="15" t="s">
+        <v>243</v>
+      </c>
+      <c r="L41" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M41" s="18" t="n">
+        <f aca="false">IF(H41="not applicable",IF(K41&lt;&gt;"",1,0),IF(I41="yes",IF(H41="verified",1,0),IF(OR(H41="tested",H41="verified"),1,0)))</f>
         <v>0</v>
       </c>
     </row>
@@ -4380,39 +4977,74 @@
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A6:M6"/>
   </mergeCells>
-  <conditionalFormatting sqref="H9:H34">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+  <conditionalFormatting sqref="H9:H41">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>$H9="not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>$H9="partial"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>$H9="implemented"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>$H9="tested"</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>$H9="verified"</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>$H9="blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$H9="not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H9:H34" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H9:H41" type="list">
       <formula1>_Lists!$A$1:$A$7</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I9:I34" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I9:I41" type="list">
       <formula1>_Lists!$B$1:$B$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="G9" r:id="rId1" display="../src/components/card/Card.tsx"/>
+    <hyperlink ref="G10" r:id="rId2" display="../../docs/card-component-brief.md"/>
+    <hyperlink ref="G11" r:id="rId3" display="../src/card.ts"/>
+    <hyperlink ref="G12" r:id="rId4" display="../test/components/card.test.tsx"/>
+    <hyperlink ref="G13" r:id="rId5" display="../test/components/card.test.tsx"/>
+    <hyperlink ref="G14" r:id="rId6" display="manual-tests/card.md"/>
+    <hyperlink ref="G15" r:id="rId7" display="../test/components/card.test.tsx"/>
+    <hyperlink ref="G16" r:id="rId8" display="../test/components/card.test.tsx"/>
+    <hyperlink ref="G17" r:id="rId9" display="tests/card.spec.ts"/>
+    <hyperlink ref="G18" r:id="rId10" display="../test/components/card.test.tsx"/>
+    <hyperlink ref="G19" r:id="rId11" display="manual-tests/card.md"/>
+    <hyperlink ref="G20" r:id="rId12" display="../src/components/card/card.css"/>
+    <hyperlink ref="G21" r:id="rId13" display="manual-tests/card.md"/>
+    <hyperlink ref="G22" r:id="rId14" display="manual-tests/card.md"/>
+    <hyperlink ref="G23" r:id="rId15" display="tests/card.spec.ts"/>
+    <hyperlink ref="G24" r:id="rId16" display="manual-tests/card.md"/>
+    <hyperlink ref="G25" r:id="rId17" display="tests/preferences.spec.ts"/>
+    <hyperlink ref="G26" r:id="rId18" display="manual-tests/card.md"/>
+    <hyperlink ref="G27" r:id="rId19" display="manual-tests/card.md"/>
+    <hyperlink ref="G28" r:id="rId20" display="tests/card.spec.ts"/>
+    <hyperlink ref="G29" r:id="rId21" display="../test/components/card.test.tsx"/>
+    <hyperlink ref="G30" r:id="rId22" display="../test/types/public-api.test.ts"/>
+    <hyperlink ref="G31" r:id="rId23" display="tests/card.spec.ts"/>
+    <hyperlink ref="G32" r:id="rId24" display="tests/foundation.spec.ts"/>
+    <hyperlink ref="G33" r:id="rId25" display="tests/visual.spec.ts"/>
+    <hyperlink ref="G34" r:id="rId26" display="../playwright.config.ts"/>
+    <hyperlink ref="G35" r:id="rId27" display="../test/package/ssr.test.mjs"/>
+    <hyperlink ref="G36" r:id="rId28" display="manual-tests/card.md"/>
+    <hyperlink ref="G37" r:id="rId29" display="manual-tests/card.md"/>
+    <hyperlink ref="G38" r:id="rId30" display="../docs/components/card/README.md"/>
+    <hyperlink ref="G39" r:id="rId31" display="../docs/components/card/CHANGELOG.md"/>
+    <hyperlink ref="G40" r:id="rId32" display="../../../../apps/brick-consumer/tests/consumer.spec.ts"/>
+    <hyperlink ref="G41" r:id="rId33" display="../../docs/core-dependency-ledger.md"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -4420,9 +5052,9 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId34"/>
   <tableParts>
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId35"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4452,7 +5084,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>190</v>
+        <v>244</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4469,7 +5101,7 @@
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>153</v>
+        <v>245</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -4588,7 +5220,7 @@
     </row>
     <row r="9" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>191</v>
+        <v>246</v>
       </c>
       <c r="B9" s="15" t="s">
         <v>59</v>
@@ -4597,7 +5229,7 @@
         <v>6</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>155</v>
+        <v>247</v>
       </c>
       <c r="E9" s="15" t="s">
         <v>61</v>
@@ -4624,7 +5256,7 @@
     </row>
     <row r="10" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>192</v>
+        <v>248</v>
       </c>
       <c r="B10" s="15" t="s">
         <v>67</v>
@@ -4633,7 +5265,7 @@
         <v>6</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>157</v>
+        <v>249</v>
       </c>
       <c r="E10" s="15" t="s">
         <v>61</v>
@@ -4660,7 +5292,7 @@
     </row>
     <row r="11" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>193</v>
+        <v>250</v>
       </c>
       <c r="B11" s="15" t="s">
         <v>59</v>
@@ -4669,7 +5301,7 @@
         <v>6</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>159</v>
+        <v>251</v>
       </c>
       <c r="E11" s="15" t="s">
         <v>61</v>
@@ -4696,7 +5328,7 @@
     </row>
     <row r="12" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>194</v>
+        <v>252</v>
       </c>
       <c r="B12" s="15" t="s">
         <v>59</v>
@@ -4705,7 +5337,7 @@
         <v>6</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>161</v>
+        <v>253</v>
       </c>
       <c r="E12" s="15" t="s">
         <v>61</v>
@@ -4732,7 +5364,7 @@
     </row>
     <row r="13" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>195</v>
+        <v>254</v>
       </c>
       <c r="B13" s="15" t="s">
         <v>81</v>
@@ -4768,7 +5400,7 @@
     </row>
     <row r="14" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>196</v>
+        <v>255</v>
       </c>
       <c r="B14" s="15" t="s">
         <v>81</v>
@@ -4777,7 +5409,7 @@
         <v>6</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>164</v>
+        <v>256</v>
       </c>
       <c r="E14" s="15" t="s">
         <v>61</v>
@@ -4804,7 +5436,7 @@
     </row>
     <row r="15" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>197</v>
+        <v>257</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>88</v>
@@ -4840,7 +5472,7 @@
     </row>
     <row r="16" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
-        <v>198</v>
+        <v>258</v>
       </c>
       <c r="B16" s="15" t="s">
         <v>88</v>
@@ -4849,7 +5481,7 @@
         <v>6</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>167</v>
+        <v>259</v>
       </c>
       <c r="E16" s="15" t="s">
         <v>61</v>
@@ -4876,7 +5508,7 @@
     </row>
     <row r="17" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>199</v>
+        <v>260</v>
       </c>
       <c r="B17" s="15" t="s">
         <v>88</v>
@@ -4912,7 +5544,7 @@
     </row>
     <row r="18" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="15" t="s">
-        <v>200</v>
+        <v>261</v>
       </c>
       <c r="B18" s="15" t="s">
         <v>88</v>
@@ -4921,7 +5553,7 @@
         <v>6</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>170</v>
+        <v>262</v>
       </c>
       <c r="E18" s="15" t="s">
         <v>61</v>
@@ -4948,7 +5580,7 @@
     </row>
     <row r="19" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>201</v>
+        <v>263</v>
       </c>
       <c r="B19" s="15" t="s">
         <v>88</v>
@@ -4984,7 +5616,7 @@
     </row>
     <row r="20" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
-        <v>202</v>
+        <v>264</v>
       </c>
       <c r="B20" s="15" t="s">
         <v>88</v>
@@ -4993,7 +5625,7 @@
         <v>6</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>173</v>
+        <v>265</v>
       </c>
       <c r="E20" s="15" t="s">
         <v>61</v>
@@ -5020,7 +5652,7 @@
     </row>
     <row r="21" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
-        <v>203</v>
+        <v>266</v>
       </c>
       <c r="B21" s="15" t="s">
         <v>88</v>
@@ -5056,7 +5688,7 @@
     </row>
     <row r="22" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>204</v>
+        <v>267</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>107</v>
@@ -5092,7 +5724,7 @@
     </row>
     <row r="23" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="s">
-        <v>205</v>
+        <v>268</v>
       </c>
       <c r="B23" s="15" t="s">
         <v>107</v>
@@ -5101,7 +5733,7 @@
         <v>6</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>177</v>
+        <v>269</v>
       </c>
       <c r="E23" s="15" t="s">
         <v>61</v>
@@ -5128,7 +5760,7 @@
     </row>
     <row r="24" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>206</v>
+        <v>270</v>
       </c>
       <c r="B24" s="15" t="s">
         <v>107</v>
@@ -5164,7 +5796,7 @@
     </row>
     <row r="25" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>207</v>
+        <v>271</v>
       </c>
       <c r="B25" s="15" t="s">
         <v>107</v>
@@ -5200,7 +5832,7 @@
     </row>
     <row r="26" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>208</v>
+        <v>272</v>
       </c>
       <c r="B26" s="15" t="s">
         <v>107</v>
@@ -5236,7 +5868,7 @@
     </row>
     <row r="27" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="s">
-        <v>209</v>
+        <v>273</v>
       </c>
       <c r="B27" s="15" t="s">
         <v>107</v>
@@ -5272,7 +5904,7 @@
     </row>
     <row r="28" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="15" t="s">
-        <v>210</v>
+        <v>274</v>
       </c>
       <c r="B28" s="15" t="s">
         <v>107</v>
@@ -5281,7 +5913,7 @@
         <v>6</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>183</v>
+        <v>275</v>
       </c>
       <c r="E28" s="15" t="s">
         <v>61</v>
@@ -5308,7 +5940,7 @@
     </row>
     <row r="29" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
-        <v>211</v>
+        <v>276</v>
       </c>
       <c r="B29" s="15" t="s">
         <v>128</v>
@@ -5344,7 +5976,7 @@
     </row>
     <row r="30" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="15" t="s">
-        <v>212</v>
+        <v>277</v>
       </c>
       <c r="B30" s="15" t="s">
         <v>128</v>
@@ -5380,7 +6012,7 @@
     </row>
     <row r="31" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="15" t="s">
-        <v>213</v>
+        <v>278</v>
       </c>
       <c r="B31" s="15" t="s">
         <v>134</v>
@@ -5416,7 +6048,7 @@
     </row>
     <row r="32" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="15" t="s">
-        <v>214</v>
+        <v>279</v>
       </c>
       <c r="B32" s="15" t="s">
         <v>134</v>
@@ -5452,7 +6084,7 @@
     </row>
     <row r="33" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="15" t="s">
-        <v>215</v>
+        <v>280</v>
       </c>
       <c r="B33" s="15" t="s">
         <v>142</v>
@@ -5488,7 +6120,7 @@
     </row>
     <row r="34" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="15" t="s">
-        <v>216</v>
+        <v>281</v>
       </c>
       <c r="B34" s="15" t="s">
         <v>147</v>
@@ -5530,25 +6162,25 @@
     <mergeCell ref="A6:M6"/>
   </mergeCells>
   <conditionalFormatting sqref="H9:H34">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>$H9="not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>$H9="partial"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>$H9="implemented"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>$H9="tested"</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>$H9="verified"</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>$H9="blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$H9="not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5594,7 +6226,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>217</v>
+        <v>282</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>65</v>
@@ -5602,7 +6234,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>218</v>
+        <v>283</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5617,12 +6249,12 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>219</v>
+        <v>242</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>220</v>
+        <v>284</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(brick): add Dialog and consumer flow
</commit_message>
<xml_diff>
--- a/playground/component-coverage.xlsx
+++ b/playground/component-coverage.xlsx
@@ -22,9 +22,9 @@
     <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Card!$A$1:$M$41</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Titles" vbProcedure="false">Card!$1:$8</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Card!$A$8:$M$34</definedName>
-    <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Area" vbProcedure="false">Dialog!$A$1:$M$34</definedName>
+    <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Area" vbProcedure="false">Dialog!$A$1:$M$45</definedName>
     <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Titles" vbProcedure="false">Dialog!$1:$8</definedName>
-    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">Dialog!$A$8:$M$34</definedName>
+    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">Dialog!$A$8:$M$45</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Index!$A$1:$N$10</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">Instructions!$A$1:$B$18</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Instructions!$A$4:$B$18</definedName>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="869" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="995" uniqueCount="338">
   <si>
     <t xml:space="preserve">Brick Component Coverage Index</t>
   </si>
@@ -776,115 +776,274 @@
     <t xml:space="preserve">Dialog Evidence Matrix</t>
   </si>
   <si>
-    <t xml:space="preserve">Common requirements from Brick's adopted quality contract. Add approved anatomy and component-specific rows after the component brief lands.</t>
+    <t xml:space="preserve">Evidence gates for the adopted modal Dialog compound, its twelve public parts, package proof, consumer cutover, and dependency-blocked legacy retirement.</t>
   </si>
   <si>
     <t xml:space="preserve">DIA-01</t>
   </si>
   <si>
-    <t xml:space="preserve">Implementation uses public Atom behavior without Core or local headless wrappers</t>
+    <t xml:space="preserve">Implementation directly composes public Atom 0.3.2 behavior without Core or local headless wrappers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../src/components/dialog/Dialog.tsx</t>
   </si>
   <si>
     <t xml:space="preserve">DIA-02</t>
   </si>
   <si>
-    <t xml:space="preserve">Atom capability audit covers mobile behavior and every Atom-owned gap is resolved through a released dependency</t>
+    <t xml:space="preserve">Adopted capability audit covers focus, nested layers, portals, isolation, scrolling, touch focus, presence, and dismissal; released Atom gaps are resolved</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../../docs/dialog-component-brief.md</t>
   </si>
   <si>
     <t xml:space="preserve">DIA-03</t>
   </si>
   <si>
-    <t xml:space="preserve">Public export and declaration surface match the approved brief</t>
+    <t xml:space="preserve">Root and dialog-subpath namespaces, direct part exports, declarations, and closed prop unions match the adopted brief</t>
   </si>
   <si>
     <t xml:space="preserve">DIA-04</t>
   </si>
   <si>
-    <t xml:space="preserve">Native props, refs, composition, and public slots follow the adopted API contract</t>
+    <t xml:space="preserve">Controlled and uncontrolled state, modal policy, dismissal controls, and close-reason detail remain public Atom behavior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../test/components/dialog.test.tsx</t>
   </si>
   <si>
     <t xml:space="preserve">DIA-05</t>
   </si>
   <si>
+    <t xml:space="preserve">Trigger</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trigger preserves native props, ref, stable Brick hooks, and Atom asChild and render composition</t>
+  </si>
+  <si>
     <t xml:space="preserve">DIA-06</t>
   </si>
   <si>
-    <t xml:space="preserve">Default recipe and every approved visual option are implemented</t>
+    <t xml:space="preserve">Portal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portal preserves default body, inline disabled, and custom-container composition without copying behavior into Brick</t>
   </si>
   <si>
     <t xml:space="preserve">DIA-07</t>
   </si>
   <si>
+    <t xml:space="preserve">Overlay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Overlay remains a sibling of Content, exposes the semantic scrim, and preserves exact-target and disabled dismissal behavior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/dialog.spec.ts</t>
+  </si>
+  <si>
     <t xml:space="preserve">DIA-08</t>
   </si>
   <si>
-    <t xml:space="preserve">Every public recipe, size, and important state</t>
+    <t xml:space="preserve">Modal semantics, ARIA ownership, focus scope, native props, ref, stable hooks, and sm, md, and lg sizes follow the adopted contract</t>
   </si>
   <si>
     <t xml:space="preserve">DIA-09</t>
   </si>
   <si>
+    <t xml:space="preserve">Header renders one native visual region for title, description, and optional explicit controls without generated behavior</t>
+  </si>
+  <si>
     <t xml:space="preserve">DIA-10</t>
   </si>
   <si>
-    <t xml:space="preserve">Light, dark, and relevant preference modes</t>
+    <t xml:space="preserve">Visible accessible naming and h1 through h6 heading control preserve Atom ARIA relationships</t>
   </si>
   <si>
     <t xml:space="preserve">DIA-11</t>
   </si>
   <si>
+    <t xml:space="preserve">Optional paragraph content supplies the accessible description without inventing copy or empty relationships</t>
+  </si>
+  <si>
     <t xml:space="preserve">DIA-12</t>
   </si>
   <si>
-    <t xml:space="preserve">Token, className, style, slot, and documented part customization</t>
+    <t xml:space="preserve">Body</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bounded body scrolling keeps long content readable without moving Header, Footer, or the background page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">manual-tests/dialog.md</t>
   </si>
   <si>
     <t xml:space="preserve">DIA-13</t>
   </si>
   <si>
+    <t xml:space="preserve">Consumer-selected actions preserve source order, wrap logically, and remain reachable at narrow and keyboard-constrained heights</t>
+  </si>
+  <si>
     <t xml:space="preserve">DIA-14</t>
   </si>
   <si>
+    <t xml:space="preserve">Close</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Close preserves native props, ref, stable Brick hooks, Atom composition, and the closeClick reason</t>
+  </si>
+  <si>
     <t xml:space="preserve">DIA-15</t>
   </si>
   <si>
-    <t xml:space="preserve">Public type and declaration fixtures</t>
+    <t xml:space="preserve">Branch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branch remains the public registration boundary for owned third-party portals and adds only stable Brick styling hooks</t>
   </si>
   <si>
     <t xml:space="preserve">DIA-16</t>
   </si>
   <si>
+    <t xml:space="preserve">Compiled CSS uses public Brick classes, component tokens, layers, logical properties, semantic roles, and direction-neutral centering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../src/components/dialog/dialog.css</t>
+  </si>
+  <si>
     <t xml:space="preserve">DIA-17</t>
   </si>
   <si>
+    <t xml:space="preserve">The semantic overlay recipe, border, elevation, spacing, three sizes, and reduced-motion states remain distinct and coherent</t>
+  </si>
+  <si>
     <t xml:space="preserve">DIA-18</t>
   </si>
   <si>
+    <t xml:space="preserve">The nine-section deterministic workbench uses public Dialog anatomy and Brick Button composition</t>
+  </si>
+  <si>
     <t xml:space="preserve">DIA-19</t>
   </si>
   <si>
+    <t xml:space="preserve">Overview, sizes, anatomy, dismissal, nesting, scoped appearance, customization, long content, and RTL scenarios are represented</t>
+  </si>
+  <si>
     <t xml:space="preserve">DIA-20</t>
   </si>
   <si>
-    <t xml:space="preserve">SSR or server-safe consumer behavior where applicable</t>
+    <t xml:space="preserve">Mobile-first constrained and intentional wide layouts preserve viewport gaps, bounded height, body scrolling, and reachable actions</t>
   </si>
   <si>
     <t xml:space="preserve">DIA-21</t>
   </si>
   <si>
+    <t xml:space="preserve">Light, dark, scoped appearance, forced colors, and reduced motion retain hierarchy, boundaries, and focus visibility</t>
+  </si>
+  <si>
     <t xml:space="preserve">DIA-22</t>
   </si>
   <si>
+    <t xml:space="preserve">Long content, unbroken text, localization, 200 and 400 percent zoom, narrow widths, and RTL remain contained and readable</t>
+  </si>
+  <si>
     <t xml:space="preserve">DIA-23</t>
   </si>
   <si>
+    <t xml:space="preserve">Public Dialog tokens, stable classes, style, data attributes, and overridable part slots remain local and inspectable</t>
+  </si>
+  <si>
     <t xml:space="preserve">DIA-24</t>
   </si>
   <si>
+    <t xml:space="preserve">Stable Dialog route and deterministic selectors support repeatable browser and visual checks</t>
+  </si>
+  <si>
     <t xml:space="preserve">DIA-25</t>
   </si>
   <si>
+    <t xml:space="preserve">Vitest and Testing Library cover default DOM, native contracts, composition, sizes, ARIA, state, and namespace identity</t>
+  </si>
+  <si>
     <t xml:space="preserve">DIA-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Public types, declarations, invalid size and flat-call exclusions, root exports, and dialog-subpath fixtures pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Playwright verifies modal anatomy, focus containment and restoration, dismissal, nested cleanup, RTL, and mobile geometry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Axe reports no automatically detectable violations for the canonical open Dialog state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Four deterministic Chromium visual baselines covering light, dark, mobile RTL, and forced colors are reviewed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chromium, Firefox, WebKit, Pixel, and iPhone Dialog release matrix records 30 passing checks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numbered nine-step Dialog manual-test protocol is complete</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latest owner run passes after nested isolation, portalled RTL direction, and direction-neutral centering findings were corrected and retested</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Public Dialog documentation follows the standard template and covers anatomy, behavior, portals, scope, Branch, tokens, and customization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../docs/components/dialog/README.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dialog component changelog and package release notes record the initial contract and post-review corrections</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../docs/components/dialog/CHANGELOG.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Independent Brick Consumer uses Dialog through public package exports and passes production, interaction, layout, and axe gates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIA-37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legacy Dialog family</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legacy Core Dialog source, exports, defaults, compatibility, and stale evidence are removed only after dependents are resolved</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AlertDialog still imports shared Dialog defaults and legacy structures.</t>
   </si>
   <si>
     <t xml:space="preserve">partial</t>
@@ -1201,23 +1360,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFE2E8F0"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
           <fgColor rgb="FFFEE2E2"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF475569"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1327,6 +1470,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFE2E8F0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFEDE9FE"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
@@ -1336,6 +1487,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF166534"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF475569"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1493,8 +1652,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="DialogEvidence" displayName="DialogEvidence" ref="A8:M34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A8:M34"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="DialogEvidence" displayName="DialogEvidence" ref="A8:M45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A8:M45"/>
   <tableColumns count="13">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Area"/>
@@ -1774,14 +1933,14 @@
       </c>
       <c r="F4" s="5" t="n">
         <f aca="false">SUM(H8:H10)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>5</v>
       </c>
       <c r="H4" s="6" t="n">
         <f aca="false">IFERROR(SUMPRODUCT(B8:B10,J8:J10)/SUM(B8:B10),0)</f>
-        <v>0.670588235294118</v>
+        <v>0.96875</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1947,56 +2106,56 @@
         <v>21</v>
       </c>
       <c r="B10" s="8" t="n">
-        <f aca="false">COUNTA(Dialog!A9:A34)</f>
-        <v>26</v>
+        <f aca="false">COUNTA(Dialog!A9:A45)</f>
+        <v>37</v>
       </c>
       <c r="C10" s="8" t="n">
-        <f aca="false">COUNTIF(Dialog!H9:H34,"not started")</f>
-        <v>26</v>
+        <f aca="false">COUNTIF(Dialog!H9:H45,"not started")</f>
+        <v>0</v>
       </c>
       <c r="D10" s="8" t="n">
-        <f aca="false">COUNTIF(Dialog!H9:H34,"partial")</f>
+        <f aca="false">COUNTIF(Dialog!H9:H45,"partial")</f>
         <v>0</v>
       </c>
       <c r="E10" s="8" t="n">
-        <f aca="false">COUNTIF(Dialog!H9:H34,"implemented")</f>
+        <f aca="false">COUNTIF(Dialog!H9:H45,"implemented")</f>
         <v>0</v>
       </c>
       <c r="F10" s="8" t="n">
-        <f aca="false">COUNTIF(Dialog!H9:H34,"tested")</f>
+        <f aca="false">COUNTIF(Dialog!H9:H45,"tested")</f>
+        <v>22</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <f aca="false">COUNTIF(Dialog!H9:H45,"verified")</f>
+        <v>14</v>
+      </c>
+      <c r="H10" s="8" t="n">
+        <f aca="false">COUNTIF(Dialog!H9:H45,"blocked")</f>
+        <v>1</v>
+      </c>
+      <c r="I10" s="8" t="n">
+        <f aca="false">COUNTIF(Dialog!H9:H45,"not applicable")</f>
         <v>0</v>
       </c>
-      <c r="G10" s="8" t="n">
-        <f aca="false">COUNTIF(Dialog!H9:H34,"verified")</f>
-        <v>0</v>
-      </c>
-      <c r="H10" s="8" t="n">
-        <f aca="false">COUNTIF(Dialog!H9:H34,"blocked")</f>
-        <v>0</v>
-      </c>
-      <c r="I10" s="8" t="n">
-        <f aca="false">COUNTIF(Dialog!H9:H34,"not applicable")</f>
-        <v>0</v>
-      </c>
       <c r="J10" s="9" t="n">
-        <f aca="false">IFERROR(SUM(Dialog!M9:M34)/SUM(Dialog!L9:L34),0)</f>
-        <v>0</v>
+        <f aca="false">IFERROR(SUM(Dialog!M9:M45)/SUM(Dialog!L9:L45),0)</f>
+        <v>0.972972972972973</v>
       </c>
       <c r="K10" s="8" t="str">
-        <f aca="false">IF(COUNTIFS(Dialog!E9:E34,"package",Dialog!M9:M34,"&lt;1")=0,"complete","open")</f>
-        <v>open</v>
+        <f aca="false">IF(COUNTIFS(Dialog!E9:E45,"package",Dialog!M9:M45,"&lt;1")=0,"complete","open")</f>
+        <v>complete</v>
       </c>
       <c r="L10" s="8" t="str">
-        <f aca="false">IF(COUNTIFS(Dialog!E9:E34,"consumer",Dialog!M9:M34,"&lt;1")=0,"complete","open")</f>
-        <v>open</v>
+        <f aca="false">IF(COUNTIFS(Dialog!E9:E45,"consumer",Dialog!M9:M45,"&lt;1")=0,"complete","open")</f>
+        <v>complete</v>
       </c>
       <c r="M10" s="8" t="str">
-        <f aca="false">IF(COUNTIFS(Dialog!E9:E34,"retirement",Dialog!M9:M34,"&lt;1")=0,"complete","open")</f>
+        <f aca="false">IF(COUNTIFS(Dialog!E9:E45,"retirement",Dialog!M9:M45,"&lt;1")=0,"complete","open")</f>
         <v>open</v>
       </c>
       <c r="N10" s="8" t="str">
         <f aca="false">IF(H10&gt;0,"blocked",IF(AND(J10=1,K10="complete",L10="complete",M10="complete"),"complete",IF(J10=0,"not started","in progress")))</f>
-        <v>not started</v>
+        <v>blocked</v>
       </c>
     </row>
   </sheetData>
@@ -2005,25 +2164,25 @@
     <mergeCell ref="A2:N2"/>
   </mergeCells>
   <conditionalFormatting sqref="N8:N10">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>$N8="not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>$N8="partial"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>$N8="implemented"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>$N8="tested"</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>$N8="verified"</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>$N8="blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>$N8="not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3416,25 +3575,25 @@
     <mergeCell ref="A6:M6"/>
   </mergeCells>
   <conditionalFormatting sqref="H9:H34">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>$H9="not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>$H9="partial"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>$H9="implemented"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>$H9="tested"</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>$H9="verified"</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>$H9="blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>$H9="not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4688,7 +4847,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="26.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="15" t="s">
         <v>223</v>
       </c>
@@ -4728,7 +4887,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="15" t="s">
         <v>226</v>
       </c>
@@ -4768,7 +4927,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="26.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="15" t="s">
         <v>228</v>
       </c>
@@ -4808,7 +4967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="26.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="15" t="s">
         <v>230</v>
       </c>
@@ -4848,7 +5007,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="26.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="15" t="s">
         <v>233</v>
       </c>
@@ -4888,7 +5047,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="26.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="15" t="s">
         <v>236</v>
       </c>
@@ -4928,7 +5087,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="26.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="15" t="s">
         <v>238</v>
       </c>
@@ -4978,25 +5137,25 @@
     <mergeCell ref="A6:M6"/>
   </mergeCells>
   <conditionalFormatting sqref="H9:H41">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>$H9="not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>$H9="partial"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>$H9="implemented"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>$H9="tested"</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>$H9="verified"</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>$H9="blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>$H9="not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5064,7 +5223,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:M34"/>
+  <dimension ref="A1:M45"/>
   <sheetFormatPr defaultColWidth="8.8046875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
@@ -5121,42 +5280,42 @@
         <v>7</v>
       </c>
       <c r="B4" s="5" t="n">
-        <f aca="false">COUNTA(A9:A34)</f>
-        <v>26</v>
+        <f aca="false">COUNTA(A9:A45)</f>
+        <v>37</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>45</v>
       </c>
       <c r="D4" s="5" t="n">
-        <f aca="false">SUM(M9:M34)</f>
-        <v>0</v>
+        <f aca="false">SUM(M9:M45)</f>
+        <v>36</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F4" s="6" t="n">
-        <f aca="false">IFERROR(D4/SUM(L9:L34),0)</f>
-        <v>0</v>
+        <f aca="false">IFERROR(D4/SUM(L9:L45),0)</f>
+        <v>0.972972972972973</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>4</v>
       </c>
       <c r="H4" s="5" t="n">
-        <f aca="false">COUNTIF(H9:H34,"blocked")</f>
-        <v>0</v>
+        <f aca="false">COUNTIF(H9:H45,"blocked")</f>
+        <v>1</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>15</v>
       </c>
       <c r="J4" s="5" t="str">
-        <f aca="false">IF(COUNTIFS(E9:E34,"package",M9:M34,"&lt;1")=0,"complete","open")</f>
-        <v>open</v>
+        <f aca="false">IF(COUNTIFS(E9:E45,"package",M9:M45,"&lt;1")=0,"complete","open")</f>
+        <v>complete</v>
       </c>
       <c r="K4" s="4" t="s">
         <v>17</v>
       </c>
       <c r="L4" s="5" t="str">
-        <f aca="false">IF(COUNTIFS(E9:E34,"retirement",M9:M34,"&lt;1")=0,"complete","open")</f>
+        <f aca="false">IF(COUNTIFS(E9:E45,"retirement",M9:M45,"&lt;1")=0,"complete","open")</f>
         <v>open</v>
       </c>
     </row>
@@ -5218,7 +5377,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
         <v>246</v>
       </c>
@@ -5237,26 +5396,30 @@
       <c r="F9" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="G9" s="15"/>
+      <c r="G9" s="15" t="s">
+        <v>248</v>
+      </c>
       <c r="H9" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I9" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="J9" s="15"/>
+      <c r="J9" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K9" s="15"/>
       <c r="L9" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M9" s="18" t="n">
         <f aca="false">IF(H9="not applicable",IF(K9&lt;&gt;"",1,0),IF(I9="yes",IF(H9="verified",1,0),IF(OR(H9="tested",H9="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B10" s="15" t="s">
         <v>67</v>
@@ -5265,7 +5428,7 @@
         <v>6</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E10" s="15" t="s">
         <v>61</v>
@@ -5273,35 +5436,39 @@
       <c r="F10" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="G10" s="15"/>
+      <c r="G10" s="15" t="s">
+        <v>251</v>
+      </c>
       <c r="H10" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I10" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="J10" s="15"/>
+      <c r="J10" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K10" s="15"/>
       <c r="L10" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M10" s="18" t="n">
         <f aca="false">IF(H10="not applicable",IF(K10&lt;&gt;"",1,0),IF(I10="yes",IF(H10="verified",1,0),IF(OR(H10="tested",H10="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B11" s="15" t="s">
         <v>59</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>6</v>
+        <v>155</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="E11" s="15" t="s">
         <v>61</v>
@@ -5309,395 +5476,439 @@
       <c r="F11" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="G11" s="15"/>
+      <c r="G11" s="15" t="s">
+        <v>112</v>
+      </c>
       <c r="H11" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I11" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="J11" s="15"/>
+      <c r="J11" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K11" s="15"/>
       <c r="L11" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M11" s="18" t="n">
         <f aca="false">IF(H11="not applicable",IF(K11&lt;&gt;"",1,0),IF(I11="yes",IF(H11="verified",1,0),IF(OR(H11="tested",H11="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>6</v>
+        <v>169</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="E12" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="G12" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G12" s="15" t="s">
+        <v>256</v>
+      </c>
       <c r="H12" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I12" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="J12" s="15"/>
+      <c r="J12" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K12" s="15"/>
       <c r="L12" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M12" s="18" t="n">
         <f aca="false">IF(H12="not applicable",IF(K12&lt;&gt;"",1,0),IF(I12="yes",IF(H12="verified",1,0),IF(OR(H12="tested",H12="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>6</v>
+        <v>258</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>82</v>
+        <v>259</v>
       </c>
       <c r="E13" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="G13" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G13" s="15" t="s">
+        <v>256</v>
+      </c>
       <c r="H13" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I13" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="J13" s="15"/>
+      <c r="J13" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K13" s="15"/>
       <c r="L13" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M13" s="18" t="n">
         <f aca="false">IF(H13="not applicable",IF(K13&lt;&gt;"",1,0),IF(I13="yes",IF(H13="verified",1,0),IF(OR(H13="tested",H13="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>6</v>
+        <v>261</v>
       </c>
       <c r="D14" s="15" t="s">
+        <v>262</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="G14" s="15" t="s">
         <v>256</v>
       </c>
-      <c r="E14" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="F14" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="G14" s="15"/>
       <c r="H14" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I14" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="J14" s="15"/>
+        <v>65</v>
+      </c>
+      <c r="J14" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K14" s="15"/>
       <c r="L14" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M14" s="18" t="n">
         <f aca="false">IF(H14="not applicable",IF(K14&lt;&gt;"",1,0),IF(I14="yes",IF(H14="verified",1,0),IF(OR(H14="tested",H14="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>6</v>
+        <v>264</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>89</v>
+        <v>265</v>
       </c>
       <c r="E15" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="G15" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G15" s="15" t="s">
+        <v>266</v>
+      </c>
       <c r="H15" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I15" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="J15" s="15"/>
+        <v>65</v>
+      </c>
+      <c r="J15" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K15" s="15"/>
       <c r="L15" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M15" s="18" t="n">
         <f aca="false">IF(H15="not applicable",IF(K15&lt;&gt;"",1,0),IF(I15="yes",IF(H15="verified",1,0),IF(OR(H15="tested",H15="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>6</v>
+        <v>186</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
       <c r="E16" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F16" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="G16" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G16" s="15" t="s">
+        <v>256</v>
+      </c>
       <c r="H16" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I16" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="J16" s="15"/>
+        <v>65</v>
+      </c>
+      <c r="J16" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K16" s="15"/>
       <c r="L16" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M16" s="18" t="n">
         <f aca="false">IF(H16="not applicable",IF(K16&lt;&gt;"",1,0),IF(I16="yes",IF(H16="verified",1,0),IF(OR(H16="tested",H16="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>6</v>
+        <v>172</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>95</v>
+        <v>270</v>
       </c>
       <c r="E17" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="G17" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G17" s="15" t="s">
+        <v>256</v>
+      </c>
       <c r="H17" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I17" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="J17" s="15"/>
+        <v>65</v>
+      </c>
+      <c r="J17" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K17" s="15"/>
       <c r="L17" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M17" s="18" t="n">
         <f aca="false">IF(H17="not applicable",IF(K17&lt;&gt;"",1,0),IF(I17="yes",IF(H17="verified",1,0),IF(OR(H17="tested",H17="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="15" t="s">
-        <v>261</v>
+        <v>271</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>6</v>
+        <v>176</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>262</v>
+        <v>272</v>
       </c>
       <c r="E18" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F18" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="G18" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G18" s="15" t="s">
+        <v>256</v>
+      </c>
       <c r="H18" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I18" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="J18" s="15"/>
+        <v>65</v>
+      </c>
+      <c r="J18" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K18" s="15"/>
       <c r="L18" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M18" s="18" t="n">
         <f aca="false">IF(H18="not applicable",IF(K18&lt;&gt;"",1,0),IF(I18="yes",IF(H18="verified",1,0),IF(OR(H18="tested",H18="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>263</v>
+        <v>273</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>6</v>
+        <v>179</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>100</v>
+        <v>274</v>
       </c>
       <c r="E19" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="G19" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G19" s="15" t="s">
+        <v>256</v>
+      </c>
       <c r="H19" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I19" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="J19" s="15"/>
+        <v>65</v>
+      </c>
+      <c r="J19" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K19" s="15"/>
       <c r="L19" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M19" s="18" t="n">
         <f aca="false">IF(H19="not applicable",IF(K19&lt;&gt;"",1,0),IF(I19="yes",IF(H19="verified",1,0),IF(OR(H19="tested",H19="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
-        <v>264</v>
+        <v>275</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>6</v>
+        <v>276</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
       <c r="E20" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="G20" s="15"/>
+        <v>130</v>
+      </c>
+      <c r="G20" s="15" t="s">
+        <v>278</v>
+      </c>
       <c r="H20" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I20" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="J20" s="15"/>
+      <c r="J20" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K20" s="15"/>
       <c r="L20" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M20" s="18" t="n">
         <f aca="false">IF(H20="not applicable",IF(K20&lt;&gt;"",1,0),IF(I20="yes",IF(H20="verified",1,0),IF(OR(H20="tested",H20="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
-        <v>266</v>
+        <v>279</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>6</v>
+        <v>189</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>104</v>
+        <v>280</v>
       </c>
       <c r="E21" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="G21" s="15"/>
+        <v>130</v>
+      </c>
+      <c r="G21" s="15" t="s">
+        <v>278</v>
+      </c>
       <c r="H21" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I21" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="J21" s="15"/>
+        <v>72</v>
+      </c>
+      <c r="J21" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K21" s="15"/>
       <c r="L21" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M21" s="18" t="n">
         <f aca="false">IF(H21="not applicable",IF(K21&lt;&gt;"",1,0),IF(I21="yes",IF(H21="verified",1,0),IF(OR(H21="tested",H21="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>107</v>
+        <v>39</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>6</v>
+        <v>282</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>108</v>
+        <v>283</v>
       </c>
       <c r="E22" s="15" t="s">
         <v>61</v>
@@ -5705,35 +5916,39 @@
       <c r="F22" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="G22" s="15"/>
+      <c r="G22" s="15" t="s">
+        <v>256</v>
+      </c>
       <c r="H22" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I22" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="J22" s="15"/>
+      <c r="J22" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K22" s="15"/>
       <c r="L22" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M22" s="18" t="n">
         <f aca="false">IF(H22="not applicable",IF(K22&lt;&gt;"",1,0),IF(I22="yes",IF(H22="verified",1,0),IF(OR(H22="tested",H22="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="s">
-        <v>268</v>
+        <v>284</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>107</v>
+        <v>39</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>6</v>
+        <v>285</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>269</v>
+        <v>286</v>
       </c>
       <c r="E23" s="15" t="s">
         <v>61</v>
@@ -5741,251 +5956,279 @@
       <c r="F23" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="G23" s="15"/>
+      <c r="G23" s="15" t="s">
+        <v>256</v>
+      </c>
       <c r="H23" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I23" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="J23" s="15"/>
+      <c r="J23" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K23" s="15"/>
       <c r="L23" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M23" s="18" t="n">
         <f aca="false">IF(H23="not applicable",IF(K23&lt;&gt;"",1,0),IF(I23="yes",IF(H23="verified",1,0),IF(OR(H23="tested",H23="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>270</v>
+        <v>287</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>107</v>
+        <v>81</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>6</v>
+        <v>165</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>114</v>
+        <v>288</v>
       </c>
       <c r="E24" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F24" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="G24" s="15"/>
+        <v>62</v>
+      </c>
+      <c r="G24" s="15" t="s">
+        <v>289</v>
+      </c>
       <c r="H24" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I24" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="J24" s="15"/>
+      <c r="J24" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K24" s="15"/>
       <c r="L24" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M24" s="18" t="n">
         <f aca="false">IF(H24="not applicable",IF(K24&lt;&gt;"",1,0),IF(I24="yes",IF(H24="verified",1,0),IF(OR(H24="tested",H24="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>271</v>
+        <v>290</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>107</v>
+        <v>81</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>6</v>
+        <v>186</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>116</v>
+        <v>291</v>
       </c>
       <c r="E25" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="G25" s="15"/>
+        <v>130</v>
+      </c>
+      <c r="G25" s="15" t="s">
+        <v>278</v>
+      </c>
       <c r="H25" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I25" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="J25" s="15"/>
+        <v>72</v>
+      </c>
+      <c r="J25" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K25" s="15"/>
       <c r="L25" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M25" s="18" t="n">
         <f aca="false">IF(H25="not applicable",IF(K25&lt;&gt;"",1,0),IF(I25="yes",IF(H25="verified",1,0),IF(OR(H25="tested",H25="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>272</v>
+        <v>292</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>6</v>
+        <v>165</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>119</v>
+        <v>293</v>
       </c>
       <c r="E26" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F26" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="G26" s="15"/>
+        <v>90</v>
+      </c>
+      <c r="G26" s="15" t="s">
+        <v>278</v>
+      </c>
       <c r="H26" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I26" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="J26" s="15"/>
+      <c r="J26" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K26" s="15"/>
       <c r="L26" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M26" s="18" t="n">
         <f aca="false">IF(H26="not applicable",IF(K26&lt;&gt;"",1,0),IF(I26="yes",IF(H26="verified",1,0),IF(OR(H26="tested",H26="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="s">
-        <v>273</v>
+        <v>294</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="C27" s="15" t="s">
         <v>6</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>122</v>
+        <v>295</v>
       </c>
       <c r="E27" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F27" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="G27" s="15"/>
+        <v>90</v>
+      </c>
+      <c r="G27" s="15" t="s">
+        <v>266</v>
+      </c>
       <c r="H27" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I27" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="J27" s="15"/>
+        <v>72</v>
+      </c>
+      <c r="J27" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K27" s="15"/>
       <c r="L27" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M27" s="18" t="n">
         <f aca="false">IF(H27="not applicable",IF(K27&lt;&gt;"",1,0),IF(I27="yes",IF(H27="verified",1,0),IF(OR(H27="tested",H27="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="15" t="s">
-        <v>274</v>
+        <v>296</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>6</v>
+        <v>186</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>275</v>
+        <v>297</v>
       </c>
       <c r="E28" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F28" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="G28" s="15"/>
+        <v>130</v>
+      </c>
+      <c r="G28" s="15" t="s">
+        <v>278</v>
+      </c>
       <c r="H28" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I28" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="J28" s="15"/>
+        <v>72</v>
+      </c>
+      <c r="J28" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K28" s="15"/>
       <c r="L28" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M28" s="18" t="n">
         <f aca="false">IF(H28="not applicable",IF(K28&lt;&gt;"",1,0),IF(I28="yes",IF(H28="verified",1,0),IF(OR(H28="tested",H28="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
-        <v>276</v>
+        <v>298</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>6</v>
+        <v>165</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>129</v>
+        <v>299</v>
       </c>
       <c r="E29" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F29" s="15" t="s">
-        <v>130</v>
-      </c>
-      <c r="G29" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G29" s="15" t="s">
+        <v>120</v>
+      </c>
       <c r="H29" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I29" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="J29" s="15"/>
+        <v>72</v>
+      </c>
+      <c r="J29" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K29" s="15"/>
       <c r="L29" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M29" s="18" t="n">
         <f aca="false">IF(H29="not applicable",IF(K29&lt;&gt;"",1,0),IF(I29="yes",IF(H29="verified",1,0),IF(OR(H29="tested",H29="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="15" t="s">
-        <v>277</v>
+        <v>300</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>6</v>
+        <v>165</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>132</v>
+        <v>301</v>
       </c>
       <c r="E30" s="15" t="s">
         <v>61</v>
@@ -5993,203 +6236,665 @@
       <c r="F30" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="G30" s="15"/>
+      <c r="G30" s="15" t="s">
+        <v>278</v>
+      </c>
       <c r="H30" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I30" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="J30" s="15"/>
+      <c r="J30" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K30" s="15"/>
       <c r="L30" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M30" s="18" t="n">
         <f aca="false">IF(H30="not applicable",IF(K30&lt;&gt;"",1,0),IF(I30="yes",IF(H30="verified",1,0),IF(OR(H30="tested",H30="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="15" t="s">
+        <v>302</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>303</v>
+      </c>
+      <c r="E31" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F31" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="G31" s="15" t="s">
         <v>278</v>
       </c>
-      <c r="B31" s="15" t="s">
-        <v>134</v>
-      </c>
-      <c r="C31" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="D31" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="E31" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="F31" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="G31" s="15"/>
       <c r="H31" s="15" t="s">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="I31" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="J31" s="15"/>
+      <c r="J31" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K31" s="15"/>
       <c r="L31" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M31" s="18" t="n">
         <f aca="false">IF(H31="not applicable",IF(K31&lt;&gt;"",1,0),IF(I31="yes",IF(H31="verified",1,0),IF(OR(H31="tested",H31="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="15" t="s">
-        <v>279</v>
+        <v>304</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>134</v>
+        <v>88</v>
       </c>
       <c r="C32" s="15" t="s">
         <v>6</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>139</v>
+        <v>305</v>
       </c>
       <c r="E32" s="15" t="s">
         <v>61</v>
       </c>
       <c r="F32" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="G32" s="15"/>
+        <v>90</v>
+      </c>
+      <c r="G32" s="15" t="s">
+        <v>266</v>
+      </c>
       <c r="H32" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I32" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="J32" s="15"/>
+      <c r="J32" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K32" s="15"/>
       <c r="L32" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M32" s="18" t="n">
         <f aca="false">IF(H32="not applicable",IF(K32&lt;&gt;"",1,0),IF(I32="yes",IF(H32="verified",1,0),IF(OR(H32="tested",H32="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="15" t="s">
-        <v>280</v>
+        <v>306</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>142</v>
+        <v>107</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>6</v>
+        <v>165</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>143</v>
+        <v>307</v>
       </c>
       <c r="E33" s="15" t="s">
-        <v>144</v>
+        <v>61</v>
       </c>
       <c r="F33" s="15" t="s">
-        <v>144</v>
-      </c>
-      <c r="G33" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G33" s="15" t="s">
+        <v>256</v>
+      </c>
       <c r="H33" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I33" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="J33" s="15"/>
+        <v>65</v>
+      </c>
+      <c r="J33" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K33" s="15"/>
       <c r="L33" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M33" s="18" t="n">
         <f aca="false">IF(H33="not applicable",IF(K33&lt;&gt;"",1,0),IF(I33="yes",IF(H33="verified",1,0),IF(OR(H33="tested",H33="verified"),1,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="15" t="s">
-        <v>281</v>
+        <v>308</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>147</v>
+        <v>107</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>6</v>
+        <v>155</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>148</v>
+        <v>309</v>
       </c>
       <c r="E34" s="15" t="s">
-        <v>149</v>
+        <v>61</v>
       </c>
       <c r="F34" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="G34" s="15"/>
+        <v>109</v>
+      </c>
+      <c r="G34" s="15" t="s">
+        <v>112</v>
+      </c>
       <c r="H34" s="15" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="I34" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="J34" s="15"/>
+        <v>65</v>
+      </c>
+      <c r="J34" s="19" t="n">
+        <v>46220</v>
+      </c>
       <c r="K34" s="15"/>
       <c r="L34" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M34" s="18" t="n">
         <f aca="false">IF(H34="not applicable",IF(K34&lt;&gt;"",1,0),IF(I34="yes",IF(H34="verified",1,0),IF(OR(H34="tested",H34="verified"),1,0)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="15" t="s">
+        <v>310</v>
+      </c>
+      <c r="B35" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>311</v>
+      </c>
+      <c r="E35" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F35" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="G35" s="15" t="s">
+        <v>266</v>
+      </c>
+      <c r="H35" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="I35" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="J35" s="19" t="n">
+        <v>46220</v>
+      </c>
+      <c r="K35" s="15"/>
+      <c r="L35" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M35" s="18" t="n">
+        <f aca="false">IF(H35="not applicable",IF(K35&lt;&gt;"",1,0),IF(I35="yes",IF(H35="verified",1,0),IF(OR(H35="tested",H35="verified"),1,0)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="15" t="s">
+        <v>312</v>
+      </c>
+      <c r="B36" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="C36" s="15" t="s">
+        <v>186</v>
+      </c>
+      <c r="D36" s="15" t="s">
+        <v>313</v>
+      </c>
+      <c r="E36" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F36" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="G36" s="15" t="s">
+        <v>266</v>
+      </c>
+      <c r="H36" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="I36" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="J36" s="19" t="n">
+        <v>46220</v>
+      </c>
+      <c r="K36" s="15"/>
+      <c r="L36" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M36" s="18" t="n">
+        <f aca="false">IF(H36="not applicable",IF(K36&lt;&gt;"",1,0),IF(I36="yes",IF(H36="verified",1,0),IF(OR(H36="tested",H36="verified"),1,0)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="15" t="s">
+        <v>314</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="C37" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="D37" s="15" t="s">
+        <v>315</v>
+      </c>
+      <c r="E37" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F37" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="G37" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="H37" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="I37" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="J37" s="19" t="n">
+        <v>46220</v>
+      </c>
+      <c r="K37" s="15"/>
+      <c r="L37" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M37" s="18" t="n">
+        <f aca="false">IF(H37="not applicable",IF(K37&lt;&gt;"",1,0),IF(I37="yes",IF(H37="verified",1,0),IF(OR(H37="tested",H37="verified"),1,0)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="15" t="s">
+        <v>316</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="D38" s="15" t="s">
+        <v>317</v>
+      </c>
+      <c r="E38" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F38" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="G38" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="H38" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="I38" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="J38" s="19" t="n">
+        <v>46220</v>
+      </c>
+      <c r="K38" s="15"/>
+      <c r="L38" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M38" s="18" t="n">
+        <f aca="false">IF(H38="not applicable",IF(K38&lt;&gt;"",1,0),IF(I38="yes",IF(H38="verified",1,0),IF(OR(H38="tested",H38="verified"),1,0)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="15" t="s">
+        <v>318</v>
+      </c>
+      <c r="B39" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="C39" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="D39" s="15" t="s">
+        <v>224</v>
+      </c>
+      <c r="E39" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F39" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="G39" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="H39" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="I39" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="J39" s="19" t="n">
+        <v>46220</v>
+      </c>
+      <c r="K39" s="15"/>
+      <c r="L39" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M39" s="18" t="n">
+        <f aca="false">IF(H39="not applicable",IF(K39&lt;&gt;"",1,0),IF(I39="yes",IF(H39="verified",1,0),IF(OR(H39="tested",H39="verified"),1,0)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="15" t="s">
+        <v>319</v>
+      </c>
+      <c r="B40" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="C40" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="D40" s="15" t="s">
+        <v>320</v>
+      </c>
+      <c r="E40" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F40" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="G40" s="15" t="s">
+        <v>278</v>
+      </c>
+      <c r="H40" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="I40" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="J40" s="19" t="n">
+        <v>46220</v>
+      </c>
+      <c r="K40" s="15"/>
+      <c r="L40" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M40" s="18" t="n">
+        <f aca="false">IF(H40="not applicable",IF(K40&lt;&gt;"",1,0),IF(I40="yes",IF(H40="verified",1,0),IF(OR(H40="tested",H40="verified"),1,0)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="15" t="s">
+        <v>321</v>
+      </c>
+      <c r="B41" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="C41" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="D41" s="15" t="s">
+        <v>322</v>
+      </c>
+      <c r="E41" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F41" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="G41" s="15" t="s">
+        <v>278</v>
+      </c>
+      <c r="H41" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="I41" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="J41" s="19" t="n">
+        <v>46220</v>
+      </c>
+      <c r="K41" s="15"/>
+      <c r="L41" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M41" s="18" t="n">
+        <f aca="false">IF(H41="not applicable",IF(K41&lt;&gt;"",1,0),IF(I41="yes",IF(H41="verified",1,0),IF(OR(H41="tested",H41="verified"),1,0)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="15" t="s">
+        <v>323</v>
+      </c>
+      <c r="B42" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="C42" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="D42" s="15" t="s">
+        <v>324</v>
+      </c>
+      <c r="E42" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F42" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G42" s="15" t="s">
+        <v>325</v>
+      </c>
+      <c r="H42" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="I42" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="J42" s="19" t="n">
+        <v>46220</v>
+      </c>
+      <c r="K42" s="15"/>
+      <c r="L42" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M42" s="18" t="n">
+        <f aca="false">IF(H42="not applicable",IF(K42&lt;&gt;"",1,0),IF(I42="yes",IF(H42="verified",1,0),IF(OR(H42="tested",H42="verified"),1,0)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="15" t="s">
+        <v>326</v>
+      </c>
+      <c r="B43" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="C43" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="D43" s="15" t="s">
+        <v>327</v>
+      </c>
+      <c r="E43" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F43" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G43" s="15" t="s">
+        <v>328</v>
+      </c>
+      <c r="H43" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="I43" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="J43" s="19" t="n">
+        <v>46220</v>
+      </c>
+      <c r="K43" s="15"/>
+      <c r="L43" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M43" s="18" t="n">
+        <f aca="false">IF(H43="not applicable",IF(K43&lt;&gt;"",1,0),IF(I43="yes",IF(H43="verified",1,0),IF(OR(H43="tested",H43="verified"),1,0)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="15" t="s">
+        <v>329</v>
+      </c>
+      <c r="B44" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="C44" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="D44" s="15" t="s">
+        <v>330</v>
+      </c>
+      <c r="E44" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="F44" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="G44" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="H44" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="I44" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="J44" s="19" t="n">
+        <v>46220</v>
+      </c>
+      <c r="K44" s="15"/>
+      <c r="L44" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M44" s="18" t="n">
+        <f aca="false">IF(H44="not applicable",IF(K44&lt;&gt;"",1,0),IF(I44="yes",IF(H44="verified",1,0),IF(OR(H44="tested",H44="verified"),1,0)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="15" t="s">
+        <v>331</v>
+      </c>
+      <c r="B45" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="C45" s="15" t="s">
+        <v>332</v>
+      </c>
+      <c r="D45" s="15" t="s">
+        <v>333</v>
+      </c>
+      <c r="E45" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="F45" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="G45" s="15" t="s">
+        <v>241</v>
+      </c>
+      <c r="H45" s="15" t="s">
+        <v>242</v>
+      </c>
+      <c r="I45" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="J45" s="19" t="n">
+        <v>46220</v>
+      </c>
+      <c r="K45" s="15" t="s">
+        <v>334</v>
+      </c>
+      <c r="L45" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M45" s="18" t="n">
+        <f aca="false">IF(H45="not applicable",IF(K45&lt;&gt;"",1,0),IF(I45="yes",IF(H45="verified",1,0),IF(OR(H45="tested",H45="verified"),1,0)))</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A8:M34"/>
+  <autoFilter ref="A8:M45"/>
   <mergeCells count="3">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A6:M6"/>
   </mergeCells>
-  <conditionalFormatting sqref="H9:H34">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+  <conditionalFormatting sqref="H9:H45">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>$H9="not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>$H9="partial"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>$H9="implemented"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>$H9="tested"</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>$H9="verified"</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>$H9="blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>$H9="not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H9:H34" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H9:H45" type="list">
       <formula1>_Lists!$A$1:$A$7</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I9:I34" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I9:I45" type="list">
       <formula1>_Lists!$B$1:$B$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -6226,7 +6931,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>282</v>
+        <v>335</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>65</v>
@@ -6234,7 +6939,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>283</v>
+        <v>336</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6254,7 +6959,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>284</v>
+        <v>337</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Complete Brick reference quality review
</commit_message>
<xml_diff>
--- a/playground/component-coverage.xlsx
+++ b/playground/component-coverage.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="995" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="995" uniqueCount="339">
   <si>
     <t xml:space="preserve">Brick Component Coverage Index</t>
   </si>
@@ -149,7 +149,7 @@
     <t xml:space="preserve">Human-review rows resolve only at verified. Other rows resolve at tested or verified. A documented not-applicable row also resolves.</t>
   </si>
   <si>
-    <t xml:space="preserve">Implementation, playground, automated tests, manual evidence, and documentation are complete.</t>
+    <t xml:space="preserve">Implementation, playground, automated tests, manual evidence, and documentation are complete; every tested or verified claim has been sampled against its exact assertion.</t>
   </si>
   <si>
     <t xml:space="preserve">A live consumer uses the finished Brick component and the cutover is verified.</t>
@@ -167,7 +167,7 @@
     <t xml:space="preserve">Editing</t>
   </si>
   <si>
-    <t xml:space="preserve">Use list values, keep evidence links short, record blocker and not-applicable reasons, recalculate, and visually inspect every changed sheet.</t>
+    <t xml:space="preserve">Use list values; classify Atom, Brick adapter, browser, and manual ownership; keep claims assertion-specific; record blocker and not-applicable reasons; recalculate; and visually inspect every changed sheet.</t>
   </si>
   <si>
     <t xml:space="preserve">Button Evidence Matrix</t>
@@ -806,7 +806,7 @@
     <t xml:space="preserve">DIA-04</t>
   </si>
   <si>
-    <t xml:space="preserve">Controlled and uncontrolled state, modal policy, dismissal controls, and close-reason detail remain public Atom behavior</t>
+    <t xml:space="preserve">Atom owns exhaustive controlled and uncontrolled state and modal policy; Brick verifies disabled Root forwarding and representative close-reason preservation</t>
   </si>
   <si>
     <t xml:space="preserve">../test/components/dialog.test.tsx</t>
@@ -818,7 +818,7 @@
     <t xml:space="preserve">Trigger</t>
   </si>
   <si>
-    <t xml:space="preserve">Trigger preserves native props, ref, stable Brick hooks, and Atom asChild and render composition</t>
+    <t xml:space="preserve">Trigger preserves disabled state, native props, ref, stable Brick hooks, and representative Atom asChild and render composition</t>
   </si>
   <si>
     <t xml:space="preserve">DIA-06</t>
@@ -830,6 +830,9 @@
     <t xml:space="preserve">Portal preserves default body, inline disabled, and custom-container composition without copying behavior into Brick</t>
   </si>
   <si>
+    <t xml:space="preserve">../test/components/dialog.test.tsx + tests/dialog.spec.ts</t>
+  </si>
+  <si>
     <t xml:space="preserve">DIA-07</t>
   </si>
   <si>
@@ -857,7 +860,7 @@
     <t xml:space="preserve">DIA-10</t>
   </si>
   <si>
-    <t xml:space="preserve">Visible accessible naming and h1 through h6 heading control preserve Atom ARIA relationships</t>
+    <t xml:space="preserve">Visible accessible naming, the default h2, and a representative h1 override preserve Atom ARIA relationships and heading forwarding</t>
   </si>
   <si>
     <t xml:space="preserve">DIA-11</t>
@@ -890,7 +893,7 @@
     <t xml:space="preserve">Close</t>
   </si>
   <si>
-    <t xml:space="preserve">Close preserves native props, ref, stable Brick hooks, Atom composition, and the closeClick reason</t>
+    <t xml:space="preserve">Close preserves native props, ref, stable Brick hooks, representative asChild and render composition, and the closeClick reason</t>
   </si>
   <si>
     <t xml:space="preserve">DIA-15</t>
@@ -899,7 +902,7 @@
     <t xml:space="preserve">Branch</t>
   </si>
   <si>
-    <t xml:space="preserve">Branch remains the public registration boundary for owned third-party portals and adds only stable Brick styling hooks</t>
+    <t xml:space="preserve">Branch preserves Atom registration ownership while Brick verifies render composition, native forwarding, ref wiring, and stable styling hooks</t>
   </si>
   <si>
     <t xml:space="preserve">DIA-16</t>
@@ -962,7 +965,7 @@
     <t xml:space="preserve">DIA-25</t>
   </si>
   <si>
-    <t xml:space="preserve">Vitest and Testing Library cover default DOM, native contracts, composition, sizes, ARIA, state, and namespace identity</t>
+    <t xml:space="preserve">Vitest and Testing Library cover default DOM, native contracts, disabled Root, asChild and render composition, portal container, heading override, sizes, ARIA, close reason, and namespace identity</t>
   </si>
   <si>
     <t xml:space="preserve">DIA-26</t>
@@ -974,7 +977,7 @@
     <t xml:space="preserve">DIA-27</t>
   </si>
   <si>
-    <t xml:space="preserve">Playwright verifies modal anatomy, focus containment and restoration, dismissal, nested cleanup, RTL, and mobile geometry</t>
+    <t xml:space="preserve">Playwright verifies modal anatomy, focus containment and restoration, dismissal, disabled Trigger and Overlay paths, nested cleanup, RTL, and mobile geometry</t>
   </si>
   <si>
     <t xml:space="preserve">DIA-28</t>
@@ -992,7 +995,7 @@
     <t xml:space="preserve">DIA-30</t>
   </si>
   <si>
-    <t xml:space="preserve">Chromium, Firefox, WebKit, Pixel, and iPhone Dialog release matrix records 30 passing checks</t>
+    <t xml:space="preserve">Chromium, Firefox, WebKit, Pixel, and iPhone Dialog release matrix records 40 passing Dialog checks</t>
   </si>
   <si>
     <t xml:space="preserve">DIA-31</t>
@@ -1013,7 +1016,7 @@
     <t xml:space="preserve">DIA-34</t>
   </si>
   <si>
-    <t xml:space="preserve">Public Dialog documentation follows the standard template and covers anatomy, behavior, portals, scope, Branch, tokens, and customization</t>
+    <t xml:space="preserve">Public Dialog documentation follows the standard template and covers use boundaries, anatomy, API, states, accessibility, responsive behavior, portals, Branch, tokens, composition, and customization</t>
   </si>
   <si>
     <t xml:space="preserve">../docs/components/dialog/README.md</t>
@@ -1022,7 +1025,7 @@
     <t xml:space="preserve">DIA-35</t>
   </si>
   <si>
-    <t xml:space="preserve">Dialog component changelog and package release notes record the initial contract and post-review corrections</t>
+    <t xml:space="preserve">Dialog component changelog records the initial contract and post-review evidence corrections</t>
   </si>
   <si>
     <t xml:space="preserve">../docs/components/dialog/CHANGELOG.md</t>
@@ -1605,6 +1608,7 @@
     <tableColumn id="12" name="Weight"/>
     <tableColumn id="13" name="Resolved"/>
   </tableColumns>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1626,6 +1630,7 @@
     <tableColumn id="12" name="Weight"/>
     <tableColumn id="13" name="Resolved"/>
   </tableColumns>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1648,6 +1653,7 @@
     <tableColumn id="13" name="Retirement gate"/>
     <tableColumn id="14" name="Status"/>
   </tableColumns>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1669,6 +1675,7 @@
     <tableColumn id="12" name="Weight"/>
     <tableColumn id="13" name="Resolved"/>
   </tableColumns>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1679,6 +1686,7 @@
     <tableColumn id="1" name="Topic"/>
     <tableColumn id="2" name="Rule"/>
   </tableColumns>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -5526,7 +5534,7 @@
         <v>65</v>
       </c>
       <c r="J12" s="19" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="K12" s="15"/>
       <c r="L12" s="18" t="n">
@@ -5566,7 +5574,7 @@
         <v>65</v>
       </c>
       <c r="J13" s="19" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="K13" s="15"/>
       <c r="L13" s="18" t="n">
@@ -5597,7 +5605,7 @@
         <v>109</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="H14" s="15" t="s">
         <v>64</v>
@@ -5606,7 +5614,7 @@
         <v>65</v>
       </c>
       <c r="J14" s="19" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="K14" s="15"/>
       <c r="L14" s="18" t="n">
@@ -5619,16 +5627,16 @@
     </row>
     <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>39</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E15" s="15" t="s">
         <v>61</v>
@@ -5637,7 +5645,7 @@
         <v>109</v>
       </c>
       <c r="G15" s="15" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H15" s="15" t="s">
         <v>64</v>
@@ -5646,7 +5654,7 @@
         <v>65</v>
       </c>
       <c r="J15" s="19" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="K15" s="15"/>
       <c r="L15" s="18" t="n">
@@ -5659,7 +5667,7 @@
     </row>
     <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B16" s="15" t="s">
         <v>39</v>
@@ -5668,7 +5676,7 @@
         <v>186</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E16" s="15" t="s">
         <v>61</v>
@@ -5699,7 +5707,7 @@
     </row>
     <row r="17" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B17" s="15" t="s">
         <v>39</v>
@@ -5708,7 +5716,7 @@
         <v>172</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E17" s="15" t="s">
         <v>61</v>
@@ -5739,7 +5747,7 @@
     </row>
     <row r="18" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="15" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B18" s="15" t="s">
         <v>39</v>
@@ -5748,7 +5756,7 @@
         <v>176</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E18" s="15" t="s">
         <v>61</v>
@@ -5766,7 +5774,7 @@
         <v>65</v>
       </c>
       <c r="J18" s="19" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="K18" s="15"/>
       <c r="L18" s="18" t="n">
@@ -5779,7 +5787,7 @@
     </row>
     <row r="19" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B19" s="15" t="s">
         <v>39</v>
@@ -5788,7 +5796,7 @@
         <v>179</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E19" s="15" t="s">
         <v>61</v>
@@ -5819,16 +5827,16 @@
     </row>
     <row r="20" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B20" s="15" t="s">
         <v>39</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E20" s="15" t="s">
         <v>61</v>
@@ -5837,7 +5845,7 @@
         <v>130</v>
       </c>
       <c r="G20" s="15" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="H20" s="15" t="s">
         <v>71</v>
@@ -5859,7 +5867,7 @@
     </row>
     <row r="21" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B21" s="15" t="s">
         <v>39</v>
@@ -5868,7 +5876,7 @@
         <v>189</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E21" s="15" t="s">
         <v>61</v>
@@ -5877,7 +5885,7 @@
         <v>130</v>
       </c>
       <c r="G21" s="15" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="H21" s="15" t="s">
         <v>71</v>
@@ -5899,16 +5907,16 @@
     </row>
     <row r="22" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>39</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E22" s="15" t="s">
         <v>61</v>
@@ -5926,7 +5934,7 @@
         <v>65</v>
       </c>
       <c r="J22" s="19" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="K22" s="15"/>
       <c r="L22" s="18" t="n">
@@ -5939,16 +5947,16 @@
     </row>
     <row r="23" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B23" s="15" t="s">
         <v>39</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E23" s="15" t="s">
         <v>61</v>
@@ -5966,7 +5974,7 @@
         <v>65</v>
       </c>
       <c r="J23" s="19" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="K23" s="15"/>
       <c r="L23" s="18" t="n">
@@ -5979,7 +5987,7 @@
     </row>
     <row r="24" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B24" s="15" t="s">
         <v>81</v>
@@ -5988,7 +5996,7 @@
         <v>165</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E24" s="15" t="s">
         <v>61</v>
@@ -5997,7 +6005,7 @@
         <v>62</v>
       </c>
       <c r="G24" s="15" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="H24" s="15" t="s">
         <v>64</v>
@@ -6019,7 +6027,7 @@
     </row>
     <row r="25" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B25" s="15" t="s">
         <v>81</v>
@@ -6028,7 +6036,7 @@
         <v>186</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E25" s="15" t="s">
         <v>61</v>
@@ -6037,7 +6045,7 @@
         <v>130</v>
       </c>
       <c r="G25" s="15" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="H25" s="15" t="s">
         <v>71</v>
@@ -6059,7 +6067,7 @@
     </row>
     <row r="26" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B26" s="15" t="s">
         <v>88</v>
@@ -6068,7 +6076,7 @@
         <v>165</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E26" s="15" t="s">
         <v>61</v>
@@ -6077,7 +6085,7 @@
         <v>90</v>
       </c>
       <c r="G26" s="15" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="H26" s="15" t="s">
         <v>71</v>
@@ -6099,7 +6107,7 @@
     </row>
     <row r="27" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B27" s="15" t="s">
         <v>88</v>
@@ -6108,7 +6116,7 @@
         <v>6</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E27" s="15" t="s">
         <v>61</v>
@@ -6117,7 +6125,7 @@
         <v>90</v>
       </c>
       <c r="G27" s="15" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H27" s="15" t="s">
         <v>71</v>
@@ -6139,7 +6147,7 @@
     </row>
     <row r="28" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="15" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B28" s="15" t="s">
         <v>88</v>
@@ -6148,7 +6156,7 @@
         <v>186</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E28" s="15" t="s">
         <v>61</v>
@@ -6157,7 +6165,7 @@
         <v>130</v>
       </c>
       <c r="G28" s="15" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="H28" s="15" t="s">
         <v>71</v>
@@ -6179,7 +6187,7 @@
     </row>
     <row r="29" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B29" s="15" t="s">
         <v>88</v>
@@ -6188,7 +6196,7 @@
         <v>165</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E29" s="15" t="s">
         <v>61</v>
@@ -6219,7 +6227,7 @@
     </row>
     <row r="30" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="15" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B30" s="15" t="s">
         <v>88</v>
@@ -6228,7 +6236,7 @@
         <v>165</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E30" s="15" t="s">
         <v>61</v>
@@ -6237,7 +6245,7 @@
         <v>130</v>
       </c>
       <c r="G30" s="15" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="H30" s="15" t="s">
         <v>71</v>
@@ -6259,7 +6267,7 @@
     </row>
     <row r="31" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="15" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B31" s="15" t="s">
         <v>88</v>
@@ -6268,7 +6276,7 @@
         <v>165</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E31" s="15" t="s">
         <v>61</v>
@@ -6277,7 +6285,7 @@
         <v>130</v>
       </c>
       <c r="G31" s="15" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="H31" s="15" t="s">
         <v>71</v>
@@ -6299,7 +6307,7 @@
     </row>
     <row r="32" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="15" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B32" s="15" t="s">
         <v>88</v>
@@ -6308,7 +6316,7 @@
         <v>6</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E32" s="15" t="s">
         <v>61</v>
@@ -6317,7 +6325,7 @@
         <v>90</v>
       </c>
       <c r="G32" s="15" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H32" s="15" t="s">
         <v>64</v>
@@ -6339,7 +6347,7 @@
     </row>
     <row r="33" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="15" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B33" s="15" t="s">
         <v>107</v>
@@ -6348,7 +6356,7 @@
         <v>165</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E33" s="15" t="s">
         <v>61</v>
@@ -6366,7 +6374,7 @@
         <v>65</v>
       </c>
       <c r="J33" s="19" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="K33" s="15"/>
       <c r="L33" s="18" t="n">
@@ -6379,7 +6387,7 @@
     </row>
     <row r="34" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="15" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B34" s="15" t="s">
         <v>107</v>
@@ -6388,7 +6396,7 @@
         <v>155</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E34" s="15" t="s">
         <v>61</v>
@@ -6419,7 +6427,7 @@
     </row>
     <row r="35" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="15" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B35" s="15" t="s">
         <v>107</v>
@@ -6428,7 +6436,7 @@
         <v>6</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E35" s="15" t="s">
         <v>61</v>
@@ -6437,7 +6445,7 @@
         <v>109</v>
       </c>
       <c r="G35" s="15" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H35" s="15" t="s">
         <v>64</v>
@@ -6446,7 +6454,7 @@
         <v>65</v>
       </c>
       <c r="J35" s="19" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="K35" s="15"/>
       <c r="L35" s="18" t="n">
@@ -6459,7 +6467,7 @@
     </row>
     <row r="36" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="15" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B36" s="15" t="s">
         <v>107</v>
@@ -6468,7 +6476,7 @@
         <v>186</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E36" s="15" t="s">
         <v>61</v>
@@ -6477,7 +6485,7 @@
         <v>109</v>
       </c>
       <c r="G36" s="15" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H36" s="15" t="s">
         <v>64</v>
@@ -6499,7 +6507,7 @@
     </row>
     <row r="37" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="15" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B37" s="15" t="s">
         <v>107</v>
@@ -6508,7 +6516,7 @@
         <v>165</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E37" s="15" t="s">
         <v>61</v>
@@ -6539,7 +6547,7 @@
     </row>
     <row r="38" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="15" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B38" s="15" t="s">
         <v>107</v>
@@ -6548,7 +6556,7 @@
         <v>165</v>
       </c>
       <c r="D38" s="15" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E38" s="15" t="s">
         <v>61</v>
@@ -6566,7 +6574,7 @@
         <v>65</v>
       </c>
       <c r="J38" s="19" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="K38" s="15"/>
       <c r="L38" s="18" t="n">
@@ -6579,7 +6587,7 @@
     </row>
     <row r="39" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="15" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B39" s="15" t="s">
         <v>107</v>
@@ -6619,7 +6627,7 @@
     </row>
     <row r="40" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="15" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B40" s="15" t="s">
         <v>128</v>
@@ -6628,7 +6636,7 @@
         <v>6</v>
       </c>
       <c r="D40" s="15" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E40" s="15" t="s">
         <v>61</v>
@@ -6637,7 +6645,7 @@
         <v>130</v>
       </c>
       <c r="G40" s="15" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="H40" s="15" t="s">
         <v>64</v>
@@ -6659,7 +6667,7 @@
     </row>
     <row r="41" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="15" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B41" s="15" t="s">
         <v>128</v>
@@ -6668,7 +6676,7 @@
         <v>165</v>
       </c>
       <c r="D41" s="15" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E41" s="15" t="s">
         <v>61</v>
@@ -6677,7 +6685,7 @@
         <v>130</v>
       </c>
       <c r="G41" s="15" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="H41" s="15" t="s">
         <v>71</v>
@@ -6699,7 +6707,7 @@
     </row>
     <row r="42" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="15" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B42" s="15" t="s">
         <v>134</v>
@@ -6708,7 +6716,7 @@
         <v>6</v>
       </c>
       <c r="D42" s="15" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E42" s="15" t="s">
         <v>61</v>
@@ -6717,7 +6725,7 @@
         <v>136</v>
       </c>
       <c r="G42" s="15" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="H42" s="15" t="s">
         <v>71</v>
@@ -6726,7 +6734,7 @@
         <v>72</v>
       </c>
       <c r="J42" s="19" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="K42" s="15"/>
       <c r="L42" s="18" t="n">
@@ -6739,7 +6747,7 @@
     </row>
     <row r="43" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="15" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B43" s="15" t="s">
         <v>134</v>
@@ -6748,7 +6756,7 @@
         <v>6</v>
       </c>
       <c r="D43" s="15" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="E43" s="15" t="s">
         <v>61</v>
@@ -6757,7 +6765,7 @@
         <v>136</v>
       </c>
       <c r="G43" s="15" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="H43" s="15" t="s">
         <v>64</v>
@@ -6766,7 +6774,7 @@
         <v>65</v>
       </c>
       <c r="J43" s="19" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="K43" s="15"/>
       <c r="L43" s="18" t="n">
@@ -6779,7 +6787,7 @@
     </row>
     <row r="44" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="15" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B44" s="15" t="s">
         <v>142</v>
@@ -6788,7 +6796,7 @@
         <v>6</v>
       </c>
       <c r="D44" s="15" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="E44" s="15" t="s">
         <v>144</v>
@@ -6819,16 +6827,16 @@
     </row>
     <row r="45" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="15" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B45" s="15" t="s">
         <v>147</v>
       </c>
       <c r="C45" s="15" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D45" s="15" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E45" s="15" t="s">
         <v>149</v>
@@ -6849,7 +6857,7 @@
         <v>46220</v>
       </c>
       <c r="K45" s="15" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="L45" s="18" t="n">
         <v>1</v>
@@ -6931,7 +6939,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>65</v>
@@ -6939,7 +6947,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6959,7 +6967,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
test: complete Brick avatar review
</commit_message>
<xml_diff>
--- a/playground/component-coverage.xlsx
+++ b/playground/component-coverage.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4781" uniqueCount="1314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4780" uniqueCount="1314">
   <si>
     <t xml:space="preserve">Brick Component Coverage Index</t>
   </si>
@@ -2182,307 +2182,307 @@
     <t xml:space="preserve">Latest owner run records every numbered result and corrects any finding before package completion</t>
   </si>
   <si>
+    <t xml:space="preserve">AVA-35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Public guide covers use boundaries, explicit alt/fallback, sizes, shapes, status meaning, composition, loading, accessibility, native/ref, and CSS hooks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../docs/components/avatar/README.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVA-36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avatar component changelog records the initial direct contract, status rings, evidence, and deferred AvatarGroup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../docs/components/avatar/CHANGELOG.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVA-37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Independent Consumer uses the public Avatar subpath for loaded and fallback collaborators, visible statuses, and NotificationBadge composition across desktop/mobile and axe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVA-38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legacy Avatar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fresh searches found no Core consumers; Avatar/AvatarGroup source, aliases, barrel export, and obsolete live examples are removed and Core builds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVA-39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AvatarGroup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AvatarGroup remains deliberately excluded until a real grouped-identity workflow defines semantics, order, overflow, hidden members, and Consumer proof</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toggle Family Evidence Matrix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence gates for adopted Toggle and ToggleGroup APIs, Atom-owned interaction, package proof, Consumer cutover, and completed Core retirement.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toggle directly composes public Atom 0.3.3 Toggle.Root without Core, framework, or local behavior state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../src/components/toggle/Toggle.tsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Owner-approved capability audit confirms Atom owns pressed/value state, activation, disabled semantics, roving focus, orientation, looping, RTL, composition, slots, and refs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../../docs/toggle-component-brief.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Root and toggle/toggle-group subpath exports, declarations, direct Toggle, compound Group namespace, named parts, and closed unions match the adopted brief</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shortest Toggle emits a native type=button with stable class/slot, false aria-pressed, off state, and soft/md/rounded defaults</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../test/components/toggle.test.tsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Behavior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atom-owned uncontrolled pointer, Space, and controlled pressed paths update aria-pressed and onPressedChange without Brick state duplication</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Native/ARIA/data props, class, style, slot, icon-only metadata, ref, asChild, and render composition are preserved</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soft, outline, and ghost variants; sm/md/lg sizes; rounded/pill shapes; and icon-only geometry form closed recipes without tone or arbitrary radius</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">States</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rest, hover, active, focus-visible, selected, disabled, and selected-disabled recipes use semantic tokens and preserve native disabled behavior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/toggle.spec.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ToggleGroup.Root</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Root emits a named role=group with stable class/slot, separated horizontal layout, soft/md/rounded defaults, and no extra behavior layer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Selection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discriminated single string and multiple string-array contracts forward controlled/uncontrolled values and narrowed callbacks without a second store</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ToggleGroup.Item</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item requires value, emits native pressed button metadata, preserves disabled/native/composition/ref paths, and exposes only item iconOnly presentation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keyboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ToggleGroup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One roving Tab stop plus Arrow, Home, End, looping, activation, and disabled-item skipping remain Atom-owned and pass in real browsers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Direction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Horizontal/vertical orientation metadata drives layout and Atom mirrors horizontal Arrow navigation in RTL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Separated default preserves inter-item gap and natural wrapping for localized multiple filter pills</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attached horizontal and vertical groups collapse adjacent borders and apply logical outer radii for rounded and pill shapes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Layout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fullWidth fills available inline size and distributes items without changing Atom selection behavior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stable visible or explicit icon labels, group naming, aria-pressed, disabled state, and controlled required-view handling preserve understandable semantics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compiled layered CSS uses Brick classes, logical properties, semantic tokens, and documented --brick-toggle variables without global leakage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../src/components/toggle/toggle.css</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reviewed light/dark baselines preserve neutral rest, accent selected hierarchy, sizes, shapes, and attached/separated group geometry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forced-colors emulation preserves explicit selected, disabled, border, and focus boundaries without color-only state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Responsive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Constrained mobile, long unbroken/localized labels, wrapping, mixed direction, and RTL remain contained without document overflow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Root class, style, slot, scoped appearance, group variables, and component-token overrides remain local and inspectable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The /toggle workbench exposes overview, complete standalone recipes, sizes/shapes/icons, attached single, separated multiple, vertical/disabled, customization, mobile stress, and RTL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vitest and Testing Library cover defaults, recipes, activation, callbacks, native props, refs, disabled paths, composition, and discriminated values</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Public root/subpath types accept supported contracts and reject standalone value, tone, invalid recipes, mismatched multiple values, item recipe overrides, and callable Group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Node package boundary, export identity, stylesheet, declarations, deterministic SSR, and dry-pack checks include both public subpaths</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clean packed React 18/19 consumers import root/subpath identities, SSR-render Toggle and ToggleGroup, typecheck, and load compiled CSS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strict typecheck, production build, CSS report, and 100% Brick component-source line coverage pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seven focused browser checks cover standalone activation, recipes, single/multiple state, roving focus, disabled behavior, mobile/RTL, axe, and forced colors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Canonical Toggle route has no automatically detectable axe violations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seven reviewed Chromium baselines cover recipes, sizes/shapes, attached single, dark standalone/multiple, mobile RTL stress, and forced colors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chromium, Firefox, WebKit, Pixel, and iPhone focused release-matrix checks pass where applicable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numbered Toggle protocol covers hierarchy, activation, keyboard/roving focus, selection modes, geometry, zoom/mobile/RTL, VoiceOver, preferences, and customization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">manual-tests/toggle.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latest owner run records every numbered Toggle and ToggleGroup result and corrects any finding before package completion</t>
+  </si>
+  <si>
     <t xml:space="preserve">Owner manual review intentionally deferred</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVA-35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Public guide covers use boundaries, explicit alt/fallback, sizes, shapes, status meaning, composition, loading, accessibility, native/ref, and CSS hooks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">../docs/components/avatar/README.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVA-36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avatar component changelog records the initial direct contract, status rings, evidence, and deferred AvatarGroup</t>
-  </si>
-  <si>
-    <t xml:space="preserve">../docs/components/avatar/CHANGELOG.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVA-37</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Independent Consumer uses the public Avatar subpath for loaded and fallback collaborators, visible statuses, and NotificationBadge composition across desktop/mobile and axe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVA-38</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Legacy Avatar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fresh searches found no Core consumers; Avatar/AvatarGroup source, aliases, barrel export, and obsolete live examples are removed and Core builds</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVA-39</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AvatarGroup</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AvatarGroup remains deliberately excluded until a real grouped-identity workflow defines semantics, order, overflow, hidden members, and Consumer proof</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Toggle Family Evidence Matrix</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evidence gates for adopted Toggle and ToggleGroup APIs, Atom-owned interaction, package proof, Consumer cutover, and completed Core retirement.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Toggle directly composes public Atom 0.3.3 Toggle.Root without Core, framework, or local behavior state</t>
-  </si>
-  <si>
-    <t xml:space="preserve">../src/components/toggle/Toggle.tsx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Owner-approved capability audit confirms Atom owns pressed/value state, activation, disabled semantics, roving focus, orientation, looping, RTL, composition, slots, and refs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">../../docs/toggle-component-brief.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Root and toggle/toggle-group subpath exports, declarations, direct Toggle, compound Group namespace, named parts, and closed unions match the adopted brief</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shortest Toggle emits a native type=button with stable class/slot, false aria-pressed, off state, and soft/md/rounded defaults</t>
-  </si>
-  <si>
-    <t xml:space="preserve">../test/components/toggle.test.tsx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Behavior</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Atom-owned uncontrolled pointer, Space, and controlled pressed paths update aria-pressed and onPressedChange without Brick state duplication</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Native/ARIA/data props, class, style, slot, icon-only metadata, ref, asChild, and render composition are preserved</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Soft, outline, and ghost variants; sm/md/lg sizes; rounded/pill shapes; and icon-only geometry form closed recipes without tone or arbitrary radius</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">States</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rest, hover, active, focus-visible, selected, disabled, and selected-disabled recipes use semantic tokens and preserve native disabled behavior</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tests/toggle.spec.ts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ToggleGroup.Root</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Root emits a named role=group with stable class/slot, separated horizontal layout, soft/md/rounded defaults, and no extra behavior layer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Selection</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Discriminated single string and multiple string-array contracts forward controlled/uncontrolled values and narrowed callbacks without a second store</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ToggleGroup.Item</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Item requires value, emits native pressed button metadata, preserves disabled/native/composition/ref paths, and exposes only item iconOnly presentation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keyboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ToggleGroup</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One roving Tab stop plus Arrow, Home, End, looping, activation, and disabled-item skipping remain Atom-owned and pass in real browsers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Direction</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Horizontal/vertical orientation metadata drives layout and Atom mirrors horizontal Arrow navigation in RTL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Separated default preserves inter-item gap and natural wrapping for localized multiple filter pills</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Attached horizontal and vertical groups collapse adjacent borders and apply logical outer radii for rounded and pill shapes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Layout</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fullWidth fills available inline size and distributes items without changing Atom selection behavior</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stable visible or explicit icon labels, group naming, aria-pressed, disabled state, and controlled required-view handling preserve understandable semantics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compiled layered CSS uses Brick classes, logical properties, semantic tokens, and documented --brick-toggle variables without global leakage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">../src/components/toggle/toggle.css</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reviewed light/dark baselines preserve neutral rest, accent selected hierarchy, sizes, shapes, and attached/separated group geometry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Forced-colors emulation preserves explicit selected, disabled, border, and focus boundaries without color-only state</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Responsive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Constrained mobile, long unbroken/localized labels, wrapping, mixed direction, and RTL remain contained without document overflow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Root class, style, slot, scoped appearance, group variables, and component-token overrides remain local and inspectable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The /toggle workbench exposes overview, complete standalone recipes, sizes/shapes/icons, attached single, separated multiple, vertical/disabled, customization, mobile stress, and RTL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vitest and Testing Library cover defaults, recipes, activation, callbacks, native props, refs, disabled paths, composition, and discriminated values</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Public root/subpath types accept supported contracts and reject standalone value, tone, invalid recipes, mismatched multiple values, item recipe overrides, and callable Group</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node package boundary, export identity, stylesheet, declarations, deterministic SSR, and dry-pack checks include both public subpaths</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clean packed React 18/19 consumers import root/subpath identities, SSR-render Toggle and ToggleGroup, typecheck, and load compiled CSS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strict typecheck, production build, CSS report, and 100% Brick component-source line coverage pass</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seven focused browser checks cover standalone activation, recipes, single/multiple state, roving focus, disabled behavior, mobile/RTL, axe, and forced colors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Canonical Toggle route has no automatically detectable axe violations</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seven reviewed Chromium baselines cover recipes, sizes/shapes, attached single, dark standalone/multiple, mobile RTL stress, and forced colors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-32</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chromium, Firefox, WebKit, Pixel, and iPhone focused release-matrix checks pass where applicable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-33</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Numbered Toggle protocol covers hierarchy, activation, keyboard/roving focus, selection modes, geometry, zoom/mobile/RTL, VoiceOver, preferences, and customization</t>
-  </si>
-  <si>
-    <t xml:space="preserve">manual-tests/toggle.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-34</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Latest owner run records every numbered Toggle and ToggleGroup result and corrects any finding before package completion</t>
   </si>
   <si>
     <t xml:space="preserve">TOG-35</t>
@@ -4273,7 +4273,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="24">
+  <dxfs count="22">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -4459,22 +4459,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF991B1B"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFEF3C7"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF92400E"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -4918,7 +4902,7 @@
       </c>
       <c r="D4" s="5" t="n">
         <f aca="false">COUNTIF(N8:N20,"complete")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>4</v>
@@ -4932,7 +4916,7 @@
       </c>
       <c r="H4" s="6" t="n">
         <f aca="false">IFERROR(SUMPRODUCT(B8:B20,J8:J20)/SUM(B8:B20),0)</f>
-        <v>0.917695473251029</v>
+        <v>0.919753086419753</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5335,7 +5319,7 @@
       </c>
       <c r="D14" s="8" t="n">
         <f aca="false">COUNTIF(Avatar!H9:H47,"partial")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" s="8" t="n">
         <f aca="false">COUNTIF(Avatar!H9:H47,"implemented")</f>
@@ -5347,7 +5331,7 @@
       </c>
       <c r="G14" s="8" t="n">
         <f aca="false">COUNTIF(Avatar!H9:H47,"verified")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H14" s="8" t="n">
         <f aca="false">COUNTIF(Avatar!H9:H47,"blocked")</f>
@@ -5359,11 +5343,11 @@
       </c>
       <c r="J14" s="9" t="n">
         <f aca="false">IFERROR(SUM(Avatar!M9:M47)/SUM(Avatar!L9:L47),0)</f>
-        <v>0.974358974358974</v>
+        <v>1</v>
       </c>
       <c r="K14" s="8" t="str">
         <f aca="false">IF(COUNTIFS(Avatar!E9:E47,"package",Avatar!M9:M47,"&lt;1")=0,"complete","open")</f>
-        <v>open</v>
+        <v>complete</v>
       </c>
       <c r="L14" s="8" t="str">
         <f aca="false">IF(COUNTIFS(Avatar!E9:E47,"consumer",Avatar!M9:M47,"&lt;1")=0,"complete","open")</f>
@@ -5375,7 +5359,7 @@
       </c>
       <c r="N14" s="1" t="str">
         <f aca="false">IF(H14&gt;0,"blocked",IF(AND(J14=1,K14="complete",L14="complete",M14="complete"),"complete",IF(J14=0,"not started","in progress")))</f>
-        <v>in progress</v>
+        <v>complete</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5842,14 +5826,14 @@
       </c>
       <c r="D4" s="5" t="n">
         <f aca="false">SUM(M9:M47)</f>
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F4" s="6" t="n">
         <f aca="false">IFERROR(D4/SUM(L9:L47),0)</f>
-        <v>0.974358974358974</v>
+        <v>1</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>4</v>
@@ -5863,7 +5847,7 @@
       </c>
       <c r="J4" s="5" t="str">
         <f aca="false">IF(COUNTIFS(E9:E47,"package",M9:M47,"&lt;1")=0,"complete","open")</f>
-        <v>open</v>
+        <v>complete</v>
       </c>
       <c r="K4" s="4" t="s">
         <v>17</v>
@@ -7274,26 +7258,26 @@
         <v>704</v>
       </c>
       <c r="H42" s="15" t="s">
-        <v>346</v>
+        <v>81</v>
       </c>
       <c r="I42" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="J42" s="19"/>
-      <c r="K42" s="15" t="s">
-        <v>707</v>
-      </c>
+      <c r="J42" s="19" t="n">
+        <v>46223</v>
+      </c>
+      <c r="K42" s="15"/>
       <c r="L42" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M42" s="18" t="n">
         <f aca="false">IF(H42="not applicable",IF(K42&lt;&gt;"",1,0),IF(I42="yes",IF(H42="verified",1,0),IF(OR(H42="tested",H42="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="15" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B43" s="15" t="s">
         <v>144</v>
@@ -7302,7 +7286,7 @@
         <v>25</v>
       </c>
       <c r="D43" s="15" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="E43" s="15" t="s">
         <v>71</v>
@@ -7311,7 +7295,7 @@
         <v>146</v>
       </c>
       <c r="G43" s="16" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="H43" s="15" t="s">
         <v>74</v>
@@ -7333,7 +7317,7 @@
     </row>
     <row r="44" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="15" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="B44" s="15" t="s">
         <v>144</v>
@@ -7342,7 +7326,7 @@
         <v>25</v>
       </c>
       <c r="D44" s="15" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="E44" s="15" t="s">
         <v>71</v>
@@ -7351,7 +7335,7 @@
         <v>146</v>
       </c>
       <c r="G44" s="16" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="H44" s="15" t="s">
         <v>74</v>
@@ -7373,7 +7357,7 @@
     </row>
     <row r="45" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="15" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="B45" s="15" t="s">
         <v>152</v>
@@ -7382,7 +7366,7 @@
         <v>25</v>
       </c>
       <c r="D45" s="15" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="E45" s="15" t="s">
         <v>154</v>
@@ -7413,16 +7397,16 @@
     </row>
     <row r="46" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="15" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="B46" s="15" t="s">
         <v>157</v>
       </c>
       <c r="C46" s="15" t="s">
+        <v>716</v>
+      </c>
+      <c r="D46" s="15" t="s">
         <v>717</v>
-      </c>
-      <c r="D46" s="15" t="s">
-        <v>718</v>
       </c>
       <c r="E46" s="15" t="s">
         <v>159</v>
@@ -7453,16 +7437,16 @@
     </row>
     <row r="47" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="15" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="B47" s="15" t="s">
         <v>625</v>
       </c>
       <c r="C47" s="15" t="s">
+        <v>719</v>
+      </c>
+      <c r="D47" s="15" t="s">
         <v>720</v>
-      </c>
-      <c r="D47" s="15" t="s">
-        <v>721</v>
       </c>
       <c r="E47" s="15" t="s">
         <v>71</v>
@@ -7608,7 +7592,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -7625,7 +7609,7 @@
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -7744,7 +7728,7 @@
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="B9" s="15" t="s">
         <v>69</v>
@@ -7753,7 +7737,7 @@
         <v>26</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E9" s="15" t="s">
         <v>71</v>
@@ -7762,7 +7746,7 @@
         <v>72</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="H9" s="15" t="s">
         <v>74</v>
@@ -7784,7 +7768,7 @@
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="B10" s="15" t="s">
         <v>77</v>
@@ -7793,7 +7777,7 @@
         <v>536</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="E10" s="15" t="s">
         <v>71</v>
@@ -7802,7 +7786,7 @@
         <v>79</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="H10" s="15" t="s">
         <v>81</v>
@@ -7824,7 +7808,7 @@
     </row>
     <row r="11" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="B11" s="15" t="s">
         <v>69</v>
@@ -7833,7 +7817,7 @@
         <v>536</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="E11" s="15" t="s">
         <v>71</v>
@@ -7864,7 +7848,7 @@
     </row>
     <row r="12" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="B12" s="15" t="s">
         <v>49</v>
@@ -7873,7 +7857,7 @@
         <v>26</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E12" s="15" t="s">
         <v>71</v>
@@ -7882,7 +7866,7 @@
         <v>119</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="H12" s="15" t="s">
         <v>74</v>
@@ -7904,16 +7888,16 @@
     </row>
     <row r="13" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
+        <v>734</v>
+      </c>
+      <c r="B13" s="15" t="s">
         <v>735</v>
-      </c>
-      <c r="B13" s="15" t="s">
-        <v>736</v>
       </c>
       <c r="C13" s="15" t="s">
         <v>26</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="E13" s="15" t="s">
         <v>71</v>
@@ -7922,7 +7906,7 @@
         <v>119</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="H13" s="15" t="s">
         <v>74</v>
@@ -7944,7 +7928,7 @@
     </row>
     <row r="14" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="B14" s="15" t="s">
         <v>69</v>
@@ -7953,7 +7937,7 @@
         <v>26</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="E14" s="15" t="s">
         <v>71</v>
@@ -7962,7 +7946,7 @@
         <v>119</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="H14" s="15" t="s">
         <v>74</v>
@@ -7984,7 +7968,7 @@
     </row>
     <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>91</v>
@@ -7993,7 +7977,7 @@
         <v>26</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="E15" s="15" t="s">
         <v>71</v>
@@ -8002,7 +7986,7 @@
         <v>119</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="H15" s="15" t="s">
         <v>74</v>
@@ -8024,16 +8008,16 @@
     </row>
     <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
+        <v>741</v>
+      </c>
+      <c r="B16" s="15" t="s">
         <v>742</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>743</v>
       </c>
       <c r="C16" s="15" t="s">
         <v>26</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="E16" s="15" t="s">
         <v>71</v>
@@ -8042,7 +8026,7 @@
         <v>119</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="H16" s="15" t="s">
         <v>74</v>
@@ -8064,16 +8048,16 @@
     </row>
     <row r="17" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="B17" s="15" t="s">
         <v>49</v>
       </c>
       <c r="C17" s="15" t="s">
+        <v>746</v>
+      </c>
+      <c r="D17" s="15" t="s">
         <v>747</v>
-      </c>
-      <c r="D17" s="15" t="s">
-        <v>748</v>
       </c>
       <c r="E17" s="15" t="s">
         <v>71</v>
@@ -8082,7 +8066,7 @@
         <v>119</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="H17" s="15" t="s">
         <v>74</v>
@@ -8104,16 +8088,16 @@
     </row>
     <row r="18" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="15" t="s">
+        <v>748</v>
+      </c>
+      <c r="B18" s="15" t="s">
         <v>749</v>
       </c>
-      <c r="B18" s="15" t="s">
+      <c r="C18" s="15" t="s">
+        <v>746</v>
+      </c>
+      <c r="D18" s="15" t="s">
         <v>750</v>
-      </c>
-      <c r="C18" s="15" t="s">
-        <v>747</v>
-      </c>
-      <c r="D18" s="15" t="s">
-        <v>751</v>
       </c>
       <c r="E18" s="15" t="s">
         <v>71</v>
@@ -8144,16 +8128,16 @@
     </row>
     <row r="19" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="B19" s="15" t="s">
         <v>49</v>
       </c>
       <c r="C19" s="15" t="s">
+        <v>752</v>
+      </c>
+      <c r="D19" s="15" t="s">
         <v>753</v>
-      </c>
-      <c r="D19" s="15" t="s">
-        <v>754</v>
       </c>
       <c r="E19" s="15" t="s">
         <v>71</v>
@@ -8162,7 +8146,7 @@
         <v>119</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="H19" s="15" t="s">
         <v>74</v>
@@ -8184,16 +8168,16 @@
     </row>
     <row r="20" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
+        <v>754</v>
+      </c>
+      <c r="B20" s="15" t="s">
         <v>755</v>
       </c>
-      <c r="B20" s="15" t="s">
+      <c r="C20" s="15" t="s">
         <v>756</v>
       </c>
-      <c r="C20" s="15" t="s">
+      <c r="D20" s="15" t="s">
         <v>757</v>
-      </c>
-      <c r="D20" s="15" t="s">
-        <v>758</v>
       </c>
       <c r="E20" s="15" t="s">
         <v>71</v>
@@ -8202,7 +8186,7 @@
         <v>119</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="H20" s="15" t="s">
         <v>74</v>
@@ -8224,16 +8208,16 @@
     </row>
     <row r="21" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
+        <v>758</v>
+      </c>
+      <c r="B21" s="15" t="s">
         <v>759</v>
       </c>
-      <c r="B21" s="15" t="s">
+      <c r="C21" s="15" t="s">
+        <v>756</v>
+      </c>
+      <c r="D21" s="15" t="s">
         <v>760</v>
-      </c>
-      <c r="C21" s="15" t="s">
-        <v>757</v>
-      </c>
-      <c r="D21" s="15" t="s">
-        <v>761</v>
       </c>
       <c r="E21" s="15" t="s">
         <v>71</v>
@@ -8242,7 +8226,7 @@
         <v>119</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="H21" s="15" t="s">
         <v>74</v>
@@ -8264,16 +8248,16 @@
     </row>
     <row r="22" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>560</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="E22" s="15" t="s">
         <v>71</v>
@@ -8304,16 +8288,16 @@
     </row>
     <row r="23" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="B23" s="15" t="s">
         <v>560</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="E23" s="15" t="s">
         <v>71</v>
@@ -8344,16 +8328,16 @@
     </row>
     <row r="24" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
+        <v>765</v>
+      </c>
+      <c r="B24" s="15" t="s">
         <v>766</v>
       </c>
-      <c r="B24" s="15" t="s">
+      <c r="C24" s="15" t="s">
+        <v>756</v>
+      </c>
+      <c r="D24" s="15" t="s">
         <v>767</v>
-      </c>
-      <c r="C24" s="15" t="s">
-        <v>757</v>
-      </c>
-      <c r="D24" s="15" t="s">
-        <v>768</v>
       </c>
       <c r="E24" s="15" t="s">
         <v>71</v>
@@ -8362,7 +8346,7 @@
         <v>119</v>
       </c>
       <c r="G24" s="16" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="H24" s="15" t="s">
         <v>74</v>
@@ -8384,7 +8368,7 @@
     </row>
     <row r="25" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="B25" s="15" t="s">
         <v>549</v>
@@ -8393,7 +8377,7 @@
         <v>536</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="E25" s="15" t="s">
         <v>71</v>
@@ -8402,7 +8386,7 @@
         <v>119</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="H25" s="15" t="s">
         <v>74</v>
@@ -8424,7 +8408,7 @@
     </row>
     <row r="26" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="B26" s="15" t="s">
         <v>91</v>
@@ -8433,7 +8417,7 @@
         <v>536</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="E26" s="15" t="s">
         <v>71</v>
@@ -8442,7 +8426,7 @@
         <v>72</v>
       </c>
       <c r="G26" s="16" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="H26" s="15" t="s">
         <v>74</v>
@@ -8464,7 +8448,7 @@
     </row>
     <row r="27" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="B27" s="15" t="s">
         <v>91</v>
@@ -8473,7 +8457,7 @@
         <v>536</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="E27" s="15" t="s">
         <v>71</v>
@@ -8504,7 +8488,7 @@
     </row>
     <row r="28" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="15" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="B28" s="15" t="s">
         <v>91</v>
@@ -8513,7 +8497,7 @@
         <v>536</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="E28" s="15" t="s">
         <v>71</v>
@@ -8522,7 +8506,7 @@
         <v>119</v>
       </c>
       <c r="G28" s="16" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="H28" s="15" t="s">
         <v>74</v>
@@ -8544,16 +8528,16 @@
     </row>
     <row r="29" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
+        <v>777</v>
+      </c>
+      <c r="B29" s="15" t="s">
         <v>778</v>
-      </c>
-      <c r="B29" s="15" t="s">
-        <v>779</v>
       </c>
       <c r="C29" s="15" t="s">
         <v>536</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="E29" s="15" t="s">
         <v>71</v>
@@ -8562,7 +8546,7 @@
         <v>119</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="H29" s="15" t="s">
         <v>74</v>
@@ -8584,7 +8568,7 @@
     </row>
     <row r="30" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="15" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="B30" s="15" t="s">
         <v>580</v>
@@ -8593,7 +8577,7 @@
         <v>536</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E30" s="15" t="s">
         <v>71</v>
@@ -8624,7 +8608,7 @@
     </row>
     <row r="31" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="15" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="B31" s="15" t="s">
         <v>98</v>
@@ -8633,7 +8617,7 @@
         <v>536</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="E31" s="15" t="s">
         <v>71</v>
@@ -8664,7 +8648,7 @@
     </row>
     <row r="32" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="15" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="B32" s="15" t="s">
         <v>117</v>
@@ -8673,7 +8657,7 @@
         <v>536</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="E32" s="15" t="s">
         <v>71</v>
@@ -8682,7 +8666,7 @@
         <v>119</v>
       </c>
       <c r="G32" s="16" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="H32" s="15" t="s">
         <v>74</v>
@@ -8704,7 +8688,7 @@
     </row>
     <row r="33" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="15" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="B33" s="15" t="s">
         <v>117</v>
@@ -8713,7 +8697,7 @@
         <v>536</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="E33" s="15" t="s">
         <v>71</v>
@@ -8744,7 +8728,7 @@
     </row>
     <row r="34" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="15" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="B34" s="15" t="s">
         <v>117</v>
@@ -8753,7 +8737,7 @@
         <v>536</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="E34" s="15" t="s">
         <v>71</v>
@@ -8784,7 +8768,7 @@
     </row>
     <row r="35" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="15" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="B35" s="15" t="s">
         <v>117</v>
@@ -8793,7 +8777,7 @@
         <v>536</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="E35" s="15" t="s">
         <v>71</v>
@@ -8824,7 +8808,7 @@
     </row>
     <row r="36" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="15" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="B36" s="15" t="s">
         <v>117</v>
@@ -8833,7 +8817,7 @@
         <v>536</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E36" s="15" t="s">
         <v>71</v>
@@ -8842,7 +8826,7 @@
         <v>119</v>
       </c>
       <c r="G36" s="16" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="H36" s="15" t="s">
         <v>74</v>
@@ -8864,7 +8848,7 @@
     </row>
     <row r="37" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="15" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="B37" s="15" t="s">
         <v>117</v>
@@ -8873,7 +8857,7 @@
         <v>536</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="E37" s="15" t="s">
         <v>71</v>
@@ -8882,7 +8866,7 @@
         <v>119</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="H37" s="15" t="s">
         <v>74</v>
@@ -8904,7 +8888,7 @@
     </row>
     <row r="38" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="15" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="B38" s="15" t="s">
         <v>117</v>
@@ -8913,7 +8897,7 @@
         <v>536</v>
       </c>
       <c r="D38" s="15" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="E38" s="15" t="s">
         <v>71</v>
@@ -8922,7 +8906,7 @@
         <v>119</v>
       </c>
       <c r="G38" s="16" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="H38" s="15" t="s">
         <v>74</v>
@@ -8944,7 +8928,7 @@
     </row>
     <row r="39" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="15" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="B39" s="15" t="s">
         <v>117</v>
@@ -8953,7 +8937,7 @@
         <v>536</v>
       </c>
       <c r="D39" s="15" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="E39" s="15" t="s">
         <v>71</v>
@@ -8984,7 +8968,7 @@
     </row>
     <row r="40" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="15" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="B40" s="15" t="s">
         <v>117</v>
@@ -8993,7 +8977,7 @@
         <v>536</v>
       </c>
       <c r="D40" s="15" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="E40" s="15" t="s">
         <v>71</v>
@@ -9024,7 +9008,7 @@
     </row>
     <row r="41" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="15" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="B41" s="15" t="s">
         <v>138</v>
@@ -9033,7 +9017,7 @@
         <v>536</v>
       </c>
       <c r="D41" s="15" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="E41" s="15" t="s">
         <v>71</v>
@@ -9042,7 +9026,7 @@
         <v>140</v>
       </c>
       <c r="G41" s="16" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="H41" s="15" t="s">
         <v>74</v>
@@ -9064,7 +9048,7 @@
     </row>
     <row r="42" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="15" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="B42" s="15" t="s">
         <v>138</v>
@@ -9073,7 +9057,7 @@
         <v>536</v>
       </c>
       <c r="D42" s="15" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="E42" s="15" t="s">
         <v>71</v>
@@ -9082,7 +9066,7 @@
         <v>140</v>
       </c>
       <c r="G42" s="16" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="H42" s="15" t="s">
         <v>346</v>
@@ -9092,7 +9076,7 @@
       </c>
       <c r="J42" s="19"/>
       <c r="K42" s="15" t="s">
-        <v>707</v>
+        <v>807</v>
       </c>
       <c r="L42" s="18" t="n">
         <v>1</v>
@@ -9150,7 +9134,7 @@
         <v>144</v>
       </c>
       <c r="C44" s="15" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="D44" s="15" t="s">
         <v>812</v>
@@ -9282,7 +9266,7 @@
         <v>79</v>
       </c>
       <c r="G47" s="16" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="H47" s="15" t="s">
         <v>81</v>
@@ -9796,7 +9780,7 @@
         <v>841</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="C15" s="15" t="s">
         <v>27</v>
@@ -9996,7 +9980,7 @@
         <v>852</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="C20" s="15" t="s">
         <v>27</v>
@@ -10196,7 +10180,7 @@
         <v>864</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="C25" s="15" t="s">
         <v>27</v>
@@ -10743,7 +10727,7 @@
         <v>46221</v>
       </c>
       <c r="K38" s="15" t="s">
-        <v>707</v>
+        <v>807</v>
       </c>
       <c r="L38" s="18" t="n">
         <v>1</v>
@@ -10905,7 +10889,7 @@
         <v>46221</v>
       </c>
       <c r="K42" s="15" t="s">
-        <v>707</v>
+        <v>807</v>
       </c>
       <c r="L42" s="18" t="n">
         <v>1</v>
@@ -12051,7 +12035,7 @@
         <v>966</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="C26" s="15" t="s">
         <v>28</v>
@@ -12091,7 +12075,7 @@
         <v>968</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="C27" s="15" t="s">
         <v>28</v>
@@ -12716,7 +12700,7 @@
       </c>
       <c r="J42" s="19"/>
       <c r="K42" s="15" t="s">
-        <v>707</v>
+        <v>807</v>
       </c>
       <c r="L42" s="18" t="n">
         <v>1</v>
@@ -13740,7 +13724,7 @@
         <v>1049</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="C23" s="15" t="s">
         <v>29</v>
@@ -13780,7 +13764,7 @@
         <v>1051</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="C24" s="15" t="s">
         <v>29</v>
@@ -14072,7 +14056,7 @@
         <v>1073</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="C31" s="15" t="s">
         <v>196</v>
@@ -14112,7 +14096,7 @@
         <v>1075</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="C32" s="15" t="s">
         <v>196</v>
@@ -14194,7 +14178,7 @@
         <v>1081</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="C34" s="15" t="s">
         <v>29</v>
@@ -14545,7 +14529,7 @@
         <v>46222</v>
       </c>
       <c r="K42" s="15" t="s">
-        <v>707</v>
+        <v>807</v>
       </c>
       <c r="L42" s="18" t="n">
         <v>1</v>
@@ -15462,7 +15446,7 @@
         <v>1158</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="C21" s="15" t="s">
         <v>30</v>
@@ -15502,7 +15486,7 @@
         <v>1160</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="C22" s="15" t="s">
         <v>30</v>
@@ -15542,7 +15526,7 @@
         <v>1162</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="C23" s="15" t="s">
         <v>30</v>
@@ -15582,7 +15566,7 @@
         <v>1164</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="C24" s="15" t="s">
         <v>30</v>
@@ -15834,7 +15818,7 @@
         <v>1180</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="C30" s="15" t="s">
         <v>196</v>
@@ -15874,7 +15858,7 @@
         <v>1182</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="C31" s="15" t="s">
         <v>196</v>
@@ -15958,7 +15942,7 @@
         <v>1186</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="C33" s="15" t="s">
         <v>30</v>
@@ -16353,7 +16337,7 @@
         <v>46222</v>
       </c>
       <c r="K42" s="15" t="s">
-        <v>707</v>
+        <v>807</v>
       </c>
       <c r="L42" s="18" t="n">
         <v>1</v>
@@ -17512,7 +17496,7 @@
         <v>1267</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="C27" s="15" t="s">
         <v>31</v>
@@ -17552,7 +17536,7 @@
         <v>1269</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="C28" s="15" t="s">
         <v>31</v>
@@ -17592,7 +17576,7 @@
         <v>1271</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="C29" s="15" t="s">
         <v>1272</v>
@@ -17632,7 +17616,7 @@
         <v>1274</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="C30" s="15" t="s">
         <v>1275</v>
@@ -17796,7 +17780,7 @@
         <v>1284</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="C34" s="15" t="s">
         <v>196</v>
@@ -17836,7 +17820,7 @@
         <v>1286</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="C35" s="15" t="s">
         <v>196</v>
@@ -17878,7 +17862,7 @@
         <v>1289</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="C36" s="15" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
feat: add solid Toggle variant
</commit_message>
<xml_diff>
--- a/playground/component-coverage.xlsx
+++ b/playground/component-coverage.xlsx
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5160" uniqueCount="1420">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5159" uniqueCount="1420">
   <si>
     <t xml:space="preserve">Brick Component Coverage Index</t>
   </si>
@@ -2285,7 +2285,7 @@
     <t xml:space="preserve">TOG-07</t>
   </si>
   <si>
-    <t xml:space="preserve">Soft, outline, and ghost variants; sm/md/lg sizes; rounded/pill shapes; and icon-only geometry form closed recipes without tone or arbitrary radius</t>
+    <t xml:space="preserve">Solid, soft, outline, and ghost variants; sm/md/lg sizes; rounded/pill shapes; and icon-only geometry form closed recipes without tone or arbitrary radius</t>
   </si>
   <si>
     <t xml:space="preserve">TOG-08</t>
@@ -2486,265 +2486,265 @@
     <t xml:space="preserve">Latest owner run records every numbered Toggle and ToggleGroup result and corrects any finding before package completion</t>
   </si>
   <si>
+    <t xml:space="preserve">TOG-35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Public Toggle guide covers role boundaries, stable labels, behavior/native/ref contract, visual API, accessibility, CSS hooks, and preferences</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../docs/components/toggle/README.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Public ToggleGroup guide and both changelogs cover discriminated selection, naming, keyboard, separated/attached/full-width geometry, ownership, and evidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../docs/components/toggle-group/README.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Independent Consumer uses public Toggle and ToggleGroup subpaths for appearance and Cards/List view and passes production, boundary, desktop/mobile, state, layout, and axe checks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legacy Toggle family</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fresh searches found no live dependents; Core Toggle/ToggleGroup sources and input-barrel exports are removed and Core builds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOG-39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tone, generic Chip/Tag, required single-selection behavior, item-level recipe overrides, navigation, disclosure, and form-setting semantics remain deliberately excluded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IconButton Evidence Matrix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence gates for the adopted IconButton API, Atom-owned action/link behavior, package proof, Consumer integration, and non-applicable legacy slice retirement.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IconButton directly styles public Atom 0.3.3 Button.Root without Core, framework, or local behavior state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../src/components/icon-button/IconButton.tsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Owner-approved audit confirms IconButton is an icon-only Button specialization and no separate IconLink is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../../docs/icon-button-component-brief.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Root and icon-button subpath exports, declarations, direct component, closed recipes, and inherited native contracts match the adopted brief</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shortest action emits one native button with stable class/slot and ghost/neutral/md/rounded defaults</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../test/components/icon-button-app-bar.test.tsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semantics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every icon-only action requires an accessible name supplied by aria-label or aria-labelledby</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/icon-button-app-bar.spec.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Navigation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">href renders a genuine anchor and preserves target plus safe rel behavior through Atom Button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pointer, keyboard, onPress, disabled, loading, native props, composition, and refs remain Atom-owned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solid, soft, outline, and ghost variants form a closed presentation matrix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neutral, accent, info, success, warning, and danger tones use semantic Brick tokens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">xs through xl sizes retain square hit geometry and rounded/circle shapes without arbitrary radius</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Icon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The visual icon is presentation-only while the control name remains on the interactive element</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rest, hover, active, focus-visible, disabled, and loading recipes remain visibly distinct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loading retains the accessible name, exposes Atom busy state, and replaces only the visual icon with a spinner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Focus visibility, native disabled semantics, link semantics, and named controls pass real-browser and axe checks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Appearance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reviewed light and dark baselines preserve hierarchy and icon contrast across variants and tones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preferences</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forced-colors preserves boundaries and loading indication; reduced-motion slows spinner animation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Narrow mobile and RTL stress examples remain contained without changing square control geometry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">class, style, slot, scoped appearance, and documented component variables remain local and inspectable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compiled layered CSS uses Brick classes, logical properties, semantic tokens, and no global leakage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../src/components/icon-button/icon-button.css</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The /icon-button workbench exposes overview, variants, tones, sizes, shapes, disabled/loading/link states, mobile stress, and RTL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vitest covers defaults, recipes, links, events, disabled/loading behavior, composition, and refs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Public root/subpath types accept supported contracts and reject invalid variants, tones, sizes, and shapes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Node boundary, export identity, stylesheet, declarations, SSR, and dry-pack checks include the icon-button subpath</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clean packed React 18/19 consumers import, SSR-render, typecheck, and load IconButton CSS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strict typecheck, production build, CSS report, and 100% component-source coverage pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Focused browser checks cover action/link semantics, recipes, inactive states, mobile/RTL, axe, and forced colors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chromium, Firefox, WebKit, Pixel, and iPhone release-matrix checks pass where applicable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Four reviewed Chromium baselines cover variants, dark tones, forced-colors states, and mobile RTL stress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numbered protocol covers semantics, pointer/keyboard, link, recipes, states, zoom/mobile/RTL, VoiceOver, preferences, and customization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">manual-tests/icon-button-app-bar.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICB-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latest owner run records every numbered IconButton result and corrects any finding before package completion</t>
+  </si>
+  <si>
     <t xml:space="preserve">Owner manual review intentionally deferred</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Public Toggle guide covers role boundaries, stable labels, behavior/native/ref contract, visual API, accessibility, CSS hooks, and preferences</t>
-  </si>
-  <si>
-    <t xml:space="preserve">../docs/components/toggle/README.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Public ToggleGroup guide and both changelogs cover discriminated selection, naming, keyboard, separated/attached/full-width geometry, ownership, and evidence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">../docs/components/toggle-group/README.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-37</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Independent Consumer uses public Toggle and ToggleGroup subpaths for appearance and Cards/List view and passes production, boundary, desktop/mobile, state, layout, and axe checks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-38</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Legacy Toggle family</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fresh searches found no live dependents; Core Toggle/ToggleGroup sources and input-barrel exports are removed and Core builds</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOG-39</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tone, generic Chip/Tag, required single-selection behavior, item-level recipe overrides, navigation, disclosure, and form-setting semantics remain deliberately excluded</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IconButton Evidence Matrix</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evidence gates for the adopted IconButton API, Atom-owned action/link behavior, package proof, Consumer integration, and non-applicable legacy slice retirement.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IconButton directly styles public Atom 0.3.3 Button.Root without Core, framework, or local behavior state</t>
-  </si>
-  <si>
-    <t xml:space="preserve">../src/components/icon-button/IconButton.tsx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Owner-approved audit confirms IconButton is an icon-only Button specialization and no separate IconLink is required</t>
-  </si>
-  <si>
-    <t xml:space="preserve">../../docs/icon-button-component-brief.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Root and icon-button subpath exports, declarations, direct component, closed recipes, and inherited native contracts match the adopted brief</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shortest action emits one native button with stable class/slot and ghost/neutral/md/rounded defaults</t>
-  </si>
-  <si>
-    <t xml:space="preserve">../test/components/icon-button-app-bar.test.tsx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Semantics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Every icon-only action requires an accessible name supplied by aria-label or aria-labelledby</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tests/icon-button-app-bar.spec.ts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Navigation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">href renders a genuine anchor and preserves target plus safe rel behavior through Atom Button</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pointer, keyboard, onPress, disabled, loading, native props, composition, and refs remain Atom-owned</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solid, soft, outline, and ghost variants form a closed presentation matrix</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Neutral, accent, info, success, warning, and danger tones use semantic Brick tokens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">xs through xl sizes retain square hit geometry and rounded/circle shapes without arbitrary radius</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Icon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The visual icon is presentation-only while the control name remains on the interactive element</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rest, hover, active, focus-visible, disabled, and loading recipes remain visibly distinct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Loading retains the accessible name, exposes Atom busy state, and replaces only the visual icon with a spinner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Focus visibility, native disabled semantics, link semantics, and named controls pass real-browser and axe checks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Appearance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reviewed light and dark baselines preserve hierarchy and icon contrast across variants and tones</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preferences</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Forced-colors preserves boundaries and loading indication; reduced-motion slows spinner animation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Narrow mobile and RTL stress examples remain contained without changing square control geometry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">class, style, slot, scoped appearance, and documented component variables remain local and inspectable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compiled layered CSS uses Brick classes, logical properties, semantic tokens, and no global leakage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">../src/components/icon-button/icon-button.css</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The /icon-button workbench exposes overview, variants, tones, sizes, shapes, disabled/loading/link states, mobile stress, and RTL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vitest covers defaults, recipes, links, events, disabled/loading behavior, composition, and refs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Public root/subpath types accept supported contracts and reject invalid variants, tones, sizes, and shapes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node boundary, export identity, stylesheet, declarations, SSR, and dry-pack checks include the icon-button subpath</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clean packed React 18/19 consumers import, SSR-render, typecheck, and load IconButton CSS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strict typecheck, production build, CSS report, and 100% component-source coverage pass</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Focused browser checks cover action/link semantics, recipes, inactive states, mobile/RTL, axe, and forced colors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chromium, Firefox, WebKit, Pixel, and iPhone release-matrix checks pass where applicable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Four reviewed Chromium baselines cover variants, dark tones, forced-colors states, and mobile RTL stress</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Numbered protocol covers semantics, pointer/keyboard, link, recipes, states, zoom/mobile/RTL, VoiceOver, preferences, and customization</t>
-  </si>
-  <si>
-    <t xml:space="preserve">manual-tests/icon-button-app-bar.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICB-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Latest owner run records every numbered IconButton result and corrects any finding before package completion</t>
   </si>
   <si>
     <t xml:space="preserve">ICB-31</t>
@@ -5221,7 +5221,7 @@
       </c>
       <c r="D4" s="5" t="n">
         <f aca="false">COUNTIF(N8:N21,"complete")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>4</v>
@@ -5235,7 +5235,7 @@
       </c>
       <c r="H4" s="6" t="n">
         <f aca="false">IFERROR(SUMPRODUCT(B8:B21,J8:J21)/SUM(B8:B21),0)</f>
-        <v>0.916190476190476</v>
+        <v>0.918095238095238</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5695,7 +5695,7 @@
       </c>
       <c r="D15" s="8" t="n">
         <f aca="false">COUNTIF(Toggle!H9:H47,"partial")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" s="8" t="n">
         <f aca="false">COUNTIF(Toggle!H9:H47,"implemented")</f>
@@ -5707,7 +5707,7 @@
       </c>
       <c r="G15" s="8" t="n">
         <f aca="false">COUNTIF(Toggle!H9:H47,"verified")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H15" s="8" t="n">
         <f aca="false">COUNTIF(Toggle!H9:H47,"blocked")</f>
@@ -5719,11 +5719,11 @@
       </c>
       <c r="J15" s="9" t="n">
         <f aca="false">IFERROR(SUM(Toggle!M9:M47)/SUM(Toggle!L9:L47),0)</f>
-        <v>0.974358974358974</v>
+        <v>1</v>
       </c>
       <c r="K15" s="8" t="str">
         <f aca="false">IF(COUNTIFS(Toggle!E9:E47,"package",Toggle!M9:M47,"&lt;1")=0,"complete","open")</f>
-        <v>open</v>
+        <v>complete</v>
       </c>
       <c r="L15" s="8" t="str">
         <f aca="false">IF(COUNTIFS(Toggle!E9:E47,"consumer",Toggle!M9:M47,"&lt;1")=0,"complete","open")</f>
@@ -5735,7 +5735,7 @@
       </c>
       <c r="N15" s="1" t="str">
         <f aca="false">IF(H15&gt;0,"blocked",IF(AND(J15=1,K15="complete",L15="complete",M15="complete"),"complete",IF(J15=0,"not started","in progress")))</f>
-        <v>in progress</v>
+        <v>complete</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8013,14 +8013,14 @@
       </c>
       <c r="D4" s="5" t="n">
         <f aca="false">SUM(M9:M47)</f>
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F4" s="6" t="n">
         <f aca="false">IFERROR(D4/SUM(L9:L47),0)</f>
-        <v>0.974358974358974</v>
+        <v>1</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>4</v>
@@ -8034,7 +8034,7 @@
       </c>
       <c r="J4" s="5" t="str">
         <f aca="false">IF(COUNTIFS(E9:E47,"package",M9:M47,"&lt;1")=0,"complete","open")</f>
-        <v>open</v>
+        <v>complete</v>
       </c>
       <c r="K4" s="4" t="s">
         <v>17</v>
@@ -8371,7 +8371,7 @@
         <v>76</v>
       </c>
       <c r="J15" s="19" t="n">
-        <v>46221</v>
+        <v>46223</v>
       </c>
       <c r="K15" s="15"/>
       <c r="L15" s="18" t="n">
@@ -9445,26 +9445,26 @@
         <v>805</v>
       </c>
       <c r="H42" s="15" t="s">
-        <v>347</v>
+        <v>82</v>
       </c>
       <c r="I42" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="J42" s="19"/>
-      <c r="K42" s="15" t="s">
-        <v>808</v>
-      </c>
+      <c r="J42" s="19" t="n">
+        <v>46223</v>
+      </c>
+      <c r="K42" s="15"/>
       <c r="L42" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M42" s="18" t="n">
         <f aca="false">IF(H42="not applicable",IF(K42&lt;&gt;"",1,0),IF(I42="yes",IF(H42="verified",1,0),IF(OR(H42="tested",H42="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="15" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="B43" s="15" t="s">
         <v>145</v>
@@ -9473,7 +9473,7 @@
         <v>26</v>
       </c>
       <c r="D43" s="15" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="E43" s="15" t="s">
         <v>72</v>
@@ -9482,7 +9482,7 @@
         <v>147</v>
       </c>
       <c r="G43" s="16" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="H43" s="15" t="s">
         <v>75</v>
@@ -9504,7 +9504,7 @@
     </row>
     <row r="44" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="15" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="B44" s="15" t="s">
         <v>145</v>
@@ -9513,7 +9513,7 @@
         <v>757</v>
       </c>
       <c r="D44" s="15" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="E44" s="15" t="s">
         <v>72</v>
@@ -9522,7 +9522,7 @@
         <v>147</v>
       </c>
       <c r="G44" s="16" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="H44" s="15" t="s">
         <v>75</v>
@@ -9544,7 +9544,7 @@
     </row>
     <row r="45" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="15" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="B45" s="15" t="s">
         <v>153</v>
@@ -9553,7 +9553,7 @@
         <v>537</v>
       </c>
       <c r="D45" s="15" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="E45" s="15" t="s">
         <v>155</v>
@@ -9584,16 +9584,16 @@
     </row>
     <row r="46" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="15" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="B46" s="15" t="s">
         <v>158</v>
       </c>
       <c r="C46" s="15" t="s">
+        <v>817</v>
+      </c>
+      <c r="D46" s="15" t="s">
         <v>818</v>
-      </c>
-      <c r="D46" s="15" t="s">
-        <v>819</v>
       </c>
       <c r="E46" s="15" t="s">
         <v>160</v>
@@ -9624,7 +9624,7 @@
     </row>
     <row r="47" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="15" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="B47" s="15" t="s">
         <v>626</v>
@@ -9633,7 +9633,7 @@
         <v>537</v>
       </c>
       <c r="D47" s="15" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="E47" s="15" t="s">
         <v>72</v>
@@ -9777,7 +9777,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -9794,7 +9794,7 @@
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -9913,7 +9913,7 @@
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="B9" s="15" t="s">
         <v>70</v>
@@ -9922,7 +9922,7 @@
         <v>27</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="E9" s="15" t="s">
         <v>72</v>
@@ -9931,7 +9931,7 @@
         <v>73</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="H9" s="15" t="s">
         <v>75</v>
@@ -9953,7 +9953,7 @@
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="B10" s="15" t="s">
         <v>78</v>
@@ -9962,7 +9962,7 @@
         <v>27</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="E10" s="15" t="s">
         <v>72</v>
@@ -9971,7 +9971,7 @@
         <v>80</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="H10" s="15" t="s">
         <v>82</v>
@@ -9993,7 +9993,7 @@
     </row>
     <row r="11" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="B11" s="15" t="s">
         <v>70</v>
@@ -10002,7 +10002,7 @@
         <v>27</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="E11" s="15" t="s">
         <v>72</v>
@@ -10033,7 +10033,7 @@
     </row>
     <row r="12" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="B12" s="15" t="s">
         <v>50</v>
@@ -10042,7 +10042,7 @@
         <v>27</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="E12" s="15" t="s">
         <v>72</v>
@@ -10051,7 +10051,7 @@
         <v>120</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="H12" s="15" t="s">
         <v>75</v>
@@ -10073,16 +10073,16 @@
     </row>
     <row r="13" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
+        <v>834</v>
+      </c>
+      <c r="B13" s="15" t="s">
         <v>835</v>
-      </c>
-      <c r="B13" s="15" t="s">
-        <v>836</v>
       </c>
       <c r="C13" s="15" t="s">
         <v>27</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="E13" s="15" t="s">
         <v>72</v>
@@ -10091,7 +10091,7 @@
         <v>120</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="H13" s="15" t="s">
         <v>75</v>
@@ -10113,16 +10113,16 @@
     </row>
     <row r="14" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
+        <v>838</v>
+      </c>
+      <c r="B14" s="15" t="s">
         <v>839</v>
-      </c>
-      <c r="B14" s="15" t="s">
-        <v>840</v>
       </c>
       <c r="C14" s="15" t="s">
         <v>27</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="E14" s="15" t="s">
         <v>72</v>
@@ -10131,7 +10131,7 @@
         <v>120</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="H14" s="15" t="s">
         <v>75</v>
@@ -10153,7 +10153,7 @@
     </row>
     <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>736</v>
@@ -10162,7 +10162,7 @@
         <v>27</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="E15" s="15" t="s">
         <v>72</v>
@@ -10171,7 +10171,7 @@
         <v>120</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="H15" s="15" t="s">
         <v>75</v>
@@ -10193,7 +10193,7 @@
     </row>
     <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="B16" s="15" t="s">
         <v>92</v>
@@ -10202,7 +10202,7 @@
         <v>27</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="E16" s="15" t="s">
         <v>72</v>
@@ -10233,7 +10233,7 @@
     </row>
     <row r="17" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="B17" s="15" t="s">
         <v>92</v>
@@ -10242,7 +10242,7 @@
         <v>27</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="E17" s="15" t="s">
         <v>72</v>
@@ -10273,7 +10273,7 @@
     </row>
     <row r="18" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="15" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="B18" s="15" t="s">
         <v>561</v>
@@ -10282,7 +10282,7 @@
         <v>27</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="E18" s="15" t="s">
         <v>72</v>
@@ -10291,7 +10291,7 @@
         <v>120</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="H18" s="15" t="s">
         <v>75</v>
@@ -10313,16 +10313,16 @@
     </row>
     <row r="19" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
+        <v>849</v>
+      </c>
+      <c r="B19" s="15" t="s">
         <v>850</v>
-      </c>
-      <c r="B19" s="15" t="s">
-        <v>851</v>
       </c>
       <c r="C19" s="15" t="s">
         <v>27</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="E19" s="15" t="s">
         <v>72</v>
@@ -10331,7 +10331,7 @@
         <v>120</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="H19" s="15" t="s">
         <v>75</v>
@@ -10353,7 +10353,7 @@
     </row>
     <row r="20" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="B20" s="15" t="s">
         <v>743</v>
@@ -10362,7 +10362,7 @@
         <v>27</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="E20" s="15" t="s">
         <v>72</v>
@@ -10393,7 +10393,7 @@
     </row>
     <row r="21" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="B21" s="15" t="s">
         <v>649</v>
@@ -10402,7 +10402,7 @@
         <v>27</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="E21" s="15" t="s">
         <v>72</v>
@@ -10411,7 +10411,7 @@
         <v>120</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="H21" s="15" t="s">
         <v>75</v>
@@ -10433,7 +10433,7 @@
     </row>
     <row r="22" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>550</v>
@@ -10442,7 +10442,7 @@
         <v>27</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="E22" s="15" t="s">
         <v>72</v>
@@ -10451,7 +10451,7 @@
         <v>120</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="H22" s="15" t="s">
         <v>75</v>
@@ -10473,16 +10473,16 @@
     </row>
     <row r="23" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="s">
+        <v>858</v>
+      </c>
+      <c r="B23" s="15" t="s">
         <v>859</v>
-      </c>
-      <c r="B23" s="15" t="s">
-        <v>860</v>
       </c>
       <c r="C23" s="15" t="s">
         <v>27</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="E23" s="15" t="s">
         <v>72</v>
@@ -10513,16 +10513,16 @@
     </row>
     <row r="24" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
+        <v>861</v>
+      </c>
+      <c r="B24" s="15" t="s">
         <v>862</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>863</v>
       </c>
       <c r="C24" s="15" t="s">
         <v>27</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="E24" s="15" t="s">
         <v>72</v>
@@ -10531,7 +10531,7 @@
         <v>120</v>
       </c>
       <c r="G24" s="16" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="H24" s="15" t="s">
         <v>75</v>
@@ -10553,7 +10553,7 @@
     </row>
     <row r="25" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="B25" s="15" t="s">
         <v>779</v>
@@ -10562,7 +10562,7 @@
         <v>27</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="E25" s="15" t="s">
         <v>72</v>
@@ -10571,7 +10571,7 @@
         <v>120</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="H25" s="15" t="s">
         <v>75</v>
@@ -10593,7 +10593,7 @@
     </row>
     <row r="26" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="B26" s="15" t="s">
         <v>581</v>
@@ -10602,7 +10602,7 @@
         <v>27</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="E26" s="15" t="s">
         <v>72</v>
@@ -10633,7 +10633,7 @@
     </row>
     <row r="27" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="B27" s="15" t="s">
         <v>92</v>
@@ -10642,7 +10642,7 @@
         <v>27</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="E27" s="15" t="s">
         <v>72</v>
@@ -10651,7 +10651,7 @@
         <v>73</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="H27" s="15" t="s">
         <v>75</v>
@@ -10673,7 +10673,7 @@
     </row>
     <row r="28" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="15" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="B28" s="15" t="s">
         <v>99</v>
@@ -10682,7 +10682,7 @@
         <v>27</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="E28" s="15" t="s">
         <v>72</v>
@@ -10713,7 +10713,7 @@
     </row>
     <row r="29" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="B29" s="15" t="s">
         <v>118</v>
@@ -10722,7 +10722,7 @@
         <v>27</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="E29" s="15" t="s">
         <v>72</v>
@@ -10731,7 +10731,7 @@
         <v>120</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="H29" s="15" t="s">
         <v>75</v>
@@ -10753,7 +10753,7 @@
     </row>
     <row r="30" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="15" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="B30" s="15" t="s">
         <v>118</v>
@@ -10762,7 +10762,7 @@
         <v>27</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="E30" s="15" t="s">
         <v>72</v>
@@ -10793,7 +10793,7 @@
     </row>
     <row r="31" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="15" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="B31" s="15" t="s">
         <v>118</v>
@@ -10802,7 +10802,7 @@
         <v>27</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="E31" s="15" t="s">
         <v>72</v>
@@ -10833,7 +10833,7 @@
     </row>
     <row r="32" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="15" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="B32" s="15" t="s">
         <v>118</v>
@@ -10842,7 +10842,7 @@
         <v>27</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="E32" s="15" t="s">
         <v>72</v>
@@ -10873,7 +10873,7 @@
     </row>
     <row r="33" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="15" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="B33" s="15" t="s">
         <v>118</v>
@@ -10882,7 +10882,7 @@
         <v>27</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="E33" s="15" t="s">
         <v>72</v>
@@ -10891,7 +10891,7 @@
         <v>120</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="H33" s="15" t="s">
         <v>75</v>
@@ -10913,7 +10913,7 @@
     </row>
     <row r="34" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="15" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="B34" s="15" t="s">
         <v>118</v>
@@ -10922,7 +10922,7 @@
         <v>27</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="E34" s="15" t="s">
         <v>72</v>
@@ -10931,7 +10931,7 @@
         <v>120</v>
       </c>
       <c r="G34" s="16" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="H34" s="15" t="s">
         <v>75</v>
@@ -10953,7 +10953,7 @@
     </row>
     <row r="35" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="15" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="B35" s="15" t="s">
         <v>118</v>
@@ -10962,7 +10962,7 @@
         <v>27</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="E35" s="15" t="s">
         <v>72</v>
@@ -10993,7 +10993,7 @@
     </row>
     <row r="36" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="15" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="B36" s="15" t="s">
         <v>118</v>
@@ -11002,7 +11002,7 @@
         <v>27</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="E36" s="15" t="s">
         <v>72</v>
@@ -11033,7 +11033,7 @@
     </row>
     <row r="37" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="15" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="B37" s="15" t="s">
         <v>139</v>
@@ -11042,7 +11042,7 @@
         <v>27</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="E37" s="15" t="s">
         <v>72</v>
@@ -11051,7 +11051,7 @@
         <v>141</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="H37" s="15" t="s">
         <v>75</v>
@@ -11073,7 +11073,7 @@
     </row>
     <row r="38" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="15" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="B38" s="15" t="s">
         <v>139</v>
@@ -11082,7 +11082,7 @@
         <v>27</v>
       </c>
       <c r="D38" s="15" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="E38" s="15" t="s">
         <v>72</v>
@@ -11091,7 +11091,7 @@
         <v>141</v>
       </c>
       <c r="G38" s="16" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="H38" s="15" t="s">
         <v>347</v>
@@ -11103,7 +11103,7 @@
         <v>46221</v>
       </c>
       <c r="K38" s="15" t="s">
-        <v>808</v>
+        <v>894</v>
       </c>
       <c r="L38" s="18" t="n">
         <v>1</v>
@@ -11265,7 +11265,7 @@
         <v>46221</v>
       </c>
       <c r="K42" s="15" t="s">
-        <v>808</v>
+        <v>894</v>
       </c>
       <c r="L42" s="18" t="n">
         <v>1</v>
@@ -11337,7 +11337,7 @@
         <v>80</v>
       </c>
       <c r="G44" s="16" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="H44" s="15" t="s">
         <v>82</v>
@@ -11866,7 +11866,7 @@
         <v>120</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="H12" s="15" t="s">
         <v>75</v>
@@ -11906,7 +11906,7 @@
         <v>120</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="H13" s="15" t="s">
         <v>75</v>
@@ -11946,7 +11946,7 @@
         <v>120</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="H14" s="15" t="s">
         <v>75</v>
@@ -11986,7 +11986,7 @@
         <v>120</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="H15" s="15" t="s">
         <v>75</v>
@@ -12026,7 +12026,7 @@
         <v>120</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="H16" s="15" t="s">
         <v>75</v>
@@ -12066,7 +12066,7 @@
         <v>120</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="H17" s="15" t="s">
         <v>75</v>
@@ -12106,7 +12106,7 @@
         <v>120</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="H18" s="15" t="s">
         <v>75</v>
@@ -12146,7 +12146,7 @@
         <v>120</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="H19" s="15" t="s">
         <v>75</v>
@@ -12186,7 +12186,7 @@
         <v>120</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="H20" s="15" t="s">
         <v>75</v>
@@ -12226,7 +12226,7 @@
         <v>120</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="H21" s="15" t="s">
         <v>75</v>
@@ -12426,7 +12426,7 @@
         <v>120</v>
       </c>
       <c r="G26" s="16" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="H26" s="15" t="s">
         <v>75</v>
@@ -12466,7 +12466,7 @@
         <v>120</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="H27" s="15" t="s">
         <v>75</v>
@@ -12506,7 +12506,7 @@
         <v>120</v>
       </c>
       <c r="G28" s="16" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="H28" s="15" t="s">
         <v>75</v>
@@ -12531,7 +12531,7 @@
         <v>973</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="C29" s="15" t="s">
         <v>28</v>
@@ -12706,7 +12706,7 @@
         <v>120</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="H33" s="15" t="s">
         <v>75</v>
@@ -12857,7 +12857,7 @@
         <v>28</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="E37" s="15" t="s">
         <v>72</v>
@@ -12866,7 +12866,7 @@
         <v>120</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="H37" s="15" t="s">
         <v>75</v>
@@ -12906,7 +12906,7 @@
         <v>120</v>
       </c>
       <c r="G38" s="16" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="H38" s="15" t="s">
         <v>75</v>
@@ -12937,7 +12937,7 @@
         <v>28</v>
       </c>
       <c r="D39" s="15" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="E39" s="15" t="s">
         <v>72</v>
@@ -13026,7 +13026,7 @@
         <v>141</v>
       </c>
       <c r="G41" s="16" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="H41" s="15" t="s">
         <v>75</v>
@@ -13066,7 +13066,7 @@
         <v>141</v>
       </c>
       <c r="G42" s="16" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="H42" s="15" t="s">
         <v>347</v>
@@ -13076,7 +13076,7 @@
       </c>
       <c r="J42" s="19"/>
       <c r="K42" s="15" t="s">
-        <v>808</v>
+        <v>894</v>
       </c>
       <c r="L42" s="18" t="n">
         <v>1</v>
@@ -14020,7 +14020,7 @@
         <v>1044</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="C21" s="15" t="s">
         <v>269</v>
@@ -14060,7 +14060,7 @@
         <v>1048</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="C22" s="15" t="s">
         <v>197</v>
@@ -14266,7 +14266,7 @@
         <v>1063</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="C27" s="15" t="s">
         <v>197</v>
@@ -14308,7 +14308,7 @@
         <v>1067</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="C28" s="15" t="s">
         <v>197</v>
@@ -14350,7 +14350,7 @@
         <v>1069</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="C29" s="15" t="s">
         <v>1042</v>
@@ -14596,7 +14596,7 @@
         <v>1085</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="C35" s="15" t="s">
         <v>29</v>
@@ -14905,7 +14905,7 @@
         <v>46222</v>
       </c>
       <c r="K42" s="15" t="s">
-        <v>808</v>
+        <v>894</v>
       </c>
       <c r="L42" s="18" t="n">
         <v>1</v>
@@ -15702,7 +15702,7 @@
         <v>1152</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="C18" s="15" t="s">
         <v>269</v>
@@ -15742,7 +15742,7 @@
         <v>1155</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="C19" s="15" t="s">
         <v>197</v>
@@ -15782,7 +15782,7 @@
         <v>1157</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="C20" s="15" t="s">
         <v>197</v>
@@ -16068,7 +16068,7 @@
         <v>1174</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="C27" s="15" t="s">
         <v>197</v>
@@ -16110,7 +16110,7 @@
         <v>1177</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="C28" s="15" t="s">
         <v>197</v>
@@ -16152,7 +16152,7 @@
         <v>1179</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="C29" s="15" t="s">
         <v>1042</v>
@@ -16360,7 +16360,7 @@
         <v>1189</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="C34" s="15" t="s">
         <v>30</v>
@@ -16713,7 +16713,7 @@
         <v>46222</v>
       </c>
       <c r="K42" s="15" t="s">
-        <v>808</v>
+        <v>894</v>
       </c>
       <c r="L42" s="18" t="n">
         <v>1</v>
@@ -17752,7 +17752,7 @@
         <v>1258</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="C24" s="15" t="s">
         <v>197</v>
@@ -17792,7 +17792,7 @@
         <v>1261</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="C25" s="15" t="s">
         <v>183</v>
@@ -18032,7 +18032,7 @@
         <v>1278</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="C31" s="15" t="s">
         <v>197</v>
@@ -18072,7 +18072,7 @@
         <v>1280</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="C32" s="15" t="s">
         <v>197</v>
@@ -18114,7 +18114,7 @@
         <v>1283</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="C33" s="15" t="s">
         <v>1042</v>
@@ -18280,7 +18280,7 @@
         <v>1292</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="C37" s="15" t="s">
         <v>31</v>
@@ -19502,7 +19502,7 @@
         <v>1356</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="C23" s="15" t="s">
         <v>1332</v>
@@ -19542,7 +19542,7 @@
         <v>1358</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="C24" s="15" t="s">
         <v>1335</v>
@@ -19742,7 +19742,7 @@
         <v>1369</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="C29" s="15" t="s">
         <v>1318</v>
@@ -20348,7 +20348,7 @@
         <v>1408</v>
       </c>
       <c r="B44" s="15" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="C44" s="15" t="s">
         <v>1318</v>

</xml_diff>

<commit_message>
Complete Brick form foundation review
</commit_message>
<xml_diff>
--- a/playground/component-coverage.xlsx
+++ b/playground/component-coverage.xlsx
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5132" uniqueCount="1423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5132" uniqueCount="1421">
   <si>
     <t xml:space="preserve">Brick Component Coverage Index</t>
   </si>
@@ -4253,52 +4253,46 @@
     <t xml:space="preserve">FFB-32</t>
   </si>
   <si>
-    <t xml:space="preserve">Nine-section workbench covers APIs, models, state, reflow, groups, composition, appearance, relationships, and stress</t>
+    <t xml:space="preserve">Nine-scenario workbench separates Form, Field, and Fieldset review sections plus shared integration, composition, appearance, relationships, and stress evidence</t>
   </si>
   <si>
     <t xml:space="preserve">FFB-33</t>
   </si>
   <si>
-    <t xml:space="preserve">Numbered visual, keyboard, touch, screen-reader, zoom, direction, preference, composition, and Consumer protocol has an owner run</t>
+    <t xml:space="preserve">Fourteen-step owner protocol has dedicated Form, Field, and Fieldset sections plus foundation integration checks</t>
   </si>
   <si>
     <t xml:space="preserve">../../docs/manual-tests/form-foundation.md</t>
   </si>
   <si>
-    <t xml:space="preserve">Owner run pending</t>
+    <t xml:space="preserve">Owner protocol passed July 21, 2026; Windows forced colors not tested (no device)</t>
   </si>
   <si>
     <t xml:space="preserve">FFB-34</t>
   </si>
   <si>
-    <t xml:space="preserve">Visual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Owner approves finished hierarchy, disabled/read-only distinction, error presentation, responsive reflow, and control alignment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Owner visual review pending</t>
+    <t xml:space="preserve">Owner approves native submission models, callback state, reset, keyboard/touch behavior, and visible feedback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Owner Form review passed July 21, 2026</t>
   </si>
   <si>
     <t xml:space="preserve">FFB-35</t>
   </si>
   <si>
-    <t xml:space="preserve">Mobile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Physical touch label activation, 200%/400% reflow, and mobile screen-reader behavior are owner-approved</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Owner mobile and zoom review pending</t>
+    <t xml:space="preserve">Owner approves one-control anatomy, states, relationships, orientation, composition, touch, screen-reader, and zoom behavior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Owner Field review passed July 21, 2026</t>
   </si>
   <si>
     <t xml:space="preserve">FFB-36</t>
   </si>
   <si>
-    <t xml:space="preserve">Reduced motion and forced colors/Windows High Contrast boundaries are owner-approved where available</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Owner preference review pending</t>
+    <t xml:space="preserve">Owner approves native group anatomy, states, relationships, composition, choice interaction, direction, and preferences where available</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Owner Fieldset review passed July 21, 2026; Windows forced colors not tested (no device)</t>
   </si>
   <si>
     <t xml:space="preserve">FFB-37</t>
@@ -5260,7 +5254,7 @@
       </c>
       <c r="H4" s="6" t="n">
         <f aca="false">IFERROR(SUMPRODUCT(B8:B21,J8:J21)/SUM(B8:B21),0)</f>
-        <v>0.975238095238095</v>
+        <v>0.982857142857143</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6062,7 +6056,7 @@
       </c>
       <c r="D21" s="8" t="n">
         <f aca="false">COUNTIF('Form Foundation'!H9:H47,"partial")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E21" s="8" t="n">
         <f aca="false">COUNTIF('Form Foundation'!H9:H47,"implemented")</f>
@@ -6074,7 +6068,7 @@
       </c>
       <c r="G21" s="8" t="n">
         <f aca="false">COUNTIF('Form Foundation'!H9:H47,"verified")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H21" s="8" t="n">
         <f aca="false">COUNTIF('Form Foundation'!H9:H47,"blocked")</f>
@@ -6086,11 +6080,11 @@
       </c>
       <c r="J21" s="9" t="n">
         <f aca="false">IFERROR(SUM('Form Foundation'!M9:M47)/SUM('Form Foundation'!L9:L47),0)</f>
-        <v>0.871794871794872</v>
+        <v>0.974358974358974</v>
       </c>
       <c r="K21" s="8" t="str">
         <f aca="false">IF(COUNTIFS('Form Foundation'!E9:E47,"package",'Form Foundation'!M9:M47,"&lt;1")=0,"complete","open")</f>
-        <v>open</v>
+        <v>complete</v>
       </c>
       <c r="L21" s="8" t="str">
         <f aca="false">IF(COUNTIFS('Form Foundation'!E9:E47,"consumer",'Form Foundation'!M9:M47,"&lt;1")=0,"complete","open")</f>
@@ -18821,14 +18815,14 @@
       </c>
       <c r="D4" s="5" t="n">
         <f aca="false">SUM(M9:M47)</f>
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F4" s="6" t="n">
         <f aca="false">IFERROR(D4/SUM(L9:L47),0)</f>
-        <v>0.871794871794872</v>
+        <v>0.974358974358974</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>4</v>
@@ -18842,7 +18836,7 @@
       </c>
       <c r="J4" s="5" t="str">
         <f aca="false">IF(COUNTIFS(E9:E47,"package",M9:M47,"&lt;1")=0,"complete","open")</f>
-        <v>open</v>
+        <v>complete</v>
       </c>
       <c r="K4" s="4" t="s">
         <v>17</v>
@@ -20213,13 +20207,13 @@
         <v>1400</v>
       </c>
       <c r="H41" s="15" t="s">
-        <v>347</v>
+        <v>82</v>
       </c>
       <c r="I41" s="15" t="s">
         <v>83</v>
       </c>
       <c r="J41" s="19" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="K41" s="15" t="s">
         <v>1401</v>
@@ -20229,7 +20223,7 @@
       </c>
       <c r="M41" s="18" t="n">
         <f aca="false">IF(H41="not applicable",IF(K41&lt;&gt;"",1,0),IF(I41="yes",IF(H41="verified",1,0),IF(OR(H41="tested",H41="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20237,13 +20231,13 @@
         <v>1402</v>
       </c>
       <c r="B42" s="15" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C42" s="15" t="s">
+        <v>1328</v>
+      </c>
+      <c r="D42" s="15" t="s">
         <v>1403</v>
-      </c>
-      <c r="C42" s="15" t="s">
-        <v>1318</v>
-      </c>
-      <c r="D42" s="15" t="s">
-        <v>1404</v>
       </c>
       <c r="E42" s="15" t="s">
         <v>72</v>
@@ -20255,37 +20249,37 @@
         <v>1400</v>
       </c>
       <c r="H42" s="15" t="s">
-        <v>347</v>
+        <v>82</v>
       </c>
       <c r="I42" s="15" t="s">
         <v>83</v>
       </c>
       <c r="J42" s="19" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="K42" s="15" t="s">
-        <v>1405</v>
+        <v>1404</v>
       </c>
       <c r="L42" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M42" s="18" t="n">
         <f aca="false">IF(H42="not applicable",IF(K42&lt;&gt;"",1,0),IF(I42="yes",IF(H42="verified",1,0),IF(OR(H42="tested",H42="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="15" t="s">
+        <v>1405</v>
+      </c>
+      <c r="B43" s="15" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C43" s="15" t="s">
+        <v>1332</v>
+      </c>
+      <c r="D43" s="15" t="s">
         <v>1406</v>
-      </c>
-      <c r="B43" s="15" t="s">
-        <v>1407</v>
-      </c>
-      <c r="C43" s="15" t="s">
-        <v>1318</v>
-      </c>
-      <c r="D43" s="15" t="s">
-        <v>1408</v>
       </c>
       <c r="E43" s="15" t="s">
         <v>72</v>
@@ -20297,37 +20291,37 @@
         <v>1400</v>
       </c>
       <c r="H43" s="15" t="s">
-        <v>347</v>
+        <v>82</v>
       </c>
       <c r="I43" s="15" t="s">
         <v>83</v>
       </c>
       <c r="J43" s="19" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="K43" s="15" t="s">
-        <v>1409</v>
+        <v>1407</v>
       </c>
       <c r="L43" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M43" s="18" t="n">
         <f aca="false">IF(H43="not applicable",IF(K43&lt;&gt;"",1,0),IF(I43="yes",IF(H43="verified",1,0),IF(OR(H43="tested",H43="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="15" t="s">
-        <v>1410</v>
+        <v>1408</v>
       </c>
       <c r="B44" s="15" t="s">
-        <v>862</v>
+        <v>1105</v>
       </c>
       <c r="C44" s="15" t="s">
-        <v>1318</v>
+        <v>1335</v>
       </c>
       <c r="D44" s="15" t="s">
-        <v>1411</v>
+        <v>1409</v>
       </c>
       <c r="E44" s="15" t="s">
         <v>72</v>
@@ -20339,28 +20333,28 @@
         <v>1400</v>
       </c>
       <c r="H44" s="15" t="s">
-        <v>347</v>
+        <v>82</v>
       </c>
       <c r="I44" s="15" t="s">
         <v>83</v>
       </c>
       <c r="J44" s="19" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="K44" s="15" t="s">
-        <v>1412</v>
+        <v>1410</v>
       </c>
       <c r="L44" s="18" t="n">
         <v>1</v>
       </c>
       <c r="M44" s="18" t="n">
         <f aca="false">IF(H44="not applicable",IF(K44&lt;&gt;"",1,0),IF(I44="yes",IF(H44="verified",1,0),IF(OR(H44="tested",H44="verified"),1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="15" t="s">
-        <v>1413</v>
+        <v>1411</v>
       </c>
       <c r="B45" s="15" t="s">
         <v>153</v>
@@ -20369,7 +20363,7 @@
         <v>1318</v>
       </c>
       <c r="D45" s="15" t="s">
-        <v>1414</v>
+        <v>1412</v>
       </c>
       <c r="E45" s="15" t="s">
         <v>155</v>
@@ -20400,7 +20394,7 @@
     </row>
     <row r="46" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="15" t="s">
-        <v>1415</v>
+        <v>1413</v>
       </c>
       <c r="B46" s="15" t="s">
         <v>158</v>
@@ -20409,13 +20403,13 @@
         <v>1328</v>
       </c>
       <c r="D46" s="15" t="s">
-        <v>1416</v>
+        <v>1414</v>
       </c>
       <c r="E46" s="15" t="s">
         <v>160</v>
       </c>
       <c r="F46" s="15" t="s">
-        <v>1417</v>
+        <v>1415</v>
       </c>
       <c r="G46" s="16" t="s">
         <v>252</v>
@@ -20430,7 +20424,7 @@
         <v>46223</v>
       </c>
       <c r="K46" s="15" t="s">
-        <v>1418</v>
+        <v>1416</v>
       </c>
       <c r="L46" s="18" t="n">
         <v>1</v>
@@ -20442,16 +20436,16 @@
     </row>
     <row r="47" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="15" t="s">
-        <v>1419</v>
+        <v>1417</v>
       </c>
       <c r="B47" s="15" t="s">
         <v>158</v>
       </c>
       <c r="C47" s="15" t="s">
-        <v>1420</v>
+        <v>1418</v>
       </c>
       <c r="D47" s="15" t="s">
-        <v>1421</v>
+        <v>1419</v>
       </c>
       <c r="E47" s="15" t="s">
         <v>160</v>
@@ -20472,7 +20466,7 @@
         <v>46223</v>
       </c>
       <c r="K47" s="15" t="s">
-        <v>1422</v>
+        <v>1420</v>
       </c>
       <c r="L47" s="18" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
feat: add Code and Code Block components
</commit_message>
<xml_diff>
--- a/playground/component-coverage.xlsx
+++ b/playground/component-coverage.xlsx
@@ -39,9 +39,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Surface" sheetId="30" state="visible" r:id="rId30"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Divider" sheetId="31" state="visible" r:id="rId31"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scroll Area" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Block" sheetId="34" state="visible" r:id="rId34"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$7:$M$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$7:$M$38</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Index'!$A$1:$M$35</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001" forceFullCalc="1"/>
@@ -1098,7 +1100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="24.71" customWidth="1" style="23" min="1" max="1"/>
@@ -1117,7 +1119,7 @@
     <row r="2" ht="27.75" customHeight="1" s="17">
       <c r="A2" s="19" t="inlineStr">
         <is>
-          <t>Current package evidence across 29 independently exported components.</t>
+          <t>Current package evidence across 31 independently exported components.</t>
         </is>
       </c>
     </row>
@@ -2766,7 +2768,7 @@
         <v/>
       </c>
     </row>
-    <row r="36">
+    <row r="36" s="17">
       <c r="A36" s="23" t="inlineStr">
         <is>
           <t>Scroll Area</t>
@@ -2821,8 +2823,118 @@
         <v/>
       </c>
     </row>
+    <row r="37" s="17">
+      <c r="A37" s="23" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="B37" s="23">
+        <f>INDIRECT("'"&amp;A37&amp;"'!B4")</f>
+        <v/>
+      </c>
+      <c r="C37" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A37&amp;"'!H9:H200"),"not started")</f>
+        <v/>
+      </c>
+      <c r="D37" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A37&amp;"'!H9:H200"),"partial")</f>
+        <v/>
+      </c>
+      <c r="E37" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A37&amp;"'!H9:H200"),"implemented")</f>
+        <v/>
+      </c>
+      <c r="F37" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A37&amp;"'!H9:H200"),"tested")</f>
+        <v/>
+      </c>
+      <c r="G37" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A37&amp;"'!H9:H200"),"verified")</f>
+        <v/>
+      </c>
+      <c r="H37" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A37&amp;"'!H9:H200"),"blocked")</f>
+        <v/>
+      </c>
+      <c r="I37" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A37&amp;"'!H9:H200"),"not applicable")</f>
+        <v/>
+      </c>
+      <c r="J37" s="24">
+        <f>INDIRECT("'"&amp;A37&amp;"'!H4")</f>
+        <v/>
+      </c>
+      <c r="K37" s="23">
+        <f>INDIRECT("'"&amp;A37&amp;"'!K4")</f>
+        <v/>
+      </c>
+      <c r="L37" s="23">
+        <f>INDIRECT("'"&amp;A37&amp;"'!E5")</f>
+        <v/>
+      </c>
+      <c r="M37" s="23">
+        <f>IF(AND(J37=1,K37="complete",L37="complete"),"complete",IF(H37&gt;0,"blocked","open"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" s="17">
+      <c r="A38" s="23" t="inlineStr">
+        <is>
+          <t>Code Block</t>
+        </is>
+      </c>
+      <c r="B38" s="23">
+        <f>INDIRECT("'"&amp;A38&amp;"'!B4")</f>
+        <v/>
+      </c>
+      <c r="C38" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A38&amp;"'!H9:H200"),"not started")</f>
+        <v/>
+      </c>
+      <c r="D38" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A38&amp;"'!H9:H200"),"partial")</f>
+        <v/>
+      </c>
+      <c r="E38" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A38&amp;"'!H9:H200"),"implemented")</f>
+        <v/>
+      </c>
+      <c r="F38" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A38&amp;"'!H9:H200"),"tested")</f>
+        <v/>
+      </c>
+      <c r="G38" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A38&amp;"'!H9:H200"),"verified")</f>
+        <v/>
+      </c>
+      <c r="H38" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A38&amp;"'!H9:H200"),"blocked")</f>
+        <v/>
+      </c>
+      <c r="I38" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A38&amp;"'!H9:H200"),"not applicable")</f>
+        <v/>
+      </c>
+      <c r="J38" s="24">
+        <f>INDIRECT("'"&amp;A38&amp;"'!H4")</f>
+        <v/>
+      </c>
+      <c r="K38" s="23">
+        <f>INDIRECT("'"&amp;A38&amp;"'!K4")</f>
+        <v/>
+      </c>
+      <c r="L38" s="23">
+        <f>INDIRECT("'"&amp;A38&amp;"'!E5")</f>
+        <v/>
+      </c>
+      <c r="M38" s="23">
+        <f>IF(AND(J38=1,K38="complete",L38="complete"),"complete",IF(H38&gt;0,"blocked","open"))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A7:M34"/>
+  <autoFilter ref="A7:M38"/>
   <mergeCells count="2">
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A1:M1"/>
@@ -29513,6 +29625,2225 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:M25"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.71" customWidth="1" style="23" min="1" max="1"/>
+    <col width="15.71" customWidth="1" style="23" min="2" max="2"/>
+    <col width="18.71" customWidth="1" style="23" min="3" max="3"/>
+    <col width="58.71" customWidth="1" style="23" min="4" max="4"/>
+    <col width="14.71" customWidth="1" style="23" min="5" max="6"/>
+    <col width="50.71" customWidth="1" style="23" min="7" max="7"/>
+    <col width="17.71" customWidth="1" style="23" min="8" max="8"/>
+    <col width="14.71" customWidth="1" style="23" min="9" max="9"/>
+    <col width="14.71" customWidth="1" style="25" min="10" max="10"/>
+    <col width="42.71" customWidth="1" style="23" min="11" max="11"/>
+    <col width="10.71" customWidth="1" style="23" min="12" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="37.5" customHeight="1" s="17">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Code Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="27.75" customHeight="1" s="17">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Assertion-level inline semantics, recipes, browser, human-review, documentation, Consumer, and adoption evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="17.25" customHeight="1" s="17">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>Requirements</t>
+        </is>
+      </c>
+      <c r="B4" s="21">
+        <f>COUNTA(A9:A25)</f>
+        <v/>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="E4" s="21">
+        <f>SUM(M9:M25)</f>
+        <v/>
+      </c>
+      <c r="G4" s="20" t="inlineStr">
+        <is>
+          <t>Completion</t>
+        </is>
+      </c>
+      <c r="H4" s="22">
+        <f>IF(B4=0,0,E4/B4)</f>
+        <v/>
+      </c>
+      <c r="J4" s="20" t="inlineStr">
+        <is>
+          <t>Package gate</t>
+        </is>
+      </c>
+      <c r="K4" s="21">
+        <f>IF(COUNTIFS(E9:E25,"package",M9:M25,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="17.25" customHeight="1" s="17">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Manual review</t>
+        </is>
+      </c>
+      <c r="B5" s="21">
+        <f>IF(COUNTIFS(I9:I25,"yes",M9:M25,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>Consumer gate</t>
+        </is>
+      </c>
+      <c r="E5" s="21">
+        <f>IF(COUNTIFS(E9:E25,"consumer",M9:M25,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="17">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="inlineStr">
+        <is>
+          <t>Evidence type</t>
+        </is>
+      </c>
+      <c r="G8" s="23" t="inlineStr">
+        <is>
+          <t>Evidence / link</t>
+        </is>
+      </c>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>Human review?</t>
+        </is>
+      </c>
+      <c r="J8" s="25" t="inlineStr">
+        <is>
+          <t>Last verified</t>
+        </is>
+      </c>
+      <c r="K8" s="23" t="inlineStr">
+        <is>
+          <t>Blocker / N/A reason</t>
+        </is>
+      </c>
+      <c r="L8" s="23" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="M8" s="23" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="54" customHeight="1" s="17">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>CO-01</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="inlineStr">
+        <is>
+          <t>Native code host, refs, slots, classes, styles, and closed recipes render from one server-safe component.</t>
+        </is>
+      </c>
+      <c r="E9" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F9" s="26" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="G9" s="27" t="inlineStr">
+        <is>
+          <t>../src/components/code</t>
+        </is>
+      </c>
+      <c r="H9" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I9" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J9" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K9" s="27" t="n"/>
+      <c r="L9" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" s="26">
+        <f>IF(OR(AND(I9="yes",H9="verified"),AND(I9="no",OR(H9="tested",H9="verified")),AND(H9="not applicable",K9&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="54" customHeight="1" s="17">
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>CO-02</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>Exports</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>Root and Code subpath exports expose the runtime and every public type.</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F10" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="G10" s="27" t="inlineStr">
+        <is>
+          <t>../test/package/package.test.mjs; ../test/package/ssr.test.mjs</t>
+        </is>
+      </c>
+      <c r="H10" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I10" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J10" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K10" s="27" t="n"/>
+      <c r="L10" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" s="26">
+        <f>IF(OR(AND(I10="yes",H10="verified"),AND(I10="no",OR(H10="tested",H10="verified")),AND(H10="not applicable",K10&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1" s="17">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>CO-03</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>Types</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D11" s="27" t="inlineStr">
+        <is>
+          <t>Recipes, native attributes, content, and HTMLElement ref contracts type-check.</t>
+        </is>
+      </c>
+      <c r="E11" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F11" s="26" t="inlineStr">
+        <is>
+          <t>types</t>
+        </is>
+      </c>
+      <c r="G11" s="27" t="inlineStr">
+        <is>
+          <t>../test/types/components/code.test.ts</t>
+        </is>
+      </c>
+      <c r="H11" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I11" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J11" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K11" s="27" t="n"/>
+      <c r="L11" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" s="26">
+        <f>IF(OR(AND(I11="yes",H11="verified"),AND(I11="no",OR(H11="tested",H11="verified")),AND(H11="not applicable",K11&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="54" customHeight="1" s="17">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>CO-04</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>CSS</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D12" s="27" t="inlineStr">
+        <is>
+          <t>Static CSS ships inline recipes, wrapping, forced colors, and public variables.</t>
+        </is>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="inlineStr">
+        <is>
+          <t>css</t>
+        </is>
+      </c>
+      <c r="G12" s="27" t="inlineStr">
+        <is>
+          <t>../src/components/code/code.css</t>
+        </is>
+      </c>
+      <c r="H12" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I12" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J12" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K12" s="27" t="n"/>
+      <c r="L12" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" s="26">
+        <f>IF(OR(AND(I12="yes",H12="verified"),AND(I12="no",OR(H12="tested",H12="verified")),AND(H12="not applicable",K12&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="54" customHeight="1" s="17">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>CO-05</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D13" s="27" t="inlineStr">
+        <is>
+          <t>Defaults, recipes, native forwarding, ref, events, and semantic host pass focused tests.</t>
+        </is>
+      </c>
+      <c r="E13" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F13" s="26" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="G13" s="27" t="inlineStr">
+        <is>
+          <t>../test/components/code/code.test.tsx</t>
+        </is>
+      </c>
+      <c r="H13" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I13" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J13" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K13" s="27" t="n"/>
+      <c r="L13" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" s="26">
+        <f>IF(OR(AND(I13="yes",H13="verified"),AND(I13="no",OR(H13="tested",H13="verified")),AND(H13="not applicable",K13&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="54" customHeight="1" s="17">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>CO-06</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>Browser</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>Inline context, native output, wrapping, RTL, zoom, and focus neutrality pass.</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F14" s="26" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+      <c r="G14" s="27" t="inlineStr">
+        <is>
+          <t>tests/components/code/behavior.spec.ts</t>
+        </is>
+      </c>
+      <c r="H14" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I14" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J14" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K14" s="27" t="n"/>
+      <c r="L14" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" s="26">
+        <f>IF(OR(AND(I14="yes",H14="verified"),AND(I14="no",OR(H14="tested",H14="verified")),AND(H14="not applicable",K14&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="54" customHeight="1" s="17">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>CO-07</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D15" s="27" t="inlineStr">
+        <is>
+          <t>Native semantics, meaningful prose context, text spacing, and axe remain correct.</t>
+        </is>
+      </c>
+      <c r="E15" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F15" s="26" t="inlineStr">
+        <is>
+          <t>axe</t>
+        </is>
+      </c>
+      <c r="G15" s="27" t="inlineStr">
+        <is>
+          <t>tests/components/code/behavior.spec.ts</t>
+        </is>
+      </c>
+      <c r="H15" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I15" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J15" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K15" s="27" t="n"/>
+      <c r="L15" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" s="26">
+        <f>IF(OR(AND(I15="yes",H15="verified"),AND(I15="no",OR(H15="tested",H15="verified")),AND(H15="not applicable",K15&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="54" customHeight="1" s="17">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>CO-08</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D16" s="27" t="inlineStr">
+        <is>
+          <t>Defaults, recipes, appearances, customization, narrow layout, and RTL own baselines.</t>
+        </is>
+      </c>
+      <c r="E16" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F16" s="26" t="inlineStr">
+        <is>
+          <t>visual</t>
+        </is>
+      </c>
+      <c r="G16" s="27" t="inlineStr">
+        <is>
+          <t>tests/components/code/visual.spec.ts</t>
+        </is>
+      </c>
+      <c r="H16" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I16" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J16" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K16" s="27" t="inlineStr">
+        <is>
+          <t>Human snapshot review is pending.</t>
+        </is>
+      </c>
+      <c r="L16" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" s="26">
+        <f>IF(OR(AND(I16="yes",H16="verified"),AND(I16="no",OR(H16="tested",H16="verified")),AND(H16="not applicable",K16&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="54" customHeight="1" s="17">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>CO-09</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>Responsive</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D17" s="27" t="inlineStr">
+        <is>
+          <t>Long literals, narrow widths, RTL prose, zoom, and text spacing remain readable.</t>
+        </is>
+      </c>
+      <c r="E17" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F17" s="26" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G17" s="27" t="inlineStr">
+        <is>
+          <t>manual-tests/code.md</t>
+        </is>
+      </c>
+      <c r="H17" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I17" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J17" s="28" t="n"/>
+      <c r="K17" s="27" t="inlineStr">
+        <is>
+          <t>Protocol exists; human run is pending.</t>
+        </is>
+      </c>
+      <c r="L17" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" s="26">
+        <f>IF(OR(AND(I17="yes",H17="verified"),AND(I17="no",OR(H17="tested",H17="verified")),AND(H17="not applicable",K17&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="54" customHeight="1" s="17">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>CO-10</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D18" s="27" t="inlineStr">
+        <is>
+          <t>The component-owned protocol covers every Code playground scenario.</t>
+        </is>
+      </c>
+      <c r="E18" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F18" s="26" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G18" s="27" t="inlineStr">
+        <is>
+          <t>manual-tests/code.md</t>
+        </is>
+      </c>
+      <c r="H18" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I18" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J18" s="28" t="n"/>
+      <c r="K18" s="27" t="inlineStr">
+        <is>
+          <t>Protocol exists; human run is pending.</t>
+        </is>
+      </c>
+      <c r="L18" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="26">
+        <f>IF(OR(AND(I18="yes",H18="verified"),AND(I18="no",OR(H18="tested",H18="verified")),AND(H18="not applicable",K18&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="54" customHeight="1" s="17">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>CO-11</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>Source-backed usage, recipes, semantics, API, tokens, and exclusions pass.</t>
+        </is>
+      </c>
+      <c r="E19" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F19" s="26" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="G19" s="27" t="inlineStr">
+        <is>
+          <t>../docs/components/code/README.md</t>
+        </is>
+      </c>
+      <c r="H19" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I19" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J19" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K19" s="27" t="n"/>
+      <c r="L19" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" s="26">
+        <f>IF(OR(AND(I19="yes",H19="verified"),AND(I19="no",OR(H19="tested",H19="verified")),AND(H19="not applicable",K19&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="54" customHeight="1" s="17">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>CO-12</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>Changelog</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="inlineStr">
+        <is>
+          <t>Code owns a public changelog and the package changelog records its addition.</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F20" s="26" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="G20" s="27" t="inlineStr">
+        <is>
+          <t>../docs/components/code/CHANGELOG.md; ../CHANGELOG.md</t>
+        </is>
+      </c>
+      <c r="H20" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I20" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J20" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K20" s="27" t="inlineStr">
+        <is>
+          <t>Protocol exists; the owner deferred the human run.</t>
+        </is>
+      </c>
+      <c r="L20" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M20" s="26">
+        <f>IF(OR(AND(I20="yes",H20="verified"),AND(I20="no",OR(H20="tested",H20="verified")),AND(H20="not applicable",K20&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="54" customHeight="1" s="17">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>CO-13</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D21" s="27" t="inlineStr">
+        <is>
+          <t>The packed Consumer proves the public subpath in realistic prose.</t>
+        </is>
+      </c>
+      <c r="E21" s="26" t="inlineStr">
+        <is>
+          <t>consumer</t>
+        </is>
+      </c>
+      <c r="F21" s="26" t="inlineStr">
+        <is>
+          <t>consumer</t>
+        </is>
+      </c>
+      <c r="G21" s="27" t="inlineStr">
+        <is>
+          <t>../apps/consumer/src/App.tsx; ../apps/consumer/tests/consumer.spec.ts</t>
+        </is>
+      </c>
+      <c r="H21" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I21" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J21" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K21" s="27" t="n"/>
+      <c r="L21" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M21" s="26">
+        <f>IF(OR(AND(I21="yes",H21="verified"),AND(I21="no",OR(H21="tested",H21="verified")),AND(H21="not applicable",K21&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="54" customHeight="1" s="17">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>CO-14</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D22" s="27" t="inlineStr">
+        <is>
+          <t>Inline technical displays adopt Code and raw code hosts are rejected.</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F22" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="G22" s="27" t="inlineStr">
+        <is>
+          <t>docs/code-adoption-audit.md; ../scripts/verify-playground-code.mjs</t>
+        </is>
+      </c>
+      <c r="H22" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I22" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J22" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K22" s="27" t="n"/>
+      <c r="L22" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" s="26">
+        <f>IF(OR(AND(I22="yes",H22="verified"),AND(I22="no",OR(H22="tested",H22="verified")),AND(H22="not applicable",K22&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="54" customHeight="1" s="17">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>CO-15</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>Package</t>
+        </is>
+      </c>
+      <c r="C23" s="26" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D23" s="27" t="inlineStr">
+        <is>
+          <t>Build, SSR, exports, CSS, tarball, consumers, browser matrix, and adoption checks pass.</t>
+        </is>
+      </c>
+      <c r="E23" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F23" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="G23" s="27" t="inlineStr">
+        <is>
+          <t>../test/package; ../scripts/verify-consumers.mjs</t>
+        </is>
+      </c>
+      <c r="H23" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I23" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J23" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K23" s="27" t="inlineStr">
+        <is>
+          <t>Automated and human release gates are pending.</t>
+        </is>
+      </c>
+      <c r="L23" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M23" s="26">
+        <f>IF(OR(AND(I23="yes",H23="verified"),AND(I23="no",OR(H23="tested",H23="verified")),AND(H23="not applicable",K23&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="54" customHeight="1" s="17">
+      <c r="A24" s="26" t="n"/>
+      <c r="B24" s="26" t="n"/>
+      <c r="C24" s="26" t="n"/>
+      <c r="D24" s="27" t="n"/>
+      <c r="E24" s="26" t="n"/>
+      <c r="F24" s="26" t="n"/>
+      <c r="G24" s="27" t="n"/>
+      <c r="H24" s="26" t="n"/>
+      <c r="I24" s="26" t="n"/>
+      <c r="J24" s="28" t="n"/>
+      <c r="K24" s="27" t="n"/>
+      <c r="L24" s="26" t="n"/>
+      <c r="M24" s="26" t="n"/>
+    </row>
+    <row r="25" ht="54" customHeight="1" s="17">
+      <c r="A25" s="26" t="n"/>
+      <c r="B25" s="26" t="n"/>
+      <c r="C25" s="26" t="n"/>
+      <c r="D25" s="27" t="n"/>
+      <c r="E25" s="26" t="n"/>
+      <c r="F25" s="26" t="n"/>
+      <c r="G25" s="27" t="n"/>
+      <c r="H25" s="26" t="n"/>
+      <c r="I25" s="26" t="n"/>
+      <c r="J25" s="28" t="n"/>
+      <c r="K25" s="27" t="n"/>
+      <c r="L25" s="26" t="n"/>
+      <c r="M25" s="26" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:M25"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.71" customWidth="1" style="23" min="1" max="1"/>
+    <col width="15.71" customWidth="1" style="23" min="2" max="2"/>
+    <col width="18.71" customWidth="1" style="23" min="3" max="3"/>
+    <col width="58.71" customWidth="1" style="23" min="4" max="4"/>
+    <col width="14.71" customWidth="1" style="23" min="5" max="6"/>
+    <col width="50.71" customWidth="1" style="23" min="7" max="7"/>
+    <col width="17.71" customWidth="1" style="23" min="8" max="8"/>
+    <col width="14.71" customWidth="1" style="23" min="9" max="9"/>
+    <col width="14.71" customWidth="1" style="25" min="10" max="10"/>
+    <col width="42.71" customWidth="1" style="23" min="11" max="11"/>
+    <col width="10.71" customWidth="1" style="23" min="12" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="37.5" customHeight="1" s="17">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Code Block Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="27.75" customHeight="1" s="17">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Assertion-level compound source, Clipboard, overflow, browser, human-review, documentation, Consumer, and adoption evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="17.25" customHeight="1" s="17">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>Requirements</t>
+        </is>
+      </c>
+      <c r="B4" s="21">
+        <f>COUNTA(A9:A25)</f>
+        <v/>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="E4" s="21">
+        <f>SUM(M9:M25)</f>
+        <v/>
+      </c>
+      <c r="G4" s="20" t="inlineStr">
+        <is>
+          <t>Completion</t>
+        </is>
+      </c>
+      <c r="H4" s="22">
+        <f>IF(B4=0,0,E4/B4)</f>
+        <v/>
+      </c>
+      <c r="J4" s="20" t="inlineStr">
+        <is>
+          <t>Package gate</t>
+        </is>
+      </c>
+      <c r="K4" s="21">
+        <f>IF(COUNTIFS(E9:E25,"package",M9:M25,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="17.25" customHeight="1" s="17">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Manual review</t>
+        </is>
+      </c>
+      <c r="B5" s="21">
+        <f>IF(COUNTIFS(I9:I25,"yes",M9:M25,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>Consumer gate</t>
+        </is>
+      </c>
+      <c r="E5" s="21">
+        <f>IF(COUNTIFS(E9:E25,"consumer",M9:M25,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="17">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="inlineStr">
+        <is>
+          <t>Evidence type</t>
+        </is>
+      </c>
+      <c r="G8" s="23" t="inlineStr">
+        <is>
+          <t>Evidence / link</t>
+        </is>
+      </c>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>Human review?</t>
+        </is>
+      </c>
+      <c r="J8" s="25" t="inlineStr">
+        <is>
+          <t>Last verified</t>
+        </is>
+      </c>
+      <c r="K8" s="23" t="inlineStr">
+        <is>
+          <t>Blocker / N/A reason</t>
+        </is>
+      </c>
+      <c r="L8" s="23" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="M8" s="23" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="54" customHeight="1" s="17">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>CB-01</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>Root and anatomy</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="inlineStr">
+        <is>
+          <t>Atom Clipboard Root plus Header, Title, Language, Actions, Content, and copy parts compose correctly.</t>
+        </is>
+      </c>
+      <c r="E9" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F9" s="26" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="G9" s="27" t="inlineStr">
+        <is>
+          <t>../src/components/code-block</t>
+        </is>
+      </c>
+      <c r="H9" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I9" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J9" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K9" s="27" t="n"/>
+      <c r="L9" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" s="26">
+        <f>IF(OR(AND(I9="yes",H9="verified"),AND(I9="no",OR(H9="tested",H9="verified")),AND(H9="not applicable",K9&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="54" customHeight="1" s="17">
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>CB-02</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>Composition</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>Content composes one Scroll Area viewport and canonical pre &gt; Brick Code markup.</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F10" s="26" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="G10" s="27" t="inlineStr">
+        <is>
+          <t>../test/components/code-block/code-block.test.tsx</t>
+        </is>
+      </c>
+      <c r="H10" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I10" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J10" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K10" s="27" t="n"/>
+      <c r="L10" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" s="26">
+        <f>IF(OR(AND(I10="yes",H10="verified"),AND(I10="no",OR(H10="tested",H10="verified")),AND(H10="not applicable",K10&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1" s="17">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>CB-03</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>Clipboard</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>Copy parts</t>
+        </is>
+      </c>
+      <c r="D11" s="27" t="inlineStr">
+        <is>
+          <t>CopyTrigger, indicators, status, pending, success, failure, timeout, and disabled state use Atom Clipboard.</t>
+        </is>
+      </c>
+      <c r="E11" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F11" s="26" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="G11" s="27" t="inlineStr">
+        <is>
+          <t>../test/components/code-block/code-block.test.tsx</t>
+        </is>
+      </c>
+      <c r="H11" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I11" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J11" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K11" s="27" t="n"/>
+      <c r="L11" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" s="26">
+        <f>IF(OR(AND(I11="yes",H11="verified"),AND(I11="no",OR(H11="tested",H11="verified")),AND(H11="not applicable",K11&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="54" customHeight="1" s="17">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>CB-04</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>Exports</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>Code Block</t>
+        </is>
+      </c>
+      <c r="D12" s="27" t="inlineStr">
+        <is>
+          <t>Root and Code Block subpath exports expose the compound runtime and every public type.</t>
+        </is>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="G12" s="27" t="inlineStr">
+        <is>
+          <t>../test/package/package.test.mjs; ../test/package/ssr.test.mjs</t>
+        </is>
+      </c>
+      <c r="H12" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I12" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J12" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K12" s="27" t="n"/>
+      <c r="L12" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" s="26">
+        <f>IF(OR(AND(I12="yes",H12="verified"),AND(I12="no",OR(H12="tested",H12="verified")),AND(H12="not applicable",K12&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="54" customHeight="1" s="17">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>CB-05</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>Types</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>Code Block</t>
+        </is>
+      </c>
+      <c r="D13" s="27" t="inlineStr">
+        <is>
+          <t>Anatomy, recipes, wrap policy, Clipboard props, native props, and refs type-check.</t>
+        </is>
+      </c>
+      <c r="E13" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F13" s="26" t="inlineStr">
+        <is>
+          <t>types</t>
+        </is>
+      </c>
+      <c r="G13" s="27" t="inlineStr">
+        <is>
+          <t>../test/types/components/code-block.test.ts</t>
+        </is>
+      </c>
+      <c r="H13" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I13" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J13" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K13" s="27" t="n"/>
+      <c r="L13" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" s="26">
+        <f>IF(OR(AND(I13="yes",H13="verified"),AND(I13="no",OR(H13="tested",H13="verified")),AND(H13="not applicable",K13&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="54" customHeight="1" s="17">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>CB-06</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>CSS</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>Code Block</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>Static CSS ships surfaces, density, overflow, wrapping, selection, focus, forced colors, and tokens.</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F14" s="26" t="inlineStr">
+        <is>
+          <t>css</t>
+        </is>
+      </c>
+      <c r="G14" s="27" t="inlineStr">
+        <is>
+          <t>../src/components/code-block/code-block.css</t>
+        </is>
+      </c>
+      <c r="H14" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I14" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J14" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K14" s="27" t="n"/>
+      <c r="L14" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" s="26">
+        <f>IF(OR(AND(I14="yes",H14="verified"),AND(I14="no",OR(H14="tested",H14="verified")),AND(H14="not applicable",K14&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="54" customHeight="1" s="17">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>CB-07</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>Browser</t>
+        </is>
+      </c>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>Code Block</t>
+        </is>
+      </c>
+      <c r="D15" s="27" t="inlineStr">
+        <is>
+          <t>Overflow, wrap, copy outcomes, focus retention, disabled state, RTL, and reflow pass.</t>
+        </is>
+      </c>
+      <c r="E15" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F15" s="26" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+      <c r="G15" s="27" t="inlineStr">
+        <is>
+          <t>tests/components/code-block/behavior.spec.ts</t>
+        </is>
+      </c>
+      <c r="H15" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I15" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J15" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K15" s="27" t="n"/>
+      <c r="L15" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" s="26">
+        <f>IF(OR(AND(I15="yes",H15="verified"),AND(I15="no",OR(H15="tested",H15="verified")),AND(H15="not applicable",K15&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="54" customHeight="1" s="17">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>CB-08</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>Content and copy</t>
+        </is>
+      </c>
+      <c r="D16" s="27" t="inlineStr">
+        <is>
+          <t>Named scroll content, truthful live feedback, keyboard reachability, and axe pass.</t>
+        </is>
+      </c>
+      <c r="E16" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F16" s="26" t="inlineStr">
+        <is>
+          <t>axe</t>
+        </is>
+      </c>
+      <c r="G16" s="27" t="inlineStr">
+        <is>
+          <t>tests/components/code-block/behavior.spec.ts</t>
+        </is>
+      </c>
+      <c r="H16" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I16" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J16" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K16" s="27" t="n"/>
+      <c r="L16" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" s="26">
+        <f>IF(OR(AND(I16="yes",H16="verified"),AND(I16="no",OR(H16="tested",H16="verified")),AND(H16="not applicable",K16&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="54" customHeight="1" s="17">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>CB-09</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>Code Block</t>
+        </is>
+      </c>
+      <c r="D17" s="27" t="inlineStr">
+        <is>
+          <t>Defaults, recipes, anatomy, content, overflow, copy, appearances, mobile, and RTL own baselines.</t>
+        </is>
+      </c>
+      <c r="E17" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F17" s="26" t="inlineStr">
+        <is>
+          <t>visual</t>
+        </is>
+      </c>
+      <c r="G17" s="27" t="inlineStr">
+        <is>
+          <t>tests/components/code-block/visual.spec.ts</t>
+        </is>
+      </c>
+      <c r="H17" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I17" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J17" s="28" t="n"/>
+      <c r="K17" s="27" t="inlineStr">
+        <is>
+          <t>Human snapshot review is pending.</t>
+        </is>
+      </c>
+      <c r="L17" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" s="26">
+        <f>IF(OR(AND(I17="yes",H17="verified"),AND(I17="no",OR(H17="tested",H17="verified")),AND(H17="not applicable",K17&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="54" customHeight="1" s="17">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>CB-10</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>Responsive</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>Code Block</t>
+        </is>
+      </c>
+      <c r="D18" s="27" t="inlineStr">
+        <is>
+          <t>Mobile, zoom, long lines, many lines, RTL chrome, LTR source, and selection remain usable.</t>
+        </is>
+      </c>
+      <c r="E18" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F18" s="26" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G18" s="27" t="inlineStr">
+        <is>
+          <t>manual-tests/code-block.md</t>
+        </is>
+      </c>
+      <c r="H18" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I18" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J18" s="28" t="n"/>
+      <c r="K18" s="27" t="inlineStr">
+        <is>
+          <t>Protocol exists; human run is pending.</t>
+        </is>
+      </c>
+      <c r="L18" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="26">
+        <f>IF(OR(AND(I18="yes",H18="verified"),AND(I18="no",OR(H18="tested",H18="verified")),AND(H18="not applicable",K18&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="54" customHeight="1" s="17">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>CB-11</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>Code Block</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>The component-owned protocol covers every Code Block playground scenario.</t>
+        </is>
+      </c>
+      <c r="E19" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F19" s="26" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G19" s="27" t="inlineStr">
+        <is>
+          <t>manual-tests/code-block.md</t>
+        </is>
+      </c>
+      <c r="H19" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I19" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J19" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K19" s="27" t="inlineStr">
+        <is>
+          <t>Protocol exists; human run is pending.</t>
+        </is>
+      </c>
+      <c r="L19" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" s="26">
+        <f>IF(OR(AND(I19="yes",H19="verified"),AND(I19="no",OR(H19="tested",H19="verified")),AND(H19="not applicable",K19&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="54" customHeight="1" s="17">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>CB-12</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>Code Block</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="inlineStr">
+        <is>
+          <t>Source-backed anatomy, copy ownership, highlighting boundary, accessibility, API, and tokens pass.</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F20" s="26" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="G20" s="27" t="inlineStr">
+        <is>
+          <t>../docs/components/code-block/README.md</t>
+        </is>
+      </c>
+      <c r="H20" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I20" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J20" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K20" s="27" t="inlineStr">
+        <is>
+          <t>Protocol exists; the owner deferred the human run.</t>
+        </is>
+      </c>
+      <c r="L20" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M20" s="26">
+        <f>IF(OR(AND(I20="yes",H20="verified"),AND(I20="no",OR(H20="tested",H20="verified")),AND(H20="not applicable",K20&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="54" customHeight="1" s="17">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>CB-13</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>Changelog</t>
+        </is>
+      </c>
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>Code Block</t>
+        </is>
+      </c>
+      <c r="D21" s="27" t="inlineStr">
+        <is>
+          <t>Code Block owns a public changelog and the package changelog records its addition.</t>
+        </is>
+      </c>
+      <c r="E21" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F21" s="26" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="G21" s="27" t="inlineStr">
+        <is>
+          <t>../docs/components/code-block/CHANGELOG.md; ../CHANGELOG.md</t>
+        </is>
+      </c>
+      <c r="H21" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I21" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J21" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K21" s="27" t="n"/>
+      <c r="L21" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M21" s="26">
+        <f>IF(OR(AND(I21="yes",H21="verified"),AND(I21="no",OR(H21="tested",H21="verified")),AND(H21="not applicable",K21&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="54" customHeight="1" s="17">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>CB-14</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>Code Block</t>
+        </is>
+      </c>
+      <c r="D22" s="27" t="inlineStr">
+        <is>
+          <t>The packed Consumer proves public subpath anatomy, native source, and copy action.</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>consumer</t>
+        </is>
+      </c>
+      <c r="F22" s="26" t="inlineStr">
+        <is>
+          <t>consumer</t>
+        </is>
+      </c>
+      <c r="G22" s="27" t="inlineStr">
+        <is>
+          <t>../apps/consumer/src/App.tsx; ../apps/consumer/tests/consumer.spec.ts</t>
+        </is>
+      </c>
+      <c r="H22" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I22" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J22" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K22" s="27" t="n"/>
+      <c r="L22" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" s="26">
+        <f>IF(OR(AND(I22="yes",H22="verified"),AND(I22="no",OR(H22="tested",H22="verified")),AND(H22="not applicable",K22&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="54" customHeight="1" s="17">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>CB-15</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="C23" s="26" t="inlineStr">
+        <is>
+          <t>Code Block</t>
+        </is>
+      </c>
+      <c r="D23" s="27" t="inlineStr">
+        <is>
+          <t>Structured technical displays adopt Code Block with no raw pre/code hosts.</t>
+        </is>
+      </c>
+      <c r="E23" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F23" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="G23" s="27" t="inlineStr">
+        <is>
+          <t>docs/code-adoption-audit.md; ../scripts/verify-playground-code.mjs</t>
+        </is>
+      </c>
+      <c r="H23" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I23" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J23" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K23" s="27" t="n"/>
+      <c r="L23" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M23" s="26">
+        <f>IF(OR(AND(I23="yes",H23="verified"),AND(I23="no",OR(H23="tested",H23="verified")),AND(H23="not applicable",K23&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="54" customHeight="1" s="17">
+      <c r="A24" s="26" t="inlineStr">
+        <is>
+          <t>CB-16</t>
+        </is>
+      </c>
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>Package</t>
+        </is>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>Code Block</t>
+        </is>
+      </c>
+      <c r="D24" s="27" t="inlineStr">
+        <is>
+          <t>Build, SSR, exports, CSS, Atom dependency, tarball, consumers, browser matrix, and adoption pass.</t>
+        </is>
+      </c>
+      <c r="E24" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F24" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="G24" s="27" t="inlineStr">
+        <is>
+          <t>../test/package; ../scripts/verify-consumers.mjs</t>
+        </is>
+      </c>
+      <c r="H24" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I24" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J24" s="28" t="n">
+        <v>46228</v>
+      </c>
+      <c r="K24" s="27" t="inlineStr">
+        <is>
+          <t>Automated and human release gates are pending.</t>
+        </is>
+      </c>
+      <c r="L24" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M24" s="26">
+        <f>IF(OR(AND(I24="yes",H24="verified"),AND(I24="no",OR(H24="tested",H24="verified")),AND(H24="not applicable",K24&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="54" customHeight="1" s="17">
+      <c r="A25" s="26" t="n"/>
+      <c r="B25" s="26" t="n"/>
+      <c r="C25" s="26" t="n"/>
+      <c r="D25" s="27" t="n"/>
+      <c r="E25" s="26" t="n"/>
+      <c r="F25" s="26" t="n"/>
+      <c r="G25" s="27" t="n"/>
+      <c r="H25" s="26" t="n"/>
+      <c r="I25" s="26" t="n"/>
+      <c r="J25" s="28" t="n"/>
+      <c r="K25" s="27" t="n"/>
+      <c r="L25" s="26" t="n"/>
+      <c r="M25" s="26" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">

</xml_diff>

<commit_message>
feat: add nav list component
</commit_message>
<xml_diff>
--- a/playground/component-coverage.xlsx
+++ b/playground/component-coverage.xlsx
@@ -41,6 +41,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scroll Area" sheetId="32" state="visible" r:id="rId32"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code" sheetId="33" state="visible" r:id="rId33"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Block" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nav List" sheetId="35" state="visible" r:id="rId35"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$7:$M$38</definedName>
@@ -1100,7 +1101,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M38"/>
+  <dimension ref="A1:M39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="24.71" customWidth="1" style="23" min="1" max="1"/>
@@ -2930,6 +2931,61 @@
       </c>
       <c r="M38" s="23">
         <f>IF(AND(J38=1,K38="complete",L38="complete"),"complete",IF(H38&gt;0,"blocked","open"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="23" t="inlineStr">
+        <is>
+          <t>Nav List</t>
+        </is>
+      </c>
+      <c r="B39" s="23">
+        <f>INDIRECT("'"&amp;A39&amp;"'!B4")</f>
+        <v/>
+      </c>
+      <c r="C39" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A39&amp;"'!H9:H200"),"not started")</f>
+        <v/>
+      </c>
+      <c r="D39" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A39&amp;"'!H9:H200"),"partial")</f>
+        <v/>
+      </c>
+      <c r="E39" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A39&amp;"'!H9:H200"),"implemented")</f>
+        <v/>
+      </c>
+      <c r="F39" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A39&amp;"'!H9:H200"),"tested")</f>
+        <v/>
+      </c>
+      <c r="G39" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A39&amp;"'!H9:H200"),"verified")</f>
+        <v/>
+      </c>
+      <c r="H39" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A39&amp;"'!H9:H200"),"blocked")</f>
+        <v/>
+      </c>
+      <c r="I39" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A39&amp;"'!H9:H200"),"not applicable")</f>
+        <v/>
+      </c>
+      <c r="J39" s="24">
+        <f>INDIRECT("'"&amp;A39&amp;"'!H4")</f>
+        <v/>
+      </c>
+      <c r="K39" s="23">
+        <f>INDIRECT("'"&amp;A39&amp;"'!K4")</f>
+        <v/>
+      </c>
+      <c r="L39" s="23">
+        <f>INDIRECT("'"&amp;A39&amp;"'!E5")</f>
+        <v/>
+      </c>
+      <c r="M39" s="23">
+        <f>IF(AND(J39=1,K39="complete",L39="complete"),"complete",IF(H39&gt;0,"blocked","open"))</f>
         <v/>
       </c>
     </row>
@@ -31844,6 +31900,1185 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:M25"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.71" customWidth="1" style="23" min="1" max="1"/>
+    <col width="15.71" customWidth="1" style="23" min="2" max="2"/>
+    <col width="18.71" customWidth="1" style="23" min="3" max="3"/>
+    <col width="58.71" customWidth="1" style="23" min="4" max="4"/>
+    <col width="14.71" customWidth="1" style="23" min="5" max="6"/>
+    <col width="50.71" customWidth="1" style="23" min="7" max="7"/>
+    <col width="17.71" customWidth="1" style="23" min="8" max="8"/>
+    <col width="14.71" customWidth="1" style="23" min="9" max="9"/>
+    <col width="14.71" customWidth="1" style="25" min="10" max="10"/>
+    <col width="42.71" customWidth="1" style="23" min="11" max="11"/>
+    <col width="10.71" customWidth="1" style="23" min="12" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="37.5" customHeight="1" s="17">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Nav List Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="27.75" customHeight="1" s="17">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Assertion-level Atom anatomy, recipes, disclosure, browser, human-review, documentation, Consumer, and adoption evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="17.25" customHeight="1" s="17">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>Requirements</t>
+        </is>
+      </c>
+      <c r="B4" s="21">
+        <f>COUNTA(A9:A25)</f>
+        <v/>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="E4" s="21">
+        <f>SUM(M9:M25)</f>
+        <v/>
+      </c>
+      <c r="G4" s="20" t="inlineStr">
+        <is>
+          <t>Completion</t>
+        </is>
+      </c>
+      <c r="H4" s="22">
+        <f>IF(B4=0,0,E4/B4)</f>
+        <v/>
+      </c>
+      <c r="J4" s="20" t="inlineStr">
+        <is>
+          <t>Package gate</t>
+        </is>
+      </c>
+      <c r="K4" s="21">
+        <f>IF(COUNTIFS(E9:E25,"package",M9:M25,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="17.25" customHeight="1" s="17">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Manual review</t>
+        </is>
+      </c>
+      <c r="B5" s="21">
+        <f>IF(COUNTIFS(I9:I25,"yes",M9:M25,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>Consumer gate</t>
+        </is>
+      </c>
+      <c r="E5" s="21">
+        <f>IF(COUNTIFS(E9:E25,"consumer",M9:M25,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="17">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="inlineStr">
+        <is>
+          <t>Evidence type</t>
+        </is>
+      </c>
+      <c r="G8" s="23" t="inlineStr">
+        <is>
+          <t>Evidence / link</t>
+        </is>
+      </c>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>Human review?</t>
+        </is>
+      </c>
+      <c r="J8" s="25" t="inlineStr">
+        <is>
+          <t>Last verified</t>
+        </is>
+      </c>
+      <c r="K8" s="23" t="inlineStr">
+        <is>
+          <t>Blocker / N/A reason</t>
+        </is>
+      </c>
+      <c r="L8" s="23" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="M8" s="23" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="54" customHeight="1" s="17">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>NL-01</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>Root and anatomy</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="inlineStr">
+        <is>
+          <t>Root, List, Item, Link, Section, SectionLabel, SectionTrigger, and SectionContent compose correctly.</t>
+        </is>
+      </c>
+      <c r="E9" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F9" s="26" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="G9" s="27" t="inlineStr">
+        <is>
+          <t>../src/components/code-block</t>
+        </is>
+      </c>
+      <c r="H9" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I9" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J9" s="28" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="K9" s="27" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="L9" s="26" t="inlineStr"/>
+      <c r="M9" s="26">
+        <f>IF(OR(H9="not started",H9="partial"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="54" customHeight="1" s="17">
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>NL-02</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>Recipes</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>Soft, solid, and outline; accent and neutral; small, medium, and large preserve declared defaults.</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F10" s="26" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="G10" s="27" t="inlineStr">
+        <is>
+          <t>../test/components/code-block/code-block.test.tsx</t>
+        </is>
+      </c>
+      <c r="H10" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I10" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J10" s="28" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="K10" s="27" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="L10" s="26" t="inlineStr"/>
+      <c r="M10" s="26">
+        <f>IF(OR(H10="not started",H10="partial"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1" s="17">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>NL-03</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="D11" s="27" t="inlineStr">
+        <is>
+          <t>Leading content, trailing content, descriptions, current, disabled, and composition remain aligned and semantic.</t>
+        </is>
+      </c>
+      <c r="E11" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F11" s="26" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="G11" s="27" t="inlineStr">
+        <is>
+          <t>../test/components/code-block/code-block.test.tsx</t>
+        </is>
+      </c>
+      <c r="H11" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I11" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J11" s="28" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="K11" s="27" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="L11" s="26" t="inlineStr"/>
+      <c r="M11" s="26">
+        <f>IF(OR(H11="not started",H11="partial"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="54" customHeight="1" s="17">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>NL-04</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>Sections</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>Disclosure</t>
+        </is>
+      </c>
+      <c r="D12" s="27" t="inlineStr">
+        <is>
+          <t>Labeled, controlled, uncontrolled, disabled, and non-collapsible sections preserve Atom relationships.</t>
+        </is>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="G12" s="27" t="inlineStr">
+        <is>
+          <t>../test/package/package.test.mjs; ../test/package/ssr.test.mjs</t>
+        </is>
+      </c>
+      <c r="H12" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I12" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J12" s="28" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="K12" s="27" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="L12" s="26" t="inlineStr"/>
+      <c r="M12" s="26">
+        <f>IF(OR(H12="not started",H12="partial"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="54" customHeight="1" s="17">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>NL-05</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>Exports</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>Nav List</t>
+        </is>
+      </c>
+      <c r="D13" s="27" t="inlineStr">
+        <is>
+          <t>Root and Nav List subpath exports expose the compound runtime and every public type.</t>
+        </is>
+      </c>
+      <c r="E13" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F13" s="26" t="inlineStr">
+        <is>
+          <t>types</t>
+        </is>
+      </c>
+      <c r="G13" s="27" t="inlineStr">
+        <is>
+          <t>../test/types/components/code-block.test.ts</t>
+        </is>
+      </c>
+      <c r="H13" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I13" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J13" s="28" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="K13" s="27" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="L13" s="26" t="inlineStr"/>
+      <c r="M13" s="26">
+        <f>IF(OR(H13="not started",H13="partial"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="54" customHeight="1" s="17">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>NL-06</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>Types</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>Nav List</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>Anatomy, recipes, native props, composition, and refs type-check.</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F14" s="26" t="inlineStr">
+        <is>
+          <t>css</t>
+        </is>
+      </c>
+      <c r="G14" s="27" t="inlineStr">
+        <is>
+          <t>../src/components/code-block/code-block.css</t>
+        </is>
+      </c>
+      <c r="H14" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I14" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J14" s="28" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="K14" s="27" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="L14" s="26" t="inlineStr"/>
+      <c r="M14" s="26">
+        <f>IF(OR(H14="not started",H14="partial"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="54" customHeight="1" s="17">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>NL-07</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>CSS</t>
+        </is>
+      </c>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>Nav List</t>
+        </is>
+      </c>
+      <c r="D15" s="27" t="inlineStr">
+        <is>
+          <t>Static CSS ships state, orientation, focus, forced-colors, logical layout, and public tokens.</t>
+        </is>
+      </c>
+      <c r="E15" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F15" s="26" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+      <c r="G15" s="27" t="inlineStr">
+        <is>
+          <t>tests/components/code-block/behavior.spec.ts</t>
+        </is>
+      </c>
+      <c r="H15" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I15" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J15" s="28" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="K15" s="27" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="L15" s="26" t="inlineStr"/>
+      <c r="M15" s="26">
+        <f>IF(OR(H15="not started",H15="partial"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="54" customHeight="1" s="17">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>NL-08</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>Browser</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>Nav List</t>
+        </is>
+      </c>
+      <c r="D16" s="27" t="inlineStr">
+        <is>
+          <t>Defaults, disclosure, disabled state, composition, horizontal wrapping, and RTL pass.</t>
+        </is>
+      </c>
+      <c r="E16" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F16" s="26" t="inlineStr">
+        <is>
+          <t>axe</t>
+        </is>
+      </c>
+      <c r="G16" s="27" t="inlineStr">
+        <is>
+          <t>tests/components/code-block/behavior.spec.ts</t>
+        </is>
+      </c>
+      <c r="H16" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I16" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J16" s="28" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="K16" s="27" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="L16" s="26" t="inlineStr"/>
+      <c r="M16" s="26">
+        <f>IF(OR(H16="not started",H16="partial"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="54" customHeight="1" s="17">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>NL-09</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>Navigation anatomy</t>
+        </is>
+      </c>
+      <c r="D17" s="27" t="inlineStr">
+        <is>
+          <t>Names, lists, current state, disabled state, disclosure relationships, keyboard use, and axe pass.</t>
+        </is>
+      </c>
+      <c r="E17" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F17" s="26" t="inlineStr">
+        <is>
+          <t>visual</t>
+        </is>
+      </c>
+      <c r="G17" s="27" t="inlineStr">
+        <is>
+          <t>tests/components/code-block/visual.spec.ts</t>
+        </is>
+      </c>
+      <c r="H17" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I17" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J17" s="28" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="K17" s="27" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="L17" s="26" t="inlineStr"/>
+      <c r="M17" s="26">
+        <f>IF(OR(H17="not started",H17="partial"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="54" customHeight="1" s="17">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>NL-10</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>Nav List</t>
+        </is>
+      </c>
+      <c r="D18" s="27" t="inlineStr">
+        <is>
+          <t>Defaults, recipes, content, sections, output, appearances, mobile, RTL, and forced colors own baselines.</t>
+        </is>
+      </c>
+      <c r="E18" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F18" s="26" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G18" s="27" t="inlineStr">
+        <is>
+          <t>manual-tests/code-block.md</t>
+        </is>
+      </c>
+      <c r="H18" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I18" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J18" s="28" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="K18" s="27" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="L18" s="26" t="inlineStr"/>
+      <c r="M18" s="26">
+        <f>IF(OR(H18="not started",H18="partial"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="54" customHeight="1" s="17">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>NL-11</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>Nav List</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>The component-owned protocol covers every Nav List playground scenario.</t>
+        </is>
+      </c>
+      <c r="E19" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F19" s="26" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G19" s="27" t="inlineStr">
+        <is>
+          <t>manual-tests/code-block.md</t>
+        </is>
+      </c>
+      <c r="H19" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I19" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J19" s="28" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="K19" s="27" t="inlineStr">
+        <is>
+          <t>not run</t>
+        </is>
+      </c>
+      <c r="L19" s="26" t="inlineStr"/>
+      <c r="M19" s="26">
+        <f>IF(OR(H19="not started",H19="partial"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="54" customHeight="1" s="17">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>NL-12</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>Nav List</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="inlineStr">
+        <is>
+          <t>Source-backed ownership, anatomy, accessibility, API, CSS, and examples pass the documentation contract.</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F20" s="26" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="G20" s="27" t="inlineStr">
+        <is>
+          <t>../docs/components/code-block/README.md</t>
+        </is>
+      </c>
+      <c r="H20" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I20" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J20" s="28" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="K20" s="27" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="L20" s="26" t="inlineStr"/>
+      <c r="M20" s="26">
+        <f>IF(OR(H20="not started",H20="partial"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="54" customHeight="1" s="17">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>NL-13</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>Changelog</t>
+        </is>
+      </c>
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>Nav List</t>
+        </is>
+      </c>
+      <c r="D21" s="27" t="inlineStr">
+        <is>
+          <t>Nav List owns a public changelog and the package changelog records its addition.</t>
+        </is>
+      </c>
+      <c r="E21" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F21" s="26" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="G21" s="27" t="inlineStr">
+        <is>
+          <t>../docs/components/code-block/CHANGELOG.md; ../CHANGELOG.md</t>
+        </is>
+      </c>
+      <c r="H21" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I21" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J21" s="28" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="K21" s="27" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="L21" s="26" t="inlineStr"/>
+      <c r="M21" s="26">
+        <f>IF(OR(H21="not started",H21="partial"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="54" customHeight="1" s="17">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>NL-14</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>Nav List</t>
+        </is>
+      </c>
+      <c r="D22" s="27" t="inlineStr">
+        <is>
+          <t>The packed Consumer proves the public subpath in realistic workspace navigation.</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>consumer</t>
+        </is>
+      </c>
+      <c r="F22" s="26" t="inlineStr">
+        <is>
+          <t>consumer</t>
+        </is>
+      </c>
+      <c r="G22" s="27" t="inlineStr">
+        <is>
+          <t>../apps/consumer/src/App.tsx; ../apps/consumer/tests/consumer.spec.ts</t>
+        </is>
+      </c>
+      <c r="H22" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I22" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J22" s="28" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="K22" s="27" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="L22" s="26" t="inlineStr"/>
+      <c r="M22" s="26">
+        <f>IF(OR(H22="not started",H22="partial"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="54" customHeight="1" s="17">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>NL-15</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="C23" s="26" t="inlineStr">
+        <is>
+          <t>Nav List</t>
+        </is>
+      </c>
+      <c r="D23" s="27" t="inlineStr">
+        <is>
+          <t>The route covers all approved scenarios and the shell adopts public Nav List anatomy.</t>
+        </is>
+      </c>
+      <c r="E23" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F23" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="G23" s="27" t="inlineStr">
+        <is>
+          <t>docs/code-adoption-audit.md; ../scripts/verify-playground-code.mjs</t>
+        </is>
+      </c>
+      <c r="H23" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I23" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J23" s="28" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="K23" s="27" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="L23" s="26" t="inlineStr"/>
+      <c r="M23" s="26">
+        <f>IF(OR(H23="not started",H23="partial"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="54" customHeight="1" s="17">
+      <c r="A24" s="26" t="inlineStr">
+        <is>
+          <t>NL-16</t>
+        </is>
+      </c>
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>Package</t>
+        </is>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>Nav List</t>
+        </is>
+      </c>
+      <c r="D24" s="27" t="inlineStr">
+        <is>
+          <t>Build, SSR, exports, CSS, Atom dependency, tarball, consumers, browser matrix, and adoption pass.</t>
+        </is>
+      </c>
+      <c r="E24" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F24" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="G24" s="27" t="inlineStr">
+        <is>
+          <t>../test/package; ../scripts/verify-consumers.mjs</t>
+        </is>
+      </c>
+      <c r="H24" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I24" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J24" s="28" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="K24" s="27" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="L24" s="26" t="inlineStr"/>
+      <c r="M24" s="26">
+        <f>IF(OR(H24="not started",H24="partial"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="54" customHeight="1" s="17">
+      <c r="A25" s="26" t="n"/>
+      <c r="B25" s="26" t="n"/>
+      <c r="C25" s="26" t="n"/>
+      <c r="D25" s="27" t="n"/>
+      <c r="E25" s="26" t="n"/>
+      <c r="F25" s="26" t="n"/>
+      <c r="G25" s="27" t="n"/>
+      <c r="H25" s="26" t="n"/>
+      <c r="I25" s="26" t="n"/>
+      <c r="J25" s="28" t="n"/>
+      <c r="K25" s="27" t="n"/>
+      <c r="L25" s="26" t="n"/>
+      <c r="M25" s="26" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">

</xml_diff>

<commit_message>
feat: add Sidebar component
</commit_message>
<xml_diff>
--- a/playground/component-coverage.xlsx
+++ b/playground/component-coverage.xlsx
@@ -42,6 +42,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code" sheetId="33" state="visible" r:id="rId33"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Block" sheetId="34" state="visible" r:id="rId34"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nav List" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sidebar" sheetId="36" state="visible" r:id="rId36"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$7:$M$38</definedName>
@@ -1101,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M39"/>
+  <dimension ref="A1:M40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="24.71" customWidth="1" style="23" min="1" max="1"/>
@@ -2986,6 +2987,61 @@
       </c>
       <c r="M39" s="23">
         <f>IF(AND(J39=1,K39="complete",L39="complete"),"complete",IF(H39&gt;0,"blocked","open"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="23" t="inlineStr">
+        <is>
+          <t>Sidebar</t>
+        </is>
+      </c>
+      <c r="B40" s="23">
+        <f>INDIRECT("'"&amp;A40&amp;"'!B4")</f>
+        <v/>
+      </c>
+      <c r="C40" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A40&amp;"'!H9:H200"),"not started")</f>
+        <v/>
+      </c>
+      <c r="D40" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A40&amp;"'!H9:H200"),"partial")</f>
+        <v/>
+      </c>
+      <c r="E40" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A40&amp;"'!H9:H200"),"implemented")</f>
+        <v/>
+      </c>
+      <c r="F40" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A40&amp;"'!H9:H200"),"tested")</f>
+        <v/>
+      </c>
+      <c r="G40" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A40&amp;"'!H9:H200"),"verified")</f>
+        <v/>
+      </c>
+      <c r="H40" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A40&amp;"'!H9:H200"),"blocked")</f>
+        <v/>
+      </c>
+      <c r="I40" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A40&amp;"'!H9:H200"),"not applicable")</f>
+        <v/>
+      </c>
+      <c r="J40" s="24">
+        <f>INDIRECT("'"&amp;A40&amp;"'!H4")</f>
+        <v/>
+      </c>
+      <c r="K40" s="23">
+        <f>INDIRECT("'"&amp;A40&amp;"'!K4")</f>
+        <v/>
+      </c>
+      <c r="L40" s="23">
+        <f>INDIRECT("'"&amp;A40&amp;"'!E5")</f>
+        <v/>
+      </c>
+      <c r="M40" s="23">
+        <f>IF(AND(J40=1,K40="complete",L40="complete"),"complete",IF(H40&gt;0,"blocked","open"))</f>
         <v/>
       </c>
     </row>
@@ -33079,6 +33135,1101 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:M25"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.71" customWidth="1" style="23" min="1" max="1"/>
+    <col width="15.71" customWidth="1" style="23" min="2" max="2"/>
+    <col width="18.71" customWidth="1" style="23" min="3" max="3"/>
+    <col width="58.71" customWidth="1" style="23" min="4" max="4"/>
+    <col width="14.71" customWidth="1" style="23" min="5" max="6"/>
+    <col width="50.71" customWidth="1" style="23" min="7" max="7"/>
+    <col width="17.71" customWidth="1" style="23" min="8" max="8"/>
+    <col width="14.71" customWidth="1" style="23" min="9" max="9"/>
+    <col width="14.71" customWidth="1" style="25" min="10" max="10"/>
+    <col width="42.71" customWidth="1" style="23" min="11" max="11"/>
+    <col width="10.71" customWidth="1" style="23" min="12" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="37.5" customHeight="1" s="17">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Sidebar Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="27.75" customHeight="1" s="17">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Assertion-level Atom anatomy, app-shell geometry, recipes, states, browser, human-review, documentation, Consumer, and adoption evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="17.25" customHeight="1" s="17">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>Requirements</t>
+        </is>
+      </c>
+      <c r="B4" s="21">
+        <f>COUNTA(A9:A25)</f>
+        <v/>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="E4" s="21">
+        <f>SUM(M9:M25)</f>
+        <v/>
+      </c>
+      <c r="G4" s="20" t="inlineStr">
+        <is>
+          <t>Completion</t>
+        </is>
+      </c>
+      <c r="H4" s="22">
+        <f>IF(B4=0,0,E4/B4)</f>
+        <v/>
+      </c>
+      <c r="J4" s="20" t="inlineStr">
+        <is>
+          <t>Package gate</t>
+        </is>
+      </c>
+      <c r="K4" s="21">
+        <f>IF(COUNTIFS(E9:E25,"package",M9:M25,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="17.25" customHeight="1" s="17">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Manual review</t>
+        </is>
+      </c>
+      <c r="B5" s="21">
+        <f>IF(COUNTIFS(I9:I25,"yes",M9:M25,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>Consumer gate</t>
+        </is>
+      </c>
+      <c r="E5" s="21">
+        <f>IF(COUNTIFS(E9:E25,"consumer",M9:M25,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="17">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="inlineStr">
+        <is>
+          <t>Evidence type</t>
+        </is>
+      </c>
+      <c r="G8" s="23" t="inlineStr">
+        <is>
+          <t>Evidence / link</t>
+        </is>
+      </c>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>Human review?</t>
+        </is>
+      </c>
+      <c r="J8" s="25" t="inlineStr">
+        <is>
+          <t>Last verified</t>
+        </is>
+      </c>
+      <c r="K8" s="23" t="inlineStr">
+        <is>
+          <t>Blocker / N/A reason</t>
+        </is>
+      </c>
+      <c r="L8" s="23" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="M8" s="23" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="54" customHeight="1" s="17">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>SB-01</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>Seven parts</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="inlineStr">
+        <is>
+          <t>Root, Trigger, Panel, Header, Content, Footer, and Main compose with exact Atom and Brick ownership.</t>
+        </is>
+      </c>
+      <c r="E9" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F9" s="26" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="G9" s="27" t="inlineStr">
+        <is>
+          <t>../src/components/sidebar</t>
+        </is>
+      </c>
+      <c r="H9" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I9" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J9" s="28" t="inlineStr"/>
+      <c r="K9" s="27" t="inlineStr"/>
+      <c r="L9" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" s="26">
+        <f>IF(OR(H9="not started",H9="partial",H9="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="54" customHeight="1" s="17">
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>SB-02</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>Controlled/uncontrolled expanded, rail, offcanvas, targets, side, and disabled state preserve Atom 0.8.0.</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F10" s="26" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="G10" s="27" t="inlineStr">
+        <is>
+          <t>../test/components/sidebar/sidebar.test.tsx</t>
+        </is>
+      </c>
+      <c r="H10" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I10" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J10" s="28" t="inlineStr"/>
+      <c r="K10" s="27" t="inlineStr"/>
+      <c r="L10" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" s="26">
+        <f>IF(OR(H10="not started",H10="partial",H10="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1" s="17">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>SB-03</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>Recipes</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>Root and Panel</t>
+        </is>
+      </c>
+      <c r="D11" s="27" t="inlineStr">
+        <is>
+          <t>Docked/floating, small/medium/large, and static/sticky preserve declared defaults and geometry.</t>
+        </is>
+      </c>
+      <c r="E11" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F11" s="26" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+      <c r="G11" s="27" t="inlineStr">
+        <is>
+          <t>../playground/tests/components/sidebar/behavior.spec.ts</t>
+        </is>
+      </c>
+      <c r="H11" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I11" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J11" s="28" t="inlineStr"/>
+      <c r="K11" s="27" t="inlineStr"/>
+      <c r="L11" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" s="26">
+        <f>IF(OR(H11="not started",H11="partial",H11="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="54" customHeight="1" s="17">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>SB-04</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>Trigger and Panel</t>
+        </is>
+      </c>
+      <c r="D12" s="27" t="inlineStr">
+        <is>
+          <t>Generated relationships, native activation, disabled state, inert offcanvas content, landmarks, and rail names pass.</t>
+        </is>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+      <c r="G12" s="27" t="inlineStr">
+        <is>
+          <t>../playground/tests/components/sidebar/behavior.spec.ts</t>
+        </is>
+      </c>
+      <c r="H12" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I12" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J12" s="28" t="inlineStr"/>
+      <c r="K12" s="27" t="inlineStr"/>
+      <c r="L12" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" s="26">
+        <f>IF(OR(H12="not started",H12="partial",H12="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="54" customHeight="1" s="17">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>SB-05</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>Composition</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>All parts</t>
+        </is>
+      </c>
+      <c r="D13" s="27" t="inlineStr">
+        <is>
+          <t>Native props, refs, render, asChild, classes, styles, and slot overrides preserve output.</t>
+        </is>
+      </c>
+      <c r="E13" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F13" s="26" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="G13" s="27" t="inlineStr">
+        <is>
+          <t>../test/components/sidebar/sidebar.test.tsx</t>
+        </is>
+      </c>
+      <c r="H13" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I13" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J13" s="28" t="inlineStr"/>
+      <c r="K13" s="27" t="inlineStr"/>
+      <c r="L13" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" s="26">
+        <f>IF(OR(H13="not started",H13="partial",H13="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="54" customHeight="1" s="17">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>SB-06</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>Exports</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>Sidebar</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>Root and Sidebar subpath exports expose runtime and public types.</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F14" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="G14" s="27" t="inlineStr">
+        <is>
+          <t>../test/package/package.test.mjs</t>
+        </is>
+      </c>
+      <c r="H14" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I14" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J14" s="28" t="inlineStr"/>
+      <c r="K14" s="27" t="inlineStr"/>
+      <c r="L14" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" s="26">
+        <f>IF(OR(H14="not started",H14="partial",H14="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="54" customHeight="1" s="17">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>SB-07</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>Types</t>
+        </is>
+      </c>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>Sidebar</t>
+        </is>
+      </c>
+      <c r="D15" s="27" t="inlineStr">
+        <is>
+          <t>Recipes, Atom props, refs, composition, and Root size collision type-check.</t>
+        </is>
+      </c>
+      <c r="E15" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F15" s="26" t="inlineStr">
+        <is>
+          <t>types</t>
+        </is>
+      </c>
+      <c r="G15" s="27" t="inlineStr">
+        <is>
+          <t>../test/types/components/sidebar.test.ts</t>
+        </is>
+      </c>
+      <c r="H15" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I15" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J15" s="28" t="inlineStr"/>
+      <c r="K15" s="27" t="inlineStr"/>
+      <c r="L15" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" s="26">
+        <f>IF(OR(H15="not started",H15="partial",H15="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="54" customHeight="1" s="17">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>SB-08</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>CSS</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>Sidebar</t>
+        </is>
+      </c>
+      <c r="D16" s="27" t="inlineStr">
+        <is>
+          <t>Static CSS ships state/side geometry, regions, focus, motion preferences, forced colors, and public variables.</t>
+        </is>
+      </c>
+      <c r="E16" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F16" s="26" t="inlineStr">
+        <is>
+          <t>css</t>
+        </is>
+      </c>
+      <c r="G16" s="27" t="inlineStr">
+        <is>
+          <t>../src/components/sidebar/sidebar.css</t>
+        </is>
+      </c>
+      <c r="H16" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I16" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J16" s="28" t="inlineStr"/>
+      <c r="K16" s="27" t="inlineStr"/>
+      <c r="L16" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" s="26">
+        <f>IF(OR(H16="not started",H16="partial",H16="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="54" customHeight="1" s="17">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>SB-09</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>Sidebar</t>
+        </is>
+      </c>
+      <c r="D17" s="27" t="inlineStr">
+        <is>
+          <t>Defaults, states, variants, sizes, placement, regions, behavior, appearance, stress, and forced colors own reviewed baselines.</t>
+        </is>
+      </c>
+      <c r="E17" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F17" s="26" t="inlineStr">
+        <is>
+          <t>visual</t>
+        </is>
+      </c>
+      <c r="G17" s="27" t="inlineStr">
+        <is>
+          <t>../playground/tests/components/sidebar/visual.spec.ts</t>
+        </is>
+      </c>
+      <c r="H17" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I17" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J17" s="28" t="inlineStr"/>
+      <c r="K17" s="27" t="inlineStr">
+        <is>
+          <t>Human run pending.</t>
+        </is>
+      </c>
+      <c r="L17" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" s="26">
+        <f>IF(OR(H17="not started",H17="partial",H17="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="54" customHeight="1" s="17">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>SB-10</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>Responsive</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>Sidebar</t>
+        </is>
+      </c>
+      <c r="D18" s="27" t="inlineStr">
+        <is>
+          <t>Main containment, zero offcanvas track, right placement, sticky height, narrow floating, low height, zoom, and reduced motion remain usable.</t>
+        </is>
+      </c>
+      <c r="E18" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F18" s="26" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G18" s="27" t="inlineStr">
+        <is>
+          <t>../playground/manual-tests/sidebar.md</t>
+        </is>
+      </c>
+      <c r="H18" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I18" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J18" s="28" t="inlineStr"/>
+      <c r="K18" s="27" t="inlineStr">
+        <is>
+          <t>Human run pending.</t>
+        </is>
+      </c>
+      <c r="L18" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="26">
+        <f>IF(OR(H18="not started",H18="partial",H18="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="54" customHeight="1" s="17">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>SB-11</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>Sidebar</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>The component-owned protocol covers every Sidebar playground scenario.</t>
+        </is>
+      </c>
+      <c r="E19" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F19" s="26" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G19" s="27" t="inlineStr">
+        <is>
+          <t>../playground/manual-tests/sidebar.md</t>
+        </is>
+      </c>
+      <c r="H19" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I19" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J19" s="28" t="inlineStr"/>
+      <c r="K19" s="27" t="inlineStr">
+        <is>
+          <t>Human run pending.</t>
+        </is>
+      </c>
+      <c r="L19" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" s="26">
+        <f>IF(OR(H19="not started",H19="partial",H19="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="54" customHeight="1" s="17">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>SB-12</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>Sidebar</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="inlineStr">
+        <is>
+          <t>Source-backed ownership, anatomy, states, recipes, Drawer boundary, accessibility, API, and tokens pass.</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F20" s="26" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="G20" s="27" t="inlineStr">
+        <is>
+          <t>../docs/components/sidebar/README.md</t>
+        </is>
+      </c>
+      <c r="H20" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I20" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J20" s="28" t="inlineStr"/>
+      <c r="K20" s="27" t="inlineStr"/>
+      <c r="L20" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M20" s="26">
+        <f>IF(OR(H20="not started",H20="partial",H20="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="54" customHeight="1" s="17">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>SB-13</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>Changelog</t>
+        </is>
+      </c>
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>Sidebar</t>
+        </is>
+      </c>
+      <c r="D21" s="27" t="inlineStr">
+        <is>
+          <t>Sidebar owns a public changelog and package changelog entry.</t>
+        </is>
+      </c>
+      <c r="E21" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F21" s="26" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="G21" s="27" t="inlineStr">
+        <is>
+          <t>../docs/components/sidebar/CHANGELOG.md; ../CHANGELOG.md</t>
+        </is>
+      </c>
+      <c r="H21" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I21" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J21" s="28" t="inlineStr"/>
+      <c r="K21" s="27" t="inlineStr"/>
+      <c r="L21" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M21" s="26">
+        <f>IF(OR(H21="not started",H21="partial",H21="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="54" customHeight="1" s="17">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>SB-14</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>Sidebar</t>
+        </is>
+      </c>
+      <c r="D22" s="27" t="inlineStr">
+        <is>
+          <t>The packed Consumer proves public Sidebar with Nav List and an external Trigger.</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>consumer</t>
+        </is>
+      </c>
+      <c r="F22" s="26" t="inlineStr">
+        <is>
+          <t>consumer</t>
+        </is>
+      </c>
+      <c r="G22" s="27" t="inlineStr">
+        <is>
+          <t>../apps/consumer/src/App.tsx; ../apps/consumer/tests/consumer.spec.ts</t>
+        </is>
+      </c>
+      <c r="H22" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I22" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J22" s="28" t="inlineStr"/>
+      <c r="K22" s="27" t="inlineStr"/>
+      <c r="L22" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" s="26">
+        <f>IF(OR(H22="not started",H22="partial",H22="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="54" customHeight="1" s="17">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>SB-15</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="C23" s="26" t="inlineStr">
+        <is>
+          <t>Adoption</t>
+        </is>
+      </c>
+      <c r="D23" s="27" t="inlineStr">
+        <is>
+          <t>The route covers all scenarios and desktop shell adopts Sidebar while mobile Drawer policy remains application-owned.</t>
+        </is>
+      </c>
+      <c r="E23" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F23" s="26" t="inlineStr">
+        <is>
+          <t>adoption</t>
+        </is>
+      </c>
+      <c r="G23" s="27" t="inlineStr">
+        <is>
+          <t>../scripts/verify-playground-sidebar.mjs</t>
+        </is>
+      </c>
+      <c r="H23" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I23" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J23" s="28" t="inlineStr"/>
+      <c r="K23" s="27" t="inlineStr"/>
+      <c r="L23" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M23" s="26">
+        <f>IF(OR(H23="not started",H23="partial",H23="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="54" customHeight="1" s="17">
+      <c r="A24" s="26" t="inlineStr">
+        <is>
+          <t>SB-16</t>
+        </is>
+      </c>
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>Package</t>
+        </is>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>Sidebar</t>
+        </is>
+      </c>
+      <c r="D24" s="27" t="inlineStr">
+        <is>
+          <t>Build, SSR, exports, CSS, Atom dependency, tarball, consumers, browser matrix, and adoption pass.</t>
+        </is>
+      </c>
+      <c r="E24" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F24" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="G24" s="27" t="inlineStr">
+        <is>
+          <t>../test/package/package.test.mjs; ../test/package/ssr.test.mjs</t>
+        </is>
+      </c>
+      <c r="H24" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I24" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J24" s="28" t="inlineStr"/>
+      <c r="K24" s="27" t="inlineStr"/>
+      <c r="L24" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M24" s="26">
+        <f>IF(OR(H24="not started",H24="partial",H24="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="54" customHeight="1" s="17">
+      <c r="A25" s="26" t="n"/>
+      <c r="B25" s="26" t="n"/>
+      <c r="C25" s="26" t="n"/>
+      <c r="D25" s="27" t="n"/>
+      <c r="E25" s="26" t="n"/>
+      <c r="F25" s="26" t="n"/>
+      <c r="G25" s="27" t="n"/>
+      <c r="H25" s="26" t="n"/>
+      <c r="I25" s="26" t="n"/>
+      <c r="J25" s="28" t="n"/>
+      <c r="K25" s="27" t="n"/>
+      <c r="L25" s="26" t="n"/>
+      <c r="M25" s="26" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">

</xml_diff>

<commit_message>
feat: add Icon component
</commit_message>
<xml_diff>
--- a/playground/component-coverage.xlsx
+++ b/playground/component-coverage.xlsx
@@ -43,9 +43,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Block" sheetId="34" state="visible" r:id="rId34"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nav List" sheetId="35" state="visible" r:id="rId35"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sidebar" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Icon" sheetId="37" state="visible" r:id="rId37"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$7:$M$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$8:$M$41</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Index'!$A$1:$M$35</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001" forceFullCalc="1"/>
@@ -1102,7 +1103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M40"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="24.71" customWidth="1" style="23" min="1" max="1"/>
@@ -3045,8 +3046,63 @@
         <v/>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="23" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="B41" s="23">
+        <f>INDIRECT("'"&amp;A41&amp;"'!B4")</f>
+        <v/>
+      </c>
+      <c r="C41" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A41&amp;"'!H9:H200"),"not started")</f>
+        <v/>
+      </c>
+      <c r="D41" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A41&amp;"'!H9:H200"),"partial")</f>
+        <v/>
+      </c>
+      <c r="E41" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A41&amp;"'!H9:H200"),"implemented")</f>
+        <v/>
+      </c>
+      <c r="F41" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A41&amp;"'!H9:H200"),"tested")</f>
+        <v/>
+      </c>
+      <c r="G41" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A41&amp;"'!H9:H200"),"verified")</f>
+        <v/>
+      </c>
+      <c r="H41" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A41&amp;"'!H9:H200"),"blocked")</f>
+        <v/>
+      </c>
+      <c r="I41" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A41&amp;"'!H9:H200"),"not applicable")</f>
+        <v/>
+      </c>
+      <c r="J41" s="24">
+        <f>INDIRECT("'"&amp;A41&amp;"'!H4")</f>
+        <v/>
+      </c>
+      <c r="K41" s="23">
+        <f>INDIRECT("'"&amp;A41&amp;"'!K4")</f>
+        <v/>
+      </c>
+      <c r="L41" s="23">
+        <f>INDIRECT("'"&amp;A41&amp;"'!E5")</f>
+        <v/>
+      </c>
+      <c r="M41" s="23">
+        <f>IF(AND(J41=1,K41="complete",L41="complete"),"complete",IF(H41&gt;0,"blocked","open"))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A7:M38"/>
+  <autoFilter ref="A8:M41"/>
   <mergeCells count="2">
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A1:M1"/>
@@ -34230,6 +34286,1142 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:M25"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.71" customWidth="1" style="23" min="1" max="1"/>
+    <col width="15.71" customWidth="1" style="23" min="2" max="2"/>
+    <col width="18.71" customWidth="1" style="23" min="3" max="3"/>
+    <col width="58.71" customWidth="1" style="23" min="4" max="4"/>
+    <col width="14.71" customWidth="1" style="23" min="5" max="6"/>
+    <col width="50.71" customWidth="1" style="23" min="7" max="7"/>
+    <col width="17.71" customWidth="1" style="23" min="8" max="8"/>
+    <col width="14.71" customWidth="1" style="23" min="9" max="9"/>
+    <col width="14.71" customWidth="1" style="25" min="10" max="10"/>
+    <col width="42.71" customWidth="1" style="23" min="11" max="11"/>
+    <col width="10.71" customWidth="1" style="23" min="12" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="37.5" customHeight="1" s="17">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Icon Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="27.75" customHeight="1" s="17">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Assertion-level SVG presentation, accessibility, recipes, browser, human-review, documentation, Consumer, and scoped adoption evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="17.25" customHeight="1" s="17">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>Requirements</t>
+        </is>
+      </c>
+      <c r="B4" s="21">
+        <f>COUNTA(A9:A25)</f>
+        <v/>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="E4" s="21">
+        <f>SUM(M9:M25)</f>
+        <v/>
+      </c>
+      <c r="G4" s="20" t="inlineStr">
+        <is>
+          <t>Completion</t>
+        </is>
+      </c>
+      <c r="H4" s="22">
+        <f>IF(B4=0,0,E4/B4)</f>
+        <v/>
+      </c>
+      <c r="J4" s="20" t="inlineStr">
+        <is>
+          <t>Package gate</t>
+        </is>
+      </c>
+      <c r="K4" s="21">
+        <f>IF(COUNTIFS(E9:E25,"package",M9:M25,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="17.25" customHeight="1" s="17">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Manual review</t>
+        </is>
+      </c>
+      <c r="B5" s="21">
+        <f>IF(COUNTIFS(I9:I25,"yes",M9:M25,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>Consumer gate</t>
+        </is>
+      </c>
+      <c r="E5" s="21">
+        <f>IF(COUNTIFS(E9:E25,"consumer",M9:M25,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="17">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="inlineStr">
+        <is>
+          <t>Evidence type</t>
+        </is>
+      </c>
+      <c r="G8" s="23" t="inlineStr">
+        <is>
+          <t>Evidence / link</t>
+        </is>
+      </c>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>Human review?</t>
+        </is>
+      </c>
+      <c r="J8" s="25" t="inlineStr">
+        <is>
+          <t>Last verified</t>
+        </is>
+      </c>
+      <c r="K8" s="23" t="inlineStr">
+        <is>
+          <t>Blocker / N/A reason</t>
+        </is>
+      </c>
+      <c r="L8" s="23" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="M8" s="23" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="54" customHeight="1" s="17">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>IC-01</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="inlineStr">
+        <is>
+          <t>Default wrapper and SVG-only asChild composition preserve one source graphic with deterministic props and ref.</t>
+        </is>
+      </c>
+      <c r="E9" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F9" s="26" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="G9" s="27" t="inlineStr">
+        <is>
+          <t>../src/components/icon</t>
+        </is>
+      </c>
+      <c r="H9" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I9" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J9" s="28" t="n"/>
+      <c r="K9" s="27" t="n"/>
+      <c r="L9" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" s="26">
+        <f>IF(OR(H9="not started",H9="partial",H9="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="54" customHeight="1" s="17">
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>IC-02</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>Decorative default, direct label, and label-reference modes emit mutually exclusive native image semantics.</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F10" s="26" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="G10" s="27" t="inlineStr">
+        <is>
+          <t>../test/components/icon/icon.test.tsx</t>
+        </is>
+      </c>
+      <c r="H10" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I10" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J10" s="28" t="n"/>
+      <c r="K10" s="27" t="n"/>
+      <c r="L10" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" s="26">
+        <f>IF(OR(H10="not started",H10="partial",H10="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1" s="17">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>IC-03</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>Recipes</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D11" s="27" t="inlineStr">
+        <is>
+          <t>Six sizes, nine semantic tones, default medium inherited presentation, and currentColor remain exact.</t>
+        </is>
+      </c>
+      <c r="E11" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F11" s="26" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+      <c r="G11" s="27" t="inlineStr">
+        <is>
+          <t>../playground/tests/components/icon/behavior.spec.ts</t>
+        </is>
+      </c>
+      <c r="H11" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I11" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J11" s="28" t="n"/>
+      <c r="K11" s="27" t="n"/>
+      <c r="L11" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" s="26">
+        <f>IF(OR(H11="not started",H11="partial",H11="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="54" customHeight="1" s="17">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>IC-04</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D12" s="27" t="inlineStr">
+        <is>
+          <t>Only directional icons mirror in genuine RTL; non-directional sources retain identity.</t>
+        </is>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+      <c r="G12" s="27" t="inlineStr">
+        <is>
+          <t>../playground/tests/components/icon/behavior.spec.ts</t>
+        </is>
+      </c>
+      <c r="H12" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I12" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J12" s="28" t="n"/>
+      <c r="K12" s="27" t="n"/>
+      <c r="L12" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" s="26">
+        <f>IF(OR(H12="not started",H12="partial",H12="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="54" customHeight="1" s="17">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>IC-05</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>Sources</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>Graphic</t>
+        </is>
+      </c>
+      <c r="D13" s="27" t="inlineStr">
+        <is>
+          <t>Inline, reusable React SVG, external-library-shaped, and fixed multicolor sources preserve authored geometry and fills.</t>
+        </is>
+      </c>
+      <c r="E13" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F13" s="26" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+      <c r="G13" s="27" t="inlineStr">
+        <is>
+          <t>../playground/src/components/icon/IconPage.tsx</t>
+        </is>
+      </c>
+      <c r="H13" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I13" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J13" s="28" t="n"/>
+      <c r="K13" s="27" t="n"/>
+      <c r="L13" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" s="26">
+        <f>IF(OR(H13="not started",H13="partial",H13="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="54" customHeight="1" s="17">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>IC-06</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>Composition</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>Native props, classes, styles, slot override, wrapper-free SVG, and ref composition preserve output.</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F14" s="26" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="G14" s="27" t="inlineStr">
+        <is>
+          <t>../test/components/icon/icon.test.tsx</t>
+        </is>
+      </c>
+      <c r="H14" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I14" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J14" s="28" t="n"/>
+      <c r="K14" s="27" t="n"/>
+      <c r="L14" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" s="26">
+        <f>IF(OR(H14="not started",H14="partial",H14="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="54" customHeight="1" s="17">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>IC-07</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>Exports</t>
+        </is>
+      </c>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D15" s="27" t="inlineStr">
+        <is>
+          <t>Root and Icon subpath exports expose runtime and public types.</t>
+        </is>
+      </c>
+      <c r="E15" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F15" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="G15" s="27" t="inlineStr">
+        <is>
+          <t>../test/package/package.test.mjs</t>
+        </is>
+      </c>
+      <c r="H15" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I15" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J15" s="28" t="n"/>
+      <c r="K15" s="27" t="n"/>
+      <c r="L15" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" s="26">
+        <f>IF(OR(H15="not started",H15="partial",H15="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="54" customHeight="1" s="17">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>IC-08</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>Types</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D16" s="27" t="inlineStr">
+        <is>
+          <t>Closed recipes and mutually exclusive accessibility modes reject invalid hosts, colors, sizes, and label combinations.</t>
+        </is>
+      </c>
+      <c r="E16" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F16" s="26" t="inlineStr">
+        <is>
+          <t>types</t>
+        </is>
+      </c>
+      <c r="G16" s="27" t="inlineStr">
+        <is>
+          <t>../test/types/components/icon.test.ts</t>
+        </is>
+      </c>
+      <c r="H16" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I16" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J16" s="28" t="n"/>
+      <c r="K16" s="27" t="n"/>
+      <c r="L16" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" s="26">
+        <f>IF(OR(H16="not started",H16="partial",H16="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="54" customHeight="1" s="17">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>IC-09</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>CSS</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D17" s="27" t="inlineStr">
+        <is>
+          <t>Static CSS ships sizing, semantic foregrounds, direction, forced colors, and documented public properties.</t>
+        </is>
+      </c>
+      <c r="E17" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F17" s="26" t="inlineStr">
+        <is>
+          <t>css</t>
+        </is>
+      </c>
+      <c r="G17" s="27" t="inlineStr">
+        <is>
+          <t>../src/components/icon/icon.css</t>
+        </is>
+      </c>
+      <c r="H17" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I17" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J17" s="28" t="n"/>
+      <c r="K17" s="27" t="n"/>
+      <c r="L17" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" s="26">
+        <f>IF(OR(H17="not started",H17="partial",H17="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="54" customHeight="1" s="17">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>IC-10</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D18" s="27" t="inlineStr">
+        <is>
+          <t>Defaults, sizes, tones, sources, direction, appearance, stress, and forced colors own reviewable baselines.</t>
+        </is>
+      </c>
+      <c r="E18" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F18" s="26" t="inlineStr">
+        <is>
+          <t>visual</t>
+        </is>
+      </c>
+      <c r="G18" s="27" t="inlineStr">
+        <is>
+          <t>../playground/tests/components/icon/visual.spec.ts</t>
+        </is>
+      </c>
+      <c r="H18" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I18" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J18" s="28" t="n"/>
+      <c r="K18" s="27" t="inlineStr">
+        <is>
+          <t>Human run pending.</t>
+        </is>
+      </c>
+      <c r="L18" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="26">
+        <f>IF(OR(H18="not started",H18="partial",H18="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="54" customHeight="1" s="17">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>IC-11</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>Responsive</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>Narrow frames, large sizes, long referenced labels, zoom, text spacing, and mobile widths remain contained.</t>
+        </is>
+      </c>
+      <c r="E19" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F19" s="26" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G19" s="27" t="inlineStr">
+        <is>
+          <t>../playground/manual-tests/icon.md</t>
+        </is>
+      </c>
+      <c r="H19" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I19" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J19" s="28" t="n"/>
+      <c r="K19" s="27" t="inlineStr">
+        <is>
+          <t>Human run pending.</t>
+        </is>
+      </c>
+      <c r="L19" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" s="26">
+        <f>IF(OR(H19="not started",H19="partial",H19="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="54" customHeight="1" s="17">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>IC-12</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="inlineStr">
+        <is>
+          <t>The concise protocol covers every Icon playground scenario and assistive-technology mode.</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F20" s="26" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G20" s="27" t="inlineStr">
+        <is>
+          <t>../playground/manual-tests/icon.md</t>
+        </is>
+      </c>
+      <c r="H20" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I20" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J20" s="28" t="n"/>
+      <c r="K20" s="27" t="inlineStr">
+        <is>
+          <t>Human run pending.</t>
+        </is>
+      </c>
+      <c r="L20" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M20" s="26">
+        <f>IF(OR(H20="not started",H20="partial",H20="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="54" customHeight="1" s="17">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>IC-13</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D21" s="27" t="inlineStr">
+        <is>
+          <t>Source-backed ownership, SVG boundary, accessibility, API, recipes, tokens, and composition pass.</t>
+        </is>
+      </c>
+      <c r="E21" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F21" s="26" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="G21" s="27" t="inlineStr">
+        <is>
+          <t>../docs/components/icon/README.md</t>
+        </is>
+      </c>
+      <c r="H21" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I21" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J21" s="28" t="n"/>
+      <c r="K21" s="27" t="n"/>
+      <c r="L21" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M21" s="26">
+        <f>IF(OR(H21="not started",H21="partial",H21="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="54" customHeight="1" s="17">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>IC-14</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>Changelog</t>
+        </is>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D22" s="27" t="inlineStr">
+        <is>
+          <t>Icon owns a public changelog and package changelog entry.</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F22" s="26" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="G22" s="27" t="inlineStr">
+        <is>
+          <t>../docs/components/icon/CHANGELOG.md; ../CHANGELOG.md</t>
+        </is>
+      </c>
+      <c r="H22" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I22" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J22" s="28" t="n"/>
+      <c r="K22" s="27" t="n"/>
+      <c r="L22" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" s="26">
+        <f>IF(OR(H22="not started",H22="partial",H22="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="54" customHeight="1" s="17">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>IC-15</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="C23" s="26" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D23" s="27" t="inlineStr">
+        <is>
+          <t>The Consumer proves the public Icon subpath inside a named IconButton.</t>
+        </is>
+      </c>
+      <c r="E23" s="26" t="inlineStr">
+        <is>
+          <t>consumer</t>
+        </is>
+      </c>
+      <c r="F23" s="26" t="inlineStr">
+        <is>
+          <t>consumer</t>
+        </is>
+      </c>
+      <c r="G23" s="27" t="inlineStr">
+        <is>
+          <t>../apps/consumer/src/App.tsx; ../apps/consumer/tests/consumer.spec.ts</t>
+        </is>
+      </c>
+      <c r="H23" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I23" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J23" s="28" t="n"/>
+      <c r="K23" s="27" t="n"/>
+      <c r="L23" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M23" s="26">
+        <f>IF(OR(H23="not started",H23="partial",H23="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="54" customHeight="1" s="17">
+      <c r="A24" s="26" t="inlineStr">
+        <is>
+          <t>IC-16</t>
+        </is>
+      </c>
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>Adoption</t>
+        </is>
+      </c>
+      <c r="D24" s="27" t="inlineStr">
+        <is>
+          <t>The route covers all scenarios and shell adoption follows explicit component-owned exclusions.</t>
+        </is>
+      </c>
+      <c r="E24" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F24" s="26" t="inlineStr">
+        <is>
+          <t>adoption</t>
+        </is>
+      </c>
+      <c r="G24" s="27" t="inlineStr">
+        <is>
+          <t>../scripts/verify-playground-icon.mjs; ../playground/docs/icon-adoption-audit.md</t>
+        </is>
+      </c>
+      <c r="H24" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I24" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J24" s="28" t="n"/>
+      <c r="K24" s="27" t="n"/>
+      <c r="L24" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M24" s="26">
+        <f>IF(OR(H24="not started",H24="partial",H24="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="54" customHeight="1" s="17">
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t>IC-17</t>
+        </is>
+      </c>
+      <c r="B25" s="26" t="inlineStr">
+        <is>
+          <t>Package</t>
+        </is>
+      </c>
+      <c r="C25" s="26" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="D25" s="27" t="inlineStr">
+        <is>
+          <t>Build, SSR-safe import, exports, CSS, tarball, Consumer, browser, and adoption checks pass.</t>
+        </is>
+      </c>
+      <c r="E25" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F25" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="G25" s="27" t="inlineStr">
+        <is>
+          <t>../test/package/package.test.mjs</t>
+        </is>
+      </c>
+      <c r="H25" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I25" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J25" s="28" t="n"/>
+      <c r="K25" s="27" t="n"/>
+      <c r="L25" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M25" s="26">
+        <f>IF(OR(H25="not started",H25="partial",H25="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">

</xml_diff>

<commit_message>
feat: add Image component
</commit_message>
<xml_diff>
--- a/playground/component-coverage.xlsx
+++ b/playground/component-coverage.xlsx
@@ -44,6 +44,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nav List" sheetId="35" state="visible" r:id="rId35"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sidebar" sheetId="36" state="visible" r:id="rId36"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Icon" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Image" sheetId="38" state="visible" r:id="rId38"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$8:$M$41</definedName>
@@ -1103,7 +1104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:M42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="24.71" customWidth="1" style="23" min="1" max="1"/>
@@ -3098,6 +3099,61 @@
       </c>
       <c r="M41" s="23">
         <f>IF(AND(J41=1,K41="complete",L41="complete"),"complete",IF(H41&gt;0,"blocked","open"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="23" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="B42" s="23">
+        <f>INDIRECT("'"&amp;A42&amp;"'!B4")</f>
+        <v/>
+      </c>
+      <c r="C42" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A42&amp;"'!H9:H200"),"not started")</f>
+        <v/>
+      </c>
+      <c r="D42" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A42&amp;"'!H9:H200"),"partial")</f>
+        <v/>
+      </c>
+      <c r="E42" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A42&amp;"'!H9:H200"),"implemented")</f>
+        <v/>
+      </c>
+      <c r="F42" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A42&amp;"'!H9:H200"),"tested")</f>
+        <v/>
+      </c>
+      <c r="G42" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A42&amp;"'!H9:H200"),"verified")</f>
+        <v/>
+      </c>
+      <c r="H42" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A42&amp;"'!H9:H200"),"blocked")</f>
+        <v/>
+      </c>
+      <c r="I42" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A42&amp;"'!H9:H200"),"not applicable")</f>
+        <v/>
+      </c>
+      <c r="J42" s="24">
+        <f>INDIRECT("'"&amp;A42&amp;"'!H4")</f>
+        <v/>
+      </c>
+      <c r="K42" s="23">
+        <f>INDIRECT("'"&amp;A42&amp;"'!K4")</f>
+        <v/>
+      </c>
+      <c r="L42" s="23">
+        <f>INDIRECT("'"&amp;A42&amp;"'!E5")</f>
+        <v/>
+      </c>
+      <c r="M42" s="23">
+        <f>IF(AND(J42=1,K42="complete",L42="complete"),"complete",IF(H42&gt;0,"blocked","open"))</f>
         <v/>
       </c>
     </row>
@@ -35422,6 +35478,1592 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:M200"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.71" customWidth="1" style="23" min="1" max="1"/>
+    <col width="15.71" customWidth="1" style="23" min="2" max="2"/>
+    <col width="18.71" customWidth="1" style="23" min="3" max="3"/>
+    <col width="58.71" customWidth="1" style="23" min="4" max="4"/>
+    <col width="14.71" customWidth="1" style="23" min="5" max="6"/>
+    <col width="50.71" customWidth="1" style="23" min="7" max="7"/>
+    <col width="17.71" customWidth="1" style="23" min="8" max="8"/>
+    <col width="14.71" customWidth="1" style="23" min="9" max="9"/>
+    <col width="14.71" customWidth="1" style="25" min="10" max="10"/>
+    <col width="42.71" customWidth="1" style="23" min="11" max="11"/>
+    <col width="10.71" customWidth="1" style="23" min="12" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="37.5" customHeight="1" s="17">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Image Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="27.75" customHeight="1" s="17">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Assertion-level media lifecycle, accessibility, recipes, native output, browser, human-review, documentation, Consumer, and scoped adoption evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="17.25" customHeight="1" s="17">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>Requirements</t>
+        </is>
+      </c>
+      <c r="B4" s="21">
+        <f>COUNTA(A9:A30)</f>
+        <v/>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="E4" s="21">
+        <f>SUM(M9:M30)</f>
+        <v/>
+      </c>
+      <c r="G4" s="20" t="inlineStr">
+        <is>
+          <t>Completion</t>
+        </is>
+      </c>
+      <c r="H4" s="22">
+        <f>IF(B4=0,0,E4/B4)</f>
+        <v/>
+      </c>
+      <c r="J4" s="20" t="inlineStr">
+        <is>
+          <t>Package gate</t>
+        </is>
+      </c>
+      <c r="K4" s="21">
+        <f>IF(COUNTIFS(E9:E25,"package",M9:M25,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="17.25" customHeight="1" s="17">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Manual review</t>
+        </is>
+      </c>
+      <c r="B5" s="21">
+        <f>IF(COUNTIFS(I9:I30,"yes",M9:M30,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>Consumer gate</t>
+        </is>
+      </c>
+      <c r="E5" s="21">
+        <f>IF(COUNTIFS(E9:E30,"consumer",M9:M30,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="17">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="inlineStr">
+        <is>
+          <t>Evidence type</t>
+        </is>
+      </c>
+      <c r="G8" s="23" t="inlineStr">
+        <is>
+          <t>Evidence / link</t>
+        </is>
+      </c>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>Human review?</t>
+        </is>
+      </c>
+      <c r="J8" s="25" t="inlineStr">
+        <is>
+          <t>Last verified</t>
+        </is>
+      </c>
+      <c r="K8" s="23" t="inlineStr">
+        <is>
+          <t>Blocker / N/A reason</t>
+        </is>
+      </c>
+      <c r="L8" s="23" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="M8" s="23" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="54" customHeight="1" s="17">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>IM-01</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>Root / Content / Fallback</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="inlineStr">
+        <is>
+          <t>Atom Image anatomy is styled without replacing source lifecycle, refs, or conditional parts.</t>
+        </is>
+      </c>
+      <c r="E9" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F9" s="26" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="G9" s="27" t="inlineStr">
+        <is>
+          <t>../src/components/image</t>
+        </is>
+      </c>
+      <c r="H9" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I9" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J9" s="28" t="n"/>
+      <c r="K9" s="27" t="n"/>
+      <c r="L9" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" s="26">
+        <f>IF(OR(H9="not started",H9="partial",H9="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="54" customHeight="1" s="17">
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>IM-02</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>Source state</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>Idle, loading, loaded, error, source replacement, and stale-event rejection remain Atom-owned and observable.</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F10" s="26" t="inlineStr">
+        <is>
+          <t>atom</t>
+        </is>
+      </c>
+      <c r="G10" s="27" t="inlineStr">
+        <is>
+          <t>@flowstack-ui/atom@0.9.0 Image tests; ../test/components/image/image.test.tsx</t>
+        </is>
+      </c>
+      <c r="H10" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I10" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J10" s="28" t="n"/>
+      <c r="K10" s="27" t="n"/>
+      <c r="L10" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" s="26">
+        <f>IF(OR(H10="not started",H10="partial",H10="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1" s="17">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>IM-03</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>Native output</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D11" s="27" t="inlineStr">
+        <is>
+          <t>Required authored alt plus intrinsic, responsive, loading, decoding, priority, event, slot, and ref props reach the native image.</t>
+        </is>
+      </c>
+      <c r="E11" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F11" s="26" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="G11" s="27" t="inlineStr">
+        <is>
+          <t>../test/components/image/image.test.tsx; ../playground/tests/components/image/behavior.spec.ts</t>
+        </is>
+      </c>
+      <c r="H11" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I11" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J11" s="28" t="n"/>
+      <c r="K11" s="27" t="n"/>
+      <c r="L11" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" s="26">
+        <f>IF(OR(H11="not started",H11="partial",H11="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="54" customHeight="1" s="17">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>IM-04</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>Fallback</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>Fallback</t>
+        </is>
+      </c>
+      <c r="D12" s="27" t="inlineStr">
+        <is>
+          <t>Authored idle, loading, and error fallbacks are mutually exclusive with Content and preserve reserved geometry.</t>
+        </is>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+      <c r="G12" s="27" t="inlineStr">
+        <is>
+          <t>../playground/tests/components/image/behavior.spec.ts</t>
+        </is>
+      </c>
+      <c r="H12" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I12" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J12" s="28" t="n"/>
+      <c r="K12" s="27" t="n"/>
+      <c r="L12" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" s="26">
+        <f>IF(OR(H12="not started",H12="partial",H12="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="54" customHeight="1" s="17">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>IM-05</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D13" s="27" t="inlineStr">
+        <is>
+          <t>Cover, contain, fill, none, and scale-down change only object fit inside controlled fixtures.</t>
+        </is>
+      </c>
+      <c r="E13" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F13" s="26" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+      <c r="G13" s="27" t="inlineStr">
+        <is>
+          <t>../playground/tests/components/image/behavior.spec.ts</t>
+        </is>
+      </c>
+      <c r="H13" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I13" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J13" s="28" t="n"/>
+      <c r="K13" s="27" t="n"/>
+      <c r="L13" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" s="26">
+        <f>IF(OR(H13="not started",H13="partial",H13="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="54" customHeight="1" s="17">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>IM-06</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>Center, top, bottom, logical start, and logical end move focal content; start/end reverse in RTL without mirroring pixels.</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F14" s="26" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+      <c r="G14" s="27" t="inlineStr">
+        <is>
+          <t>../playground/tests/components/image/behavior.spec.ts</t>
+        </is>
+      </c>
+      <c r="H14" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I14" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J14" s="28" t="n"/>
+      <c r="K14" s="27" t="n"/>
+      <c r="L14" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" s="26">
+        <f>IF(OR(H14="not started",H14="partial",H14="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="54" customHeight="1" s="17">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>IM-07</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>Geometry</t>
+        </is>
+      </c>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="D15" s="27" t="inlineStr">
+        <is>
+          <t>Five radius recipes, transparent/subtle frame, and explicit Atom Aspect Ratio preserve one clipped media box.</t>
+        </is>
+      </c>
+      <c r="E15" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F15" s="26" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+      <c r="G15" s="27" t="inlineStr">
+        <is>
+          <t>../playground/tests/components/image/behavior.spec.ts</t>
+        </is>
+      </c>
+      <c r="H15" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I15" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J15" s="28" t="n"/>
+      <c r="K15" s="27" t="n"/>
+      <c r="L15" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" s="26">
+        <f>IF(OR(H15="not started",H15="partial",H15="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="54" customHeight="1" s="17">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>IM-08</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>Content / Fallback</t>
+        </is>
+      </c>
+      <c r="D16" s="27" t="inlineStr">
+        <is>
+          <t>Informative, decorative, and named-action alt ownership is explicit; fallback adds no focus or live-region policy.</t>
+        </is>
+      </c>
+      <c r="E16" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F16" s="26" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+      <c r="G16" s="27" t="inlineStr">
+        <is>
+          <t>../playground/tests/components/image/behavior.spec.ts</t>
+        </is>
+      </c>
+      <c r="H16" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I16" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J16" s="28" t="n"/>
+      <c r="K16" s="27" t="n"/>
+      <c r="L16" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" s="26">
+        <f>IF(OR(H16="not started",H16="partial",H16="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="54" customHeight="1" s="17">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>IM-09</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>Composition</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>All parts</t>
+        </is>
+      </c>
+      <c r="D17" s="27" t="inlineStr">
+        <is>
+          <t>Default, asChild, render, native props, custom slots, styles, and refs preserve Atom composition and valid hosts.</t>
+        </is>
+      </c>
+      <c r="E17" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F17" s="26" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="G17" s="27" t="inlineStr">
+        <is>
+          <t>../test/components/image/image.test.tsx</t>
+        </is>
+      </c>
+      <c r="H17" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I17" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J17" s="28" t="n"/>
+      <c r="K17" s="27" t="n"/>
+      <c r="L17" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" s="26">
+        <f>IF(OR(H17="not started",H17="partial",H17="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="54" customHeight="1" s="17">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>IM-10</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>Exports</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D18" s="27" t="inlineStr">
+        <is>
+          <t>Package root and Image subpath expose one runtime namespace and public types.</t>
+        </is>
+      </c>
+      <c r="E18" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F18" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="G18" s="27" t="inlineStr">
+        <is>
+          <t>../test/package/package.test.mjs</t>
+        </is>
+      </c>
+      <c r="H18" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I18" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J18" s="28" t="n"/>
+      <c r="K18" s="27" t="n"/>
+      <c r="L18" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="26">
+        <f>IF(OR(H18="not started",H18="partial",H18="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="54" customHeight="1" s="17">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>IM-11</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>Types</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>Required alt, closed recipes, root source ownership, native responsive props, and refs are enforced.</t>
+        </is>
+      </c>
+      <c r="E19" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F19" s="26" t="inlineStr">
+        <is>
+          <t>types</t>
+        </is>
+      </c>
+      <c r="G19" s="27" t="inlineStr">
+        <is>
+          <t>../test/types/components/image.test.ts</t>
+        </is>
+      </c>
+      <c r="H19" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I19" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J19" s="28" t="n"/>
+      <c r="K19" s="27" t="n"/>
+      <c r="L19" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" s="26">
+        <f>IF(OR(H19="not started",H19="partial",H19="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="54" customHeight="1" s="17">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>IM-12</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>CSS</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="inlineStr">
+        <is>
+          <t>Static CSS ships fit, logical position, clipping, frame, fallback, forced colors, and documented public properties.</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F20" s="26" t="inlineStr">
+        <is>
+          <t>css</t>
+        </is>
+      </c>
+      <c r="G20" s="27" t="inlineStr">
+        <is>
+          <t>../src/components/image/image.css</t>
+        </is>
+      </c>
+      <c r="H20" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I20" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J20" s="28" t="n"/>
+      <c r="K20" s="27" t="n"/>
+      <c r="L20" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M20" s="26">
+        <f>IF(OR(H20="not started",H20="partial",H20="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="54" customHeight="1" s="17">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>IM-13</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>SSR</t>
+        </is>
+      </c>
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D21" s="27" t="inlineStr">
+        <is>
+          <t>Idle/loading fallback output and recipe metadata render deterministically without a CSS loader.</t>
+        </is>
+      </c>
+      <c r="E21" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F21" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="G21" s="27" t="inlineStr">
+        <is>
+          <t>../test/package/ssr.test.mjs</t>
+        </is>
+      </c>
+      <c r="H21" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I21" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J21" s="28" t="n"/>
+      <c r="K21" s="27" t="n"/>
+      <c r="L21" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M21" s="26">
+        <f>IF(OR(H21="not started",H21="partial",H21="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="54" customHeight="1" s="17">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>IM-14</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D22" s="27" t="inlineStr">
+        <is>
+          <t>Nine numbered scenarios cover defaults, accessibility, fits, positions, geometry, native output, states, appearance, and stress.</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F22" s="26" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+      <c r="G22" s="27" t="inlineStr">
+        <is>
+          <t>../playground/src/components/image/ImagePage.tsx; ../playground/tests/components/image/behavior.spec.ts</t>
+        </is>
+      </c>
+      <c r="H22" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I22" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J22" s="28" t="n"/>
+      <c r="K22" s="27" t="n"/>
+      <c r="L22" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" s="26">
+        <f>IF(OR(H22="not started",H22="partial",H22="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="54" customHeight="1" s="17">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>IM-15</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C23" s="26" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D23" s="27" t="inlineStr">
+        <is>
+          <t>Defaults, fits, positions, geometry, fallback, appearance, mobile, and forced colors own reviewed-risk baselines.</t>
+        </is>
+      </c>
+      <c r="E23" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F23" s="26" t="inlineStr">
+        <is>
+          <t>visual</t>
+        </is>
+      </c>
+      <c r="G23" s="27" t="inlineStr">
+        <is>
+          <t>../playground/tests/components/image/visual.spec.ts</t>
+        </is>
+      </c>
+      <c r="H23" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I23" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J23" s="28" t="n"/>
+      <c r="K23" s="27" t="inlineStr">
+        <is>
+          <t>Owner manual review pending.</t>
+        </is>
+      </c>
+      <c r="L23" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M23" s="26">
+        <f>IF(OR(H23="not started",H23="partial",H23="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="54" customHeight="1" s="17">
+      <c r="A24" s="26" t="inlineStr">
+        <is>
+          <t>IM-16</t>
+        </is>
+      </c>
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>Responsive</t>
+        </is>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D24" s="27" t="inlineStr">
+        <is>
+          <t>Narrow, long fallback, RTL, mobile, zoom, text spacing, and physical-device containment are reviewed.</t>
+        </is>
+      </c>
+      <c r="E24" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F24" s="26" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G24" s="27" t="inlineStr">
+        <is>
+          <t>../playground/manual-tests/image.md</t>
+        </is>
+      </c>
+      <c r="H24" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I24" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J24" s="28" t="n"/>
+      <c r="K24" s="27" t="inlineStr">
+        <is>
+          <t>Owner manual review pending.</t>
+        </is>
+      </c>
+      <c r="L24" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M24" s="26">
+        <f>IF(OR(H24="not started",H24="partial",H24="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="54" customHeight="1" s="17">
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t>IM-17</t>
+        </is>
+      </c>
+      <c r="B25" s="26" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="C25" s="26" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D25" s="27" t="inlineStr">
+        <is>
+          <t>The concise protocol covers every Image scenario, source flow, appearance, device, and assistive-technology judgment.</t>
+        </is>
+      </c>
+      <c r="E25" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F25" s="26" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G25" s="27" t="inlineStr">
+        <is>
+          <t>../playground/manual-tests/image.md</t>
+        </is>
+      </c>
+      <c r="H25" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I25" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J25" s="28" t="n"/>
+      <c r="K25" s="27" t="inlineStr">
+        <is>
+          <t>Owner manual review pending.</t>
+        </is>
+      </c>
+      <c r="L25" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M25" s="26">
+        <f>IF(OR(H25="not started",H25="partial",H25="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="54" customHeight="1" s="17">
+      <c r="A26" s="26" t="inlineStr">
+        <is>
+          <t>IM-18</t>
+        </is>
+      </c>
+      <c r="B26" s="26" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C26" s="26" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D26" s="27" t="inlineStr">
+        <is>
+          <t>Source-backed ownership, alt guidance, API, recipes, native attrs, tokens, composition, and exclusions pass.</t>
+        </is>
+      </c>
+      <c r="E26" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F26" s="26" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="G26" s="27" t="inlineStr">
+        <is>
+          <t>../docs/components/image/README.md</t>
+        </is>
+      </c>
+      <c r="H26" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I26" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J26" s="28" t="n"/>
+      <c r="K26" s="27" t="n"/>
+      <c r="L26" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M26" s="26">
+        <f>IF(OR(H26="not started",H26="partial",H26="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="54" customHeight="1" s="17">
+      <c r="A27" s="26" t="inlineStr">
+        <is>
+          <t>IM-19</t>
+        </is>
+      </c>
+      <c r="B27" s="26" t="inlineStr">
+        <is>
+          <t>Changelog</t>
+        </is>
+      </c>
+      <c r="C27" s="26" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D27" s="27" t="inlineStr">
+        <is>
+          <t>Image owns a public changelog and package release-facing entry.</t>
+        </is>
+      </c>
+      <c r="E27" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F27" s="26" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="G27" s="27" t="inlineStr">
+        <is>
+          <t>../docs/components/image/CHANGELOG.md; ../CHANGELOG.md</t>
+        </is>
+      </c>
+      <c r="H27" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I27" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J27" s="28" t="n"/>
+      <c r="K27" s="27" t="n"/>
+      <c r="L27" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M27" s="26">
+        <f>IF(OR(H27="not started",H27="partial",H27="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="54" customHeight="1" s="17">
+      <c r="A28" s="26" t="inlineStr">
+        <is>
+          <t>IM-20</t>
+        </is>
+      </c>
+      <c r="B28" s="26" t="inlineStr">
+        <is>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="C28" s="26" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D28" s="27" t="inlineStr">
+        <is>
+          <t>Consumer proves the public Image subpath as informative project media inside Card on desktop and mobile.</t>
+        </is>
+      </c>
+      <c r="E28" s="26" t="inlineStr">
+        <is>
+          <t>consumer</t>
+        </is>
+      </c>
+      <c r="F28" s="26" t="inlineStr">
+        <is>
+          <t>consumer</t>
+        </is>
+      </c>
+      <c r="G28" s="27" t="inlineStr">
+        <is>
+          <t>../apps/consumer/src/App.tsx; ../apps/consumer/tests/consumer.spec.ts</t>
+        </is>
+      </c>
+      <c r="H28" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I28" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J28" s="28" t="n"/>
+      <c r="K28" s="27" t="n"/>
+      <c r="L28" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M28" s="26">
+        <f>IF(OR(H28="not started",H28="partial",H28="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="54" customHeight="1" s="17">
+      <c r="A29" s="26" t="inlineStr">
+        <is>
+          <t>IM-21</t>
+        </is>
+      </c>
+      <c r="B29" s="26" t="inlineStr">
+        <is>
+          <t>Adoption</t>
+        </is>
+      </c>
+      <c r="C29" s="26" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D29" s="27" t="inlineStr">
+        <is>
+          <t>Card finished media and Consumer adopt Image while Avatar and Icon Button native child evidence remain correctly owned.</t>
+        </is>
+      </c>
+      <c r="E29" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F29" s="26" t="inlineStr">
+        <is>
+          <t>adoption</t>
+        </is>
+      </c>
+      <c r="G29" s="27" t="inlineStr">
+        <is>
+          <t>../scripts/verify-playground-image.mjs; ../playground/docs/image-adoption-audit.md</t>
+        </is>
+      </c>
+      <c r="H29" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I29" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J29" s="28" t="n"/>
+      <c r="K29" s="27" t="n"/>
+      <c r="L29" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M29" s="26">
+        <f>IF(OR(H29="not started",H29="partial",H29="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="54" customHeight="1" s="17">
+      <c r="A30" s="26" t="inlineStr">
+        <is>
+          <t>IM-22</t>
+        </is>
+      </c>
+      <c r="B30" s="26" t="inlineStr">
+        <is>
+          <t>Package</t>
+        </is>
+      </c>
+      <c r="C30" s="26" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D30" s="27" t="inlineStr">
+        <is>
+          <t>Build, SSR, exports, CSS, archive, Consumer, browser, visual, docs, and adoption gates pass.</t>
+        </is>
+      </c>
+      <c r="E30" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F30" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="G30" s="27" t="inlineStr">
+        <is>
+          <t>../test/package/package.test.mjs</t>
+        </is>
+      </c>
+      <c r="H30" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I30" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J30" s="28" t="n"/>
+      <c r="K30" s="27" t="n"/>
+      <c r="L30" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M30" s="26">
+        <f>IF(OR(H30="not started",H30="partial",H30="implemented"),0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">

</xml_diff>

<commit_message>
feat: add List component
</commit_message>
<xml_diff>
--- a/playground/component-coverage.xlsx
+++ b/playground/component-coverage.xlsx
@@ -45,10 +45,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sidebar" sheetId="36" state="visible" r:id="rId36"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Icon" sheetId="37" state="visible" r:id="rId37"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Image" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="List" sheetId="39" ns1:id="rId39"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$8:$M$41</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Index'!$A$1:$M$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$7:$M$43</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Index'!$A$1:$M$43</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001" forceFullCalc="1"/>
 </workbook>
@@ -1104,7 +1105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M42"/>
+  <dimension ref="A1:M43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="24.71" customWidth="1" style="23" min="1" max="1"/>
@@ -1123,7 +1124,7 @@
     <row r="2" ht="27.75" customHeight="1" s="17">
       <c r="A2" s="19" t="inlineStr">
         <is>
-          <t>Current package evidence across 31 independently exported components.</t>
+          <t>Current package evidence across 36 independently exported components.</t>
         </is>
       </c>
     </row>
@@ -1134,7 +1135,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTA(A8:A36)</f>
+        <f>COUNTA(A8:A43)</f>
         <v/>
       </c>
       <c r="D4" s="20" t="inlineStr">
@@ -1143,7 +1144,7 @@
         </is>
       </c>
       <c r="E4" s="21">
-        <f>COUNTIF(M8:M36,"complete")</f>
+        <f>COUNTIF(M8:M43,"complete")</f>
         <v/>
       </c>
       <c r="G4" s="20" t="inlineStr">
@@ -1152,7 +1153,7 @@
         </is>
       </c>
       <c r="H4" s="21">
-        <f>COUNTIF(M8:M36,"blocked")</f>
+        <f>COUNTIF(M8:M43,"blocked")</f>
         <v/>
       </c>
       <c r="J4" s="20" t="inlineStr">
@@ -3157,8 +3158,63 @@
         <v/>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="23" t="inlineStr">
+        <is>
+          <t>List</t>
+        </is>
+      </c>
+      <c r="B43" s="23">
+        <f>INDIRECT("'"&amp;A43&amp;"'!B4")</f>
+        <v/>
+      </c>
+      <c r="C43" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A43&amp;"'!H9:H200"),"not started")</f>
+        <v/>
+      </c>
+      <c r="D43" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A43&amp;"'!H9:H200"),"partial")</f>
+        <v/>
+      </c>
+      <c r="E43" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A43&amp;"'!H9:H200"),"implemented")</f>
+        <v/>
+      </c>
+      <c r="F43" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A43&amp;"'!H9:H200"),"tested")</f>
+        <v/>
+      </c>
+      <c r="G43" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A43&amp;"'!H9:H200"),"verified")</f>
+        <v/>
+      </c>
+      <c r="H43" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A43&amp;"'!H9:H200"),"blocked")</f>
+        <v/>
+      </c>
+      <c r="I43" s="23">
+        <f>COUNTIF(INDIRECT("'"&amp;A43&amp;"'!H9:H200"),"not applicable")</f>
+        <v/>
+      </c>
+      <c r="J43" s="24">
+        <f>INDIRECT("'"&amp;A43&amp;"'!H4")</f>
+        <v/>
+      </c>
+      <c r="K43" s="23">
+        <f>INDIRECT("'"&amp;A43&amp;"'!K4")</f>
+        <v/>
+      </c>
+      <c r="L43" s="23">
+        <f>INDIRECT("'"&amp;A43&amp;"'!E5")</f>
+        <v/>
+      </c>
+      <c r="M43" s="23">
+        <f>IF(AND(J43=1,K43="complete",L43="complete"),"complete",IF(H43&gt;0,"blocked","open"))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:M41"/>
+  <autoFilter ref="A7:M43"/>
   <mergeCells count="2">
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A1:M1"/>
@@ -37064,6 +37120,1299 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:M27"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.71" customWidth="1" style="23" min="1" max="1"/>
+    <col width="15.71" customWidth="1" style="23" min="2" max="2"/>
+    <col width="18.71" customWidth="1" style="23" min="3" max="3"/>
+    <col width="58.71" customWidth="1" style="23" min="4" max="4"/>
+    <col width="14.71" customWidth="1" style="23" min="5" max="6"/>
+    <col width="50.71" customWidth="1" style="23" min="7" max="7"/>
+    <col width="17.71" customWidth="1" style="23" min="8" max="8"/>
+    <col width="14.71" customWidth="1" style="23" min="9" max="9"/>
+    <col width="14.71" customWidth="1" style="25" min="10" max="10"/>
+    <col width="42.71" customWidth="1" style="23" min="11" max="11"/>
+    <col width="10.71" customWidth="1" style="23" min="12" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="37.5" customHeight="1" s="17">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>List Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="27.75" customHeight="1" s="17">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Assertion-level native semantics, anatomy, recipes, browser, human-review, documentation, Consumer, and adoption evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="17.25" customHeight="1" s="17">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>Requirements</t>
+        </is>
+      </c>
+      <c r="B4" s="21">
+        <f>COUNTA(A9:A27)</f>
+        <v/>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="E4" s="21">
+        <f>SUM(M9:M27)</f>
+        <v/>
+      </c>
+      <c r="G4" s="20" t="inlineStr">
+        <is>
+          <t>Completion</t>
+        </is>
+      </c>
+      <c r="H4" s="22">
+        <f>IF(B4=0,0,E4/B4)</f>
+        <v/>
+      </c>
+      <c r="J4" s="20" t="inlineStr">
+        <is>
+          <t>Package gate</t>
+        </is>
+      </c>
+      <c r="K4" s="21">
+        <f>IF(COUNTIFS(E9:E27,"package",M9:M27,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="17.25" customHeight="1" s="17">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Manual review</t>
+        </is>
+      </c>
+      <c r="B5" s="21">
+        <f>IF(COUNTIFS(I9:I27,"yes",M9:M27,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>Consumer gate</t>
+        </is>
+      </c>
+      <c r="E5" s="21">
+        <f>IF(COUNTIFS(E9:E27,"consumer",M9:M27,0)&gt;0,"open","complete")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="17">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="inlineStr">
+        <is>
+          <t>Evidence type</t>
+        </is>
+      </c>
+      <c r="G8" s="23" t="inlineStr">
+        <is>
+          <t>Evidence / link</t>
+        </is>
+      </c>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>Human review?</t>
+        </is>
+      </c>
+      <c r="J8" s="25" t="inlineStr">
+        <is>
+          <t>Last verified</t>
+        </is>
+      </c>
+      <c r="K8" s="23" t="inlineStr">
+        <is>
+          <t>Blocker / N/A reason</t>
+        </is>
+      </c>
+      <c r="L8" s="23" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="M8" s="23" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="54" customHeight="1" s="17">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>L-01</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>Root and Item</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="inlineStr">
+        <is>
+          <t>Root and Item adapt released Atom List while preserving native ul, ol, li, attributes, slots, composition, refs, and authored children.</t>
+        </is>
+      </c>
+      <c r="E9" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F9" s="26" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="G9" s="27" t="inlineStr">
+        <is>
+          <t>../src/components/list</t>
+        </is>
+      </c>
+      <c r="H9" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I9" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J9" s="28" t="n">
+        <v>46229</v>
+      </c>
+      <c r="K9" s="27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M9" s="26">
+        <f>IF(OR(AND(I9="yes",H9="verified"),AND(I9="no",OR(H9="tested",H9="verified")),AND(H9="not applicable",K9&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="54" customHeight="1" s="17">
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>L-02</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>Anatomy</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>Leading, Content, Title, Description, Trailing</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>All five optional structured parts expose stable native hosts, refs, slots, and aligned passive row anatomy.</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F10" s="26" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="G10" s="27" t="inlineStr">
+        <is>
+          <t>../test/components/list/list.test.tsx</t>
+        </is>
+      </c>
+      <c r="H10" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I10" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J10" s="28" t="n">
+        <v>46229</v>
+      </c>
+      <c r="K10" s="27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M10" s="26">
+        <f>IF(OR(AND(I10="yes",H10="verified"),AND(I10="no",OR(H10="tested",H10="verified")),AND(H10="not applicable",K10&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1" s="17">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>L-03</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>Exports</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>List</t>
+        </is>
+      </c>
+      <c r="D11" s="27" t="inlineStr">
+        <is>
+          <t>Root and List subpath exports expose the compound runtime and every public List type.</t>
+        </is>
+      </c>
+      <c r="E11" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F11" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="G11" s="27" t="inlineStr">
+        <is>
+          <t>../test/package/package.test.mjs; ../test/package/ssr.test.mjs</t>
+        </is>
+      </c>
+      <c r="H11" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I11" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J11" s="28" t="n">
+        <v>46229</v>
+      </c>
+      <c r="K11" s="27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M11" s="26">
+        <f>IF(OR(AND(I11="yes",H11="verified"),AND(I11="no",OR(H11="tested",H11="verified")),AND(H11="not applicable",K11&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="54" customHeight="1" s="17">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>L-04</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>Types</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>List</t>
+        </is>
+      </c>
+      <c r="D12" s="27" t="inlineStr">
+        <is>
+          <t>Recipes, ordered attributes, native props, refs, disabled metadata, and Root/Item composition type-check.</t>
+        </is>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="inlineStr">
+        <is>
+          <t>types</t>
+        </is>
+      </c>
+      <c r="G12" s="27" t="inlineStr">
+        <is>
+          <t>../test/types/components/list.test.ts</t>
+        </is>
+      </c>
+      <c r="H12" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I12" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J12" s="28" t="n">
+        <v>46229</v>
+      </c>
+      <c r="K12" s="27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M12" s="26">
+        <f>IF(OR(AND(I12="yes",H12="verified"),AND(I12="no",OR(H12="tested",H12="verified")),AND(H12="not applicable",K12&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="54" customHeight="1" s="17">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>L-05</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>CSS</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>List</t>
+        </is>
+      </c>
+      <c r="D13" s="27" t="inlineStr">
+        <is>
+          <t>Static CSS ships variants, sizes, densities, all markers, structured anatomy, nesting, forced colors, and public variables.</t>
+        </is>
+      </c>
+      <c r="E13" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F13" s="26" t="inlineStr">
+        <is>
+          <t>css</t>
+        </is>
+      </c>
+      <c r="G13" s="27" t="inlineStr">
+        <is>
+          <t>../src/components/list/list.css</t>
+        </is>
+      </c>
+      <c r="H13" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I13" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J13" s="28" t="n">
+        <v>46229</v>
+      </c>
+      <c r="K13" s="27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M13" s="26">
+        <f>IF(OR(AND(I13="yes",H13="verified"),AND(I13="no",OR(H13="tested",H13="verified")),AND(H13="not applicable",K13&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="54" customHeight="1" s="17">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>L-06</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>List</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>Defaults, recipes, native ordered output, disabled metadata, parts, composition, refs, and overrides pass focused tests.</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F14" s="26" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="G14" s="27" t="inlineStr">
+        <is>
+          <t>../test/components/list/list.test.tsx</t>
+        </is>
+      </c>
+      <c r="H14" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I14" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J14" s="28" t="n">
+        <v>46229</v>
+      </c>
+      <c r="K14" s="27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M14" s="26">
+        <f>IF(OR(AND(I14="yes",H14="verified"),AND(I14="no",OR(H14="tested",H14="verified")),AND(H14="not applicable",K14&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="54" customHeight="1" s="17">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>L-07</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>Browser</t>
+        </is>
+      </c>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>Recipes and semantics</t>
+        </is>
+      </c>
+      <c r="D15" s="27" t="inlineStr">
+        <is>
+          <t>Real-browser defaults, ordered and unordered output, variants, sizes, densities, markers, nesting, and native attributes pass.</t>
+        </is>
+      </c>
+      <c r="E15" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F15" s="26" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+      <c r="G15" s="27" t="inlineStr">
+        <is>
+          <t>tests/components/list/behavior.spec.ts</t>
+        </is>
+      </c>
+      <c r="H15" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I15" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J15" s="28" t="n">
+        <v>46229</v>
+      </c>
+      <c r="K15" s="27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M15" s="26">
+        <f>IF(OR(AND(I15="yes",H15="verified"),AND(I15="no",OR(H15="tested",H15="verified")),AND(H15="not applicable",K15&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="54" customHeight="1" s="17">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>L-08</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>Geometry</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>Structured rows</t>
+        </is>
+      </c>
+      <c r="D16" s="27" t="inlineStr">
+        <is>
+          <t>Leading, content, and trailing columns align, descriptions wrap, actions stay contained, and logical placement reverses in RTL.</t>
+        </is>
+      </c>
+      <c r="E16" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F16" s="26" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+      <c r="G16" s="27" t="inlineStr">
+        <is>
+          <t>tests/components/list/behavior.spec.ts</t>
+        </is>
+      </c>
+      <c r="H16" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I16" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J16" s="28" t="n">
+        <v>46229</v>
+      </c>
+      <c r="K16" s="27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M16" s="26">
+        <f>IF(OR(AND(I16="yes",H16="verified"),AND(I16="no",OR(H16="tested",H16="verified")),AND(H16="not applicable",K16&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="54" customHeight="1" s="17">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>L-09</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>Native list</t>
+        </is>
+      </c>
+      <c r="D17" s="27" t="inlineStr">
+        <is>
+          <t>List roles, item relationships, marker-free semantics, authored controls, disabled metadata, and axe pass without invented interaction.</t>
+        </is>
+      </c>
+      <c r="E17" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F17" s="26" t="inlineStr">
+        <is>
+          <t>axe</t>
+        </is>
+      </c>
+      <c r="G17" s="27" t="inlineStr">
+        <is>
+          <t>tests/components/list/behavior.spec.ts</t>
+        </is>
+      </c>
+      <c r="H17" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I17" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J17" s="28" t="n">
+        <v>46229</v>
+      </c>
+      <c r="K17" s="27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M17" s="26">
+        <f>IF(OR(AND(I17="yes",H17="verified"),AND(I17="no",OR(H17="tested",H17="verified")),AND(H17="not applicable",K17&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="54" customHeight="1" s="17">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>L-10</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>List</t>
+        </is>
+      </c>
+      <c r="D18" s="27" t="inlineStr">
+        <is>
+          <t>Reviewed baselines cover defaults, boundaries, sizing, marker recipes, anatomy, dark customization, mobile RTL, and forced colors.</t>
+        </is>
+      </c>
+      <c r="E18" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F18" s="26" t="inlineStr">
+        <is>
+          <t>visual</t>
+        </is>
+      </c>
+      <c r="G18" s="27" t="inlineStr">
+        <is>
+          <t>tests/components/list/visual.spec.ts</t>
+        </is>
+      </c>
+      <c r="H18" s="26" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="I18" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J18" s="28" t="n">
+        <v>46229</v>
+      </c>
+      <c r="K18" s="27" t="inlineStr">
+        <is>
+          <t>Current List playground and all eight visual baselines were reviewed during implementation.</t>
+        </is>
+      </c>
+      <c r="M18" s="26">
+        <f>IF(OR(AND(I18="yes",H18="verified"),AND(I18="no",OR(H18="tested",H18="verified")),AND(H18="not applicable",K18&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="54" customHeight="1" s="17">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>L-11</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>Responsive</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>List</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>Physical mobile, 200%/400% zoom, rotation, narrow content, long copy, structured actions, and RTL remain readable and contained.</t>
+        </is>
+      </c>
+      <c r="E19" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F19" s="26" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G19" s="27" t="inlineStr">
+        <is>
+          <t>manual-tests/list.md</t>
+        </is>
+      </c>
+      <c r="H19" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I19" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J19" s="28" t="n"/>
+      <c r="K19" s="27" t="inlineStr">
+        <is>
+          <t>Automated reflow evidence passes; the human manual run is intentionally pending.</t>
+        </is>
+      </c>
+      <c r="M19" s="26">
+        <f>IF(OR(AND(I19="yes",H19="verified"),AND(I19="no",OR(H19="tested",H19="verified")),AND(H19="not applicable",K19&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="54" customHeight="1" s="17">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>L-12</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>List</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="inlineStr">
+        <is>
+          <t>Light, dark, forced colors, text spacing, markers, boundaries, and authored focus preserve hierarchy and contrast.</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F20" s="26" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G20" s="27" t="inlineStr">
+        <is>
+          <t>manual-tests/list.md; tests/components/list/visual.spec.ts</t>
+        </is>
+      </c>
+      <c r="H20" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I20" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J20" s="28" t="n"/>
+      <c r="K20" s="27" t="inlineStr">
+        <is>
+          <t>Automated appearance evidence passes; complete human appearance review is pending.</t>
+        </is>
+      </c>
+      <c r="M20" s="26">
+        <f>IF(OR(AND(I20="yes",H20="verified"),AND(I20="no",OR(H20="tested",H20="verified")),AND(H20="not applicable",K20&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="54" customHeight="1" s="17">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>L-13</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>Native output</t>
+        </is>
+      </c>
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>Root and Item</t>
+        </is>
+      </c>
+      <c r="D21" s="27" t="inlineStr">
+        <is>
+          <t>start, reversed, value, ordered output, nested lists, asChild, render ownership, and marker-none role behavior match the contract.</t>
+        </is>
+      </c>
+      <c r="E21" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F21" s="26" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+      <c r="G21" s="27" t="inlineStr">
+        <is>
+          <t>tests/components/list/behavior.spec.ts; ../test/components/list/list.test.tsx</t>
+        </is>
+      </c>
+      <c r="H21" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I21" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J21" s="28" t="n">
+        <v>46229</v>
+      </c>
+      <c r="K21" s="27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M21" s="26">
+        <f>IF(OR(AND(I21="yes",H21="verified"),AND(I21="no",OR(H21="tested",H21="verified")),AND(H21="not applicable",K21&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="54" customHeight="1" s="17">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>L-14</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>List</t>
+        </is>
+      </c>
+      <c r="D22" s="27" t="inlineStr">
+        <is>
+          <t>The component-owned protocol covers every List playground scenario in one top-to-bottom review flow.</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F22" s="26" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G22" s="27" t="inlineStr">
+        <is>
+          <t>manual-tests/list.md</t>
+        </is>
+      </c>
+      <c r="H22" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J22" s="28" t="n"/>
+      <c r="K22" s="27" t="inlineStr">
+        <is>
+          <t>Protocol exists; the owner deferred the human run.</t>
+        </is>
+      </c>
+      <c r="M22" s="26">
+        <f>IF(OR(AND(I22="yes",H22="verified"),AND(I22="no",OR(H22="tested",H22="verified")),AND(H22="not applicable",K22&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="54" customHeight="1" s="17">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>L-15</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C23" s="26" t="inlineStr">
+        <is>
+          <t>List</t>
+        </is>
+      </c>
+      <c r="D23" s="27" t="inlineStr">
+        <is>
+          <t>Source-backed ownership, anatomy, API, defaults, accessibility, CSS, customization, composition, and examples pass documentation gates.</t>
+        </is>
+      </c>
+      <c r="E23" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F23" s="26" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="G23" s="27" t="inlineStr">
+        <is>
+          <t>../docs/components/list/README.md</t>
+        </is>
+      </c>
+      <c r="H23" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I23" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J23" s="28" t="n">
+        <v>46229</v>
+      </c>
+      <c r="K23" s="27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M23" s="26">
+        <f>IF(OR(AND(I23="yes",H23="verified"),AND(I23="no",OR(H23="tested",H23="verified")),AND(H23="not applicable",K23&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="54" customHeight="1" s="17">
+      <c r="A24" s="26" t="inlineStr">
+        <is>
+          <t>L-16</t>
+        </is>
+      </c>
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>Changelog</t>
+        </is>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>List</t>
+        </is>
+      </c>
+      <c r="D24" s="27" t="inlineStr">
+        <is>
+          <t>List owns a public component changelog and the package changelog records its addition.</t>
+        </is>
+      </c>
+      <c r="E24" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F24" s="26" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="G24" s="27" t="inlineStr">
+        <is>
+          <t>../docs/components/list/CHANGELOG.md; ../CHANGELOG.md</t>
+        </is>
+      </c>
+      <c r="H24" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I24" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J24" s="28" t="n">
+        <v>46229</v>
+      </c>
+      <c r="K24" s="27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M24" s="26">
+        <f>IF(OR(AND(I24="yes",H24="verified"),AND(I24="no",OR(H24="tested",H24="verified")),AND(H24="not applicable",K24&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="54" customHeight="1" s="17">
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t>L-17</t>
+        </is>
+      </c>
+      <c r="B25" s="26" t="inlineStr">
+        <is>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="C25" s="26" t="inlineStr">
+        <is>
+          <t>List</t>
+        </is>
+      </c>
+      <c r="D25" s="27" t="inlineStr">
+        <is>
+          <t>The packed Consumer proves the public List subpath in a realistic structured release checklist.</t>
+        </is>
+      </c>
+      <c r="E25" s="26" t="inlineStr">
+        <is>
+          <t>consumer</t>
+        </is>
+      </c>
+      <c r="F25" s="26" t="inlineStr">
+        <is>
+          <t>consumer</t>
+        </is>
+      </c>
+      <c r="G25" s="27" t="inlineStr">
+        <is>
+          <t>../apps/consumer/src/App.tsx; ../apps/consumer/tests/consumer.spec.ts</t>
+        </is>
+      </c>
+      <c r="H25" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I25" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J25" s="28" t="n">
+        <v>46229</v>
+      </c>
+      <c r="K25" s="27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M25" s="26">
+        <f>IF(OR(AND(I25="yes",H25="verified"),AND(I25="no",OR(H25="tested",H25="verified")),AND(H25="not applicable",K25&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="54" customHeight="1" s="17">
+      <c r="A26" s="26" t="inlineStr">
+        <is>
+          <t>L-18</t>
+        </is>
+      </c>
+      <c r="B26" s="26" t="inlineStr">
+        <is>
+          <t>Playground</t>
+        </is>
+      </c>
+      <c r="C26" s="26" t="inlineStr">
+        <is>
+          <t>List</t>
+        </is>
+      </c>
+      <c r="D26" s="27" t="inlineStr">
+        <is>
+          <t>The route covers all approved scenarios and eligible Consumer, Card, and Surface content lists adopt List with classified exclusions.</t>
+        </is>
+      </c>
+      <c r="E26" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F26" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="G26" s="27" t="inlineStr">
+        <is>
+          <t>docs/list-adoption-audit.md; ../scripts/verify-playground-list.mjs</t>
+        </is>
+      </c>
+      <c r="H26" s="26" t="inlineStr">
+        <is>
+          <t>tested</t>
+        </is>
+      </c>
+      <c r="I26" s="26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J26" s="28" t="n">
+        <v>46229</v>
+      </c>
+      <c r="K26" s="27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M26" s="26">
+        <f>IF(OR(AND(I26="yes",H26="verified"),AND(I26="no",OR(H26="tested",H26="verified")),AND(H26="not applicable",K26&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="54" customHeight="1" s="17">
+      <c r="A27" s="26" t="inlineStr">
+        <is>
+          <t>L-19</t>
+        </is>
+      </c>
+      <c r="B27" s="26" t="inlineStr">
+        <is>
+          <t>Package</t>
+        </is>
+      </c>
+      <c r="C27" s="26" t="inlineStr">
+        <is>
+          <t>List</t>
+        </is>
+      </c>
+      <c r="D27" s="27" t="inlineStr">
+        <is>
+          <t>Build, SSR, exports, CSS, Atom 0.9.1, tarball, React 18/19, packed Consumer, browser matrix, and adoption checks pass.</t>
+        </is>
+      </c>
+      <c r="E27" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="F27" s="26" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="G27" s="27" t="inlineStr">
+        <is>
+          <t>../test/package; ../scripts/verify-package.mjs; ../scripts/verify-consumers.mjs; ../scripts/verify-playground-list.mjs</t>
+        </is>
+      </c>
+      <c r="H27" s="26" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="I27" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J27" s="28" t="n"/>
+      <c r="K27" s="27" t="inlineStr">
+        <is>
+          <t>Automated package gates are tracked in the workstream; complete status waits for the component-owned human manual run.</t>
+        </is>
+      </c>
+      <c r="M27" s="26">
+        <f>IF(OR(AND(I27="yes",H27="verified"),AND(I27="no",OR(H27="tested",H27="verified")),AND(H27="not applicable",K27&lt;&gt;"")),1,0)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="H9:H27" type="list" allowBlank="0" showDropDown="0">
+      <formula1>"not started,partial,implemented,tested,verified,blocked,not applicable"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I9:I27" type="list" allowBlank="0" showDropDown="0">
+      <formula1>"yes,no"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <mergeCells count="2">
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">

</xml_diff>

<commit_message>
fix: refine Table playground evidence
</commit_message>
<xml_diff>
--- a/playground/component-coverage.xlsx
+++ b/playground/component-coverage.xlsx
@@ -7637,10 +7637,10 @@
     <t xml:space="preserve">Agent inspected the final appearance baselines.</t>
   </si>
   <si>
-    <t xml:space="preserve">Eight reviewed baselines cover overview, variants, sizing, sorting, sticky, dark, mobile RTL, and forced colors.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Agent inspected every final Table baseline.</t>
+    <t xml:space="preserve">Ten reviewed baselines cover overview, variants, sizing, alignment, sorting, sticky, dark, responsive mobile, RTL mobile, and forced colors.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agent inspected every final Table baseline after the playground review corrections.</t>
   </si>
   <si>
     <t xml:space="preserve">Native structure, independent tab stops, no grid role/tabindex, labelled scrolling, and axe remain valid.</t>
@@ -11700,7 +11700,7 @@
         <v>open</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
         <v>69</v>
       </c>
@@ -57725,7 +57725,7 @@
         <v>98</v>
       </c>
       <c r="J24" s="14" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="K24" s="13" t="s">
         <v>2515</v>

</xml_diff>